<commit_message>
Update analysis, utilities, election data, and tables/figures outputs
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tables_and_figures/input_tables/national_errors.xlsx
+++ b/tables_and_figures/input_tables/national_errors.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S377"/>
+  <dimension ref="A1:S381"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -5670,10 +5670,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N78">
-        <v>21.68983558756392</v>
+        <v>21.68983558756369</v>
       </c>
       <c r="O78">
-        <v>21.68983558756405</v>
+        <v>21.68983558756393</v>
       </c>
       <c r="P78">
         <v>55400</v>
@@ -5738,10 +5738,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N79">
-        <v>21.68983558756392</v>
+        <v>21.68983558756369</v>
       </c>
       <c r="O79">
-        <v>21.68983558756405</v>
+        <v>21.68983558756393</v>
       </c>
       <c r="P79">
         <v>55400</v>
@@ -5806,10 +5806,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N80">
-        <v>21.68983558756392</v>
+        <v>21.68983558756369</v>
       </c>
       <c r="O80">
-        <v>21.68983558756405</v>
+        <v>21.68983558756393</v>
       </c>
       <c r="P80">
         <v>55400</v>
@@ -5820,7 +5820,7 @@
         </is>
       </c>
       <c r="S80">
-        <v>1.936748087924742</v>
+        <v>1.936748087924511</v>
       </c>
     </row>
     <row r="81">
@@ -5874,10 +5874,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N81">
-        <v>21.68983558756392</v>
+        <v>21.68983558756369</v>
       </c>
       <c r="O81">
-        <v>21.68983558756405</v>
+        <v>21.68983558756393</v>
       </c>
       <c r="P81">
         <v>55400</v>
@@ -5888,7 +5888,7 @@
         </is>
       </c>
       <c r="S81">
-        <v>1.936748087924864</v>
+        <v>1.936748087924747</v>
       </c>
     </row>
     <row r="82">
@@ -5942,10 +5942,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N82">
-        <v>32.13108402346401</v>
+        <v>32.131084023464</v>
       </c>
       <c r="O82">
-        <v>32.13108402346418</v>
+        <v>32.13108402346392</v>
       </c>
       <c r="P82">
         <v>55400</v>
@@ -6010,10 +6010,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N83">
-        <v>32.13108402346401</v>
+        <v>32.131084023464</v>
       </c>
       <c r="O83">
-        <v>32.13108402346418</v>
+        <v>32.13108402346392</v>
       </c>
       <c r="P83">
         <v>55400</v>
@@ -6078,10 +6078,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N84">
-        <v>32.13108402346401</v>
+        <v>32.131084023464</v>
       </c>
       <c r="O84">
-        <v>32.13108402346418</v>
+        <v>32.13108402346392</v>
       </c>
       <c r="P84">
         <v>55400</v>
@@ -6092,7 +6092,7 @@
         </is>
       </c>
       <c r="S84">
-        <v>0.4445337920600756</v>
+        <v>0.44453379206007</v>
       </c>
     </row>
     <row r="85">
@@ -6146,10 +6146,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N85">
-        <v>32.13108402346401</v>
+        <v>32.131084023464</v>
       </c>
       <c r="O85">
-        <v>32.13108402346418</v>
+        <v>32.13108402346392</v>
       </c>
       <c r="P85">
         <v>55400</v>
@@ -6160,7 +6160,7 @@
         </is>
       </c>
       <c r="S85">
-        <v>0.4445337920602477</v>
+        <v>0.4445337920599868</v>
       </c>
     </row>
     <row r="86">
@@ -6214,10 +6214,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N86">
-        <v>60.64538348494989</v>
+        <v>60.64538348495072</v>
       </c>
       <c r="O86">
-        <v>60.64538348495076</v>
+        <v>60.64538348495044</v>
       </c>
       <c r="P86">
         <v>55400</v>
@@ -6282,10 +6282,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N87">
-        <v>60.64538348494989</v>
+        <v>60.64538348495072</v>
       </c>
       <c r="O87">
-        <v>60.64538348495076</v>
+        <v>60.64538348495044</v>
       </c>
       <c r="P87">
         <v>55400</v>
@@ -6350,10 +6350,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N88">
-        <v>60.64538348494989</v>
+        <v>60.64538348495072</v>
       </c>
       <c r="O88">
-        <v>60.64538348495076</v>
+        <v>60.64538348495044</v>
       </c>
       <c r="P88">
         <v>55400</v>
@@ -6364,7 +6364,7 @@
         </is>
       </c>
       <c r="S88">
-        <v>-0.2387361085909201</v>
+        <v>-0.2387361085900874</v>
       </c>
     </row>
     <row r="89">
@@ -6418,10 +6418,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N89">
-        <v>60.64538348494989</v>
+        <v>60.64538348495072</v>
       </c>
       <c r="O89">
-        <v>60.64538348495076</v>
+        <v>60.64538348495044</v>
       </c>
       <c r="P89">
         <v>55400</v>
@@ -6432,7 +6432,7 @@
         </is>
       </c>
       <c r="S89">
-        <v>-0.238736108590043</v>
+        <v>-0.238736108590365</v>
       </c>
     </row>
     <row r="90">
@@ -6486,10 +6486,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N90">
-        <v>23.19167199619754</v>
+        <v>23.19167199619718</v>
       </c>
       <c r="O90">
-        <v>23.19287782028184</v>
+        <v>23.19287782028157</v>
       </c>
       <c r="P90">
         <v>48612</v>
@@ -6554,10 +6554,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N91">
-        <v>23.19167199619754</v>
+        <v>23.19167199619718</v>
       </c>
       <c r="O91">
-        <v>23.19287782028184</v>
+        <v>23.19287782028157</v>
       </c>
       <c r="P91">
         <v>48612</v>
@@ -6622,10 +6622,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N92">
-        <v>23.19167199619754</v>
+        <v>23.19167199619718</v>
       </c>
       <c r="O92">
-        <v>23.19287782028184</v>
+        <v>23.19287782028157</v>
       </c>
       <c r="P92">
         <v>48612</v>
@@ -6636,7 +6636,7 @@
         </is>
       </c>
       <c r="S92">
-        <v>-0.2830345174885757</v>
+        <v>-0.2830345174889337</v>
       </c>
     </row>
     <row r="93">
@@ -6690,10 +6690,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N93">
-        <v>23.19167199619754</v>
+        <v>23.19167199619718</v>
       </c>
       <c r="O93">
-        <v>23.19287782028184</v>
+        <v>23.19287782028157</v>
       </c>
       <c r="P93">
         <v>48612</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="S93">
-        <v>-0.2818286934042763</v>
+        <v>-0.2818286934045483</v>
       </c>
     </row>
     <row r="94">
@@ -6758,10 +6758,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N94">
-        <v>90.07772910426883</v>
+        <v>90.07772910426878</v>
       </c>
       <c r="O94">
-        <v>95.56945283348823</v>
+        <v>95.5694528334882</v>
       </c>
       <c r="P94">
         <v>49058</v>
@@ -6826,10 +6826,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N95">
-        <v>90.07772910426883</v>
+        <v>90.07772910426878</v>
       </c>
       <c r="O95">
-        <v>95.56945283348823</v>
+        <v>95.5694528334882</v>
       </c>
       <c r="P95">
         <v>49058</v>
@@ -6894,10 +6894,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N96">
-        <v>90.07772910426883</v>
+        <v>90.07772910426878</v>
       </c>
       <c r="O96">
-        <v>95.56945283348823</v>
+        <v>95.5694528334882</v>
       </c>
       <c r="P96">
         <v>49058</v>
@@ -6908,7 +6908,7 @@
         </is>
       </c>
       <c r="S96">
-        <v>-2.036080868973866</v>
+        <v>-2.0360808689739</v>
       </c>
     </row>
     <row r="97">
@@ -6962,10 +6962,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N97">
-        <v>90.07772910426883</v>
+        <v>90.07772910426878</v>
       </c>
       <c r="O97">
-        <v>95.56945283348823</v>
+        <v>95.5694528334882</v>
       </c>
       <c r="P97">
         <v>49058</v>
@@ -6976,7 +6976,7 @@
         </is>
       </c>
       <c r="S97">
-        <v>3.455642860245545</v>
+        <v>3.455642860245511</v>
       </c>
     </row>
     <row r="98">
@@ -7030,10 +7030,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N98">
-        <v>60.39792154911977</v>
+        <v>60.39792154911988</v>
       </c>
       <c r="O98">
-        <v>61.3884842702589</v>
+        <v>61.38848427025866</v>
       </c>
       <c r="P98">
         <v>55325</v>
@@ -7098,10 +7098,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N99">
-        <v>60.39792154911977</v>
+        <v>60.39792154911988</v>
       </c>
       <c r="O99">
-        <v>61.3884842702589</v>
+        <v>61.38848427025866</v>
       </c>
       <c r="P99">
         <v>55325</v>
@@ -7166,10 +7166,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N100">
-        <v>60.39792154911977</v>
+        <v>60.39792154911988</v>
       </c>
       <c r="O100">
-        <v>61.3884842702589</v>
+        <v>61.38848427025866</v>
       </c>
       <c r="P100">
         <v>55325</v>
@@ -7180,7 +7180,7 @@
         </is>
       </c>
       <c r="S100">
-        <v>-1.447053910698781</v>
+        <v>-1.44705391069867</v>
       </c>
     </row>
     <row r="101">
@@ -7234,10 +7234,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N101">
-        <v>60.39792154911977</v>
+        <v>60.39792154911988</v>
       </c>
       <c r="O101">
-        <v>61.3884842702589</v>
+        <v>61.38848427025866</v>
       </c>
       <c r="P101">
         <v>55325</v>
@@ -7248,7 +7248,7 @@
         </is>
       </c>
       <c r="S101">
-        <v>-0.4564911895596491</v>
+        <v>-0.4564911895598933</v>
       </c>
     </row>
     <row r="102">
@@ -7302,10 +7302,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N102">
-        <v>51.9685103540086</v>
+        <v>51.96851035400858</v>
       </c>
       <c r="O102">
-        <v>55.16820532599615</v>
+        <v>55.16820532599596</v>
       </c>
       <c r="P102">
         <v>55400</v>
@@ -7370,10 +7370,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N103">
-        <v>51.9685103540086</v>
+        <v>51.96851035400858</v>
       </c>
       <c r="O103">
-        <v>55.16820532599615</v>
+        <v>55.16820532599596</v>
       </c>
       <c r="P103">
         <v>55400</v>
@@ -7438,10 +7438,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N104">
-        <v>51.9685103540086</v>
+        <v>51.96851035400858</v>
       </c>
       <c r="O104">
-        <v>55.16820532599615</v>
+        <v>55.16820532599596</v>
       </c>
       <c r="P104">
         <v>55400</v>
@@ -7452,7 +7452,7 @@
         </is>
       </c>
       <c r="S104">
-        <v>-0.4053152415142924</v>
+        <v>-0.4053152415143146</v>
       </c>
     </row>
     <row r="105">
@@ -7506,10 +7506,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N105">
-        <v>51.9685103540086</v>
+        <v>51.96851035400858</v>
       </c>
       <c r="O105">
-        <v>55.16820532599615</v>
+        <v>55.16820532599596</v>
       </c>
       <c r="P105">
         <v>55400</v>
@@ -7520,7 +7520,7 @@
         </is>
       </c>
       <c r="S105">
-        <v>2.794379730473251</v>
+        <v>2.794379730473062</v>
       </c>
     </row>
     <row r="106">
@@ -7574,10 +7574,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N106">
-        <v>87.32994267910608</v>
+        <v>87.32994267910654</v>
       </c>
       <c r="O106">
-        <v>92.33804839648158</v>
+        <v>92.33804839648147</v>
       </c>
       <c r="P106">
         <v>55242</v>
@@ -7642,10 +7642,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N107">
-        <v>87.32994267910608</v>
+        <v>87.32994267910654</v>
       </c>
       <c r="O107">
-        <v>92.33804839648158</v>
+        <v>92.33804839648147</v>
       </c>
       <c r="P107">
         <v>55242</v>
@@ -7710,10 +7710,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N108">
-        <v>87.32994267910608</v>
+        <v>87.32994267910654</v>
       </c>
       <c r="O108">
-        <v>92.33804839648158</v>
+        <v>92.33804839648147</v>
       </c>
       <c r="P108">
         <v>55242</v>
@@ -7724,7 +7724,7 @@
         </is>
       </c>
       <c r="S108">
-        <v>-0.1009559809642679</v>
+        <v>-0.1009559809638128</v>
       </c>
     </row>
     <row r="109">
@@ -7778,10 +7778,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N109">
-        <v>87.32994267910608</v>
+        <v>87.32994267910654</v>
       </c>
       <c r="O109">
-        <v>92.33804839648158</v>
+        <v>92.33804839648147</v>
       </c>
       <c r="P109">
         <v>55242</v>
@@ -7792,7 +7792,7 @@
         </is>
       </c>
       <c r="S109">
-        <v>4.907149736411231</v>
+        <v>4.907149736411109</v>
       </c>
     </row>
     <row r="110">
@@ -7846,10 +7846,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N110">
-        <v>90.29738719024508</v>
+        <v>90.29738719024533</v>
       </c>
       <c r="O110">
-        <v>85.14002215874885</v>
+        <v>85.14002215874858</v>
       </c>
       <c r="P110">
         <v>55400</v>
@@ -7914,10 +7914,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N111">
-        <v>90.29738719024508</v>
+        <v>90.29738719024533</v>
       </c>
       <c r="O111">
-        <v>85.14002215874885</v>
+        <v>85.14002215874858</v>
       </c>
       <c r="P111">
         <v>55400</v>
@@ -7982,10 +7982,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N112">
-        <v>90.29738719024508</v>
+        <v>90.29738719024533</v>
       </c>
       <c r="O112">
-        <v>85.14002215874885</v>
+        <v>85.14002215874858</v>
       </c>
       <c r="P112">
         <v>55400</v>
@@ -7996,7 +7996,7 @@
         </is>
       </c>
       <c r="S112">
-        <v>0.729413685619984</v>
+        <v>0.7294136856202504</v>
       </c>
     </row>
     <row r="113">
@@ -8050,10 +8050,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N113">
-        <v>90.29738719024508</v>
+        <v>90.29738719024533</v>
       </c>
       <c r="O113">
-        <v>85.14002215874885</v>
+        <v>85.14002215874858</v>
       </c>
       <c r="P113">
         <v>55400</v>
@@ -8064,7 +8064,7 @@
         </is>
       </c>
       <c r="S113">
-        <v>-4.427951345876235</v>
+        <v>-4.427951345876502</v>
       </c>
     </row>
     <row r="114">
@@ -8118,10 +8118,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N114">
-        <v>81.97678428265853</v>
+        <v>81.97678428265843</v>
       </c>
       <c r="O114">
-        <v>78.85814310205289</v>
+        <v>78.85814310205271</v>
       </c>
       <c r="P114">
         <v>37859</v>
@@ -8186,10 +8186,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N115">
-        <v>81.97678428265853</v>
+        <v>81.97678428265843</v>
       </c>
       <c r="O115">
-        <v>78.85814310205289</v>
+        <v>78.85814310205271</v>
       </c>
       <c r="P115">
         <v>37859</v>
@@ -8254,10 +8254,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N116">
-        <v>81.97678428265853</v>
+        <v>81.97678428265843</v>
       </c>
       <c r="O116">
-        <v>78.85814310205289</v>
+        <v>78.85814310205271</v>
       </c>
       <c r="P116">
         <v>37859</v>
@@ -8268,7 +8268,7 @@
         </is>
       </c>
       <c r="S116">
-        <v>-0.8086498910109485</v>
+        <v>-0.8086498910110373</v>
       </c>
     </row>
     <row r="117">
@@ -8322,10 +8322,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N117">
-        <v>81.97678428265853</v>
+        <v>81.97678428265843</v>
       </c>
       <c r="O117">
-        <v>78.85814310205289</v>
+        <v>78.85814310205271</v>
       </c>
       <c r="P117">
         <v>37859</v>
@@ -8336,7 +8336,7 @@
         </is>
       </c>
       <c r="S117">
-        <v>-3.927291071616579</v>
+        <v>-3.927291071616756</v>
       </c>
     </row>
     <row r="118">
@@ -8390,10 +8390,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N118">
-        <v>61.84561105159655</v>
+        <v>61.84561105159537</v>
       </c>
       <c r="O118">
-        <v>26.29907721541566</v>
+        <v>26.29907721541595</v>
       </c>
       <c r="P118">
         <v>44776</v>
@@ -8458,10 +8458,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N119">
-        <v>61.84561105159655</v>
+        <v>61.84561105159537</v>
       </c>
       <c r="O119">
-        <v>26.29907721541566</v>
+        <v>26.29907721541595</v>
       </c>
       <c r="P119">
         <v>44776</v>
@@ -8526,10 +8526,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N120">
-        <v>61.84561105159655</v>
+        <v>61.84561105159537</v>
       </c>
       <c r="O120">
-        <v>26.29907721541566</v>
+        <v>26.29907721541595</v>
       </c>
       <c r="P120">
         <v>44776</v>
@@ -8540,7 +8540,7 @@
         </is>
       </c>
       <c r="S120">
-        <v>0.3570698780801185</v>
+        <v>0.3570698780789416</v>
       </c>
     </row>
     <row r="121">
@@ -8594,10 +8594,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N121">
-        <v>61.84561105159655</v>
+        <v>61.84561105159537</v>
       </c>
       <c r="O121">
-        <v>26.29907721541566</v>
+        <v>26.29907721541595</v>
       </c>
       <c r="P121">
         <v>44776</v>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="S121">
-        <v>-35.18946395810077</v>
+        <v>-35.18946395810048</v>
       </c>
     </row>
     <row r="122">
@@ -8662,10 +8662,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N122">
-        <v>18.78381922591106</v>
+        <v>18.78381922591102</v>
       </c>
       <c r="O122">
-        <v>18.78376405592467</v>
+        <v>18.78376405592434</v>
       </c>
       <c r="P122">
         <v>54535</v>
@@ -8730,10 +8730,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N123">
-        <v>18.78381922591106</v>
+        <v>18.78381922591102</v>
       </c>
       <c r="O123">
-        <v>18.78376405592467</v>
+        <v>18.78376405592434</v>
       </c>
       <c r="P123">
         <v>54535</v>
@@ -8798,10 +8798,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N124">
-        <v>18.78381922591106</v>
+        <v>18.78381922591102</v>
       </c>
       <c r="O124">
-        <v>18.78376405592467</v>
+        <v>18.78376405592434</v>
       </c>
       <c r="P124">
         <v>54535</v>
@@ -8812,7 +8812,7 @@
         </is>
       </c>
       <c r="S124">
-        <v>-0.5877807213773428</v>
+        <v>-0.5877807213773845</v>
       </c>
     </row>
     <row r="125">
@@ -8866,10 +8866,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N125">
-        <v>18.78381922591106</v>
+        <v>18.78381922591102</v>
       </c>
       <c r="O125">
-        <v>18.78376405592467</v>
+        <v>18.78376405592434</v>
       </c>
       <c r="P125">
         <v>54535</v>
@@ -8880,7 +8880,7 @@
         </is>
       </c>
       <c r="S125">
-        <v>-0.587835891363736</v>
+        <v>-0.5878358913640636</v>
       </c>
     </row>
     <row r="126">
@@ -8934,10 +8934,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N126">
-        <v>30.53786279215646</v>
+        <v>30.53786279215657</v>
       </c>
       <c r="O126">
-        <v>30.53774451303555</v>
+        <v>30.53774451303544</v>
       </c>
       <c r="P126">
         <v>54535</v>
@@ -9002,10 +9002,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N127">
-        <v>30.53786279215646</v>
+        <v>30.53786279215657</v>
       </c>
       <c r="O127">
-        <v>30.53774451303555</v>
+        <v>30.53774451303544</v>
       </c>
       <c r="P127">
         <v>54535</v>
@@ -9070,10 +9070,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N128">
-        <v>30.53786279215646</v>
+        <v>30.53786279215657</v>
       </c>
       <c r="O128">
-        <v>30.53774451303555</v>
+        <v>30.53774451303544</v>
       </c>
       <c r="P128">
         <v>54535</v>
@@ -9084,7 +9084,7 @@
         </is>
       </c>
       <c r="S128">
-        <v>-0.1367483492706933</v>
+        <v>-0.1367483492705823</v>
       </c>
     </row>
     <row r="129">
@@ -9138,10 +9138,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N129">
-        <v>30.53786279215646</v>
+        <v>30.53786279215657</v>
       </c>
       <c r="O129">
-        <v>30.53774451303555</v>
+        <v>30.53774451303544</v>
       </c>
       <c r="P129">
         <v>54535</v>
@@ -9152,7 +9152,7 @@
         </is>
       </c>
       <c r="S129">
-        <v>-0.136866628391602</v>
+        <v>-0.136866628391713</v>
       </c>
     </row>
     <row r="130">
@@ -9206,10 +9206,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N130">
-        <v>60.0704815986113</v>
+        <v>60.07048159861138</v>
       </c>
       <c r="O130">
-        <v>60.07051969567441</v>
+        <v>60.07051969567385</v>
       </c>
       <c r="P130">
         <v>54535</v>
@@ -9274,10 +9274,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N131">
-        <v>60.0704815986113</v>
+        <v>60.07048159861138</v>
       </c>
       <c r="O131">
-        <v>60.07051969567441</v>
+        <v>60.07051969567385</v>
       </c>
       <c r="P131">
         <v>54535</v>
@@ -9342,10 +9342,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N132">
-        <v>60.0704815986113</v>
+        <v>60.07048159861138</v>
       </c>
       <c r="O132">
-        <v>60.07051969567441</v>
+        <v>60.07051969567385</v>
       </c>
       <c r="P132">
         <v>54535</v>
@@ -9356,7 +9356,7 @@
         </is>
       </c>
       <c r="S132">
-        <v>-0.7931925941981666</v>
+        <v>-0.7931925941980889</v>
       </c>
     </row>
     <row r="133">
@@ -9410,10 +9410,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N133">
-        <v>60.0704815986113</v>
+        <v>60.07048159861138</v>
       </c>
       <c r="O133">
-        <v>60.07051969567441</v>
+        <v>60.07051969567385</v>
       </c>
       <c r="P133">
         <v>54535</v>
@@ -9424,7 +9424,7 @@
         </is>
       </c>
       <c r="S133">
-        <v>-0.7931544971350624</v>
+        <v>-0.7931544971356175</v>
       </c>
     </row>
     <row r="134">
@@ -9478,10 +9478,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N134">
-        <v>22.8075281326633</v>
+        <v>22.80752813266336</v>
       </c>
       <c r="O134">
-        <v>22.80764277056721</v>
+        <v>22.80764277056756</v>
       </c>
       <c r="P134">
         <v>47918</v>
@@ -9546,10 +9546,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N135">
-        <v>22.8075281326633</v>
+        <v>22.80752813266336</v>
       </c>
       <c r="O135">
-        <v>22.80764277056721</v>
+        <v>22.80764277056756</v>
       </c>
       <c r="P135">
         <v>47918</v>
@@ -9614,10 +9614,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N136">
-        <v>22.8075281326633</v>
+        <v>22.80752813266336</v>
       </c>
       <c r="O136">
-        <v>22.80764277056721</v>
+        <v>22.80764277056756</v>
       </c>
       <c r="P136">
         <v>47918</v>
@@ -9628,7 +9628,7 @@
         </is>
       </c>
       <c r="S136">
-        <v>-0.6564727659102182</v>
+        <v>-0.6564727659101488</v>
       </c>
     </row>
     <row r="137">
@@ -9682,10 +9682,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N137">
-        <v>22.8075281326633</v>
+        <v>22.80752813266336</v>
       </c>
       <c r="O137">
-        <v>22.80764277056721</v>
+        <v>22.80764277056756</v>
       </c>
       <c r="P137">
         <v>47918</v>
@@ -9696,7 +9696,7 @@
         </is>
       </c>
       <c r="S137">
-        <v>-0.6563581280063013</v>
+        <v>-0.6563581280059488</v>
       </c>
     </row>
     <row r="138">
@@ -9750,7 +9750,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N138">
-        <v>89.057646837029</v>
+        <v>89.05764683702921</v>
       </c>
       <c r="O138">
         <v>96.53969112716689</v>
@@ -9818,7 +9818,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N139">
-        <v>89.057646837029</v>
+        <v>89.05764683702921</v>
       </c>
       <c r="O139">
         <v>96.53969112716689</v>
@@ -9886,7 +9886,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N140">
-        <v>89.057646837029</v>
+        <v>89.05764683702921</v>
       </c>
       <c r="O140">
         <v>96.53969112716689</v>
@@ -9900,7 +9900,7 @@
         </is>
       </c>
       <c r="S140">
-        <v>-2.609675776510978</v>
+        <v>-2.609675776510767</v>
       </c>
     </row>
     <row r="141">
@@ -9954,7 +9954,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N141">
-        <v>89.057646837029</v>
+        <v>89.05764683702921</v>
       </c>
       <c r="O141">
         <v>96.53969112716689</v>
@@ -10022,10 +10022,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N142">
-        <v>61.88484918229447</v>
+        <v>61.88484918229459</v>
       </c>
       <c r="O142">
-        <v>61.4772745944154</v>
+        <v>61.47727459441587</v>
       </c>
       <c r="P142">
         <v>54426</v>
@@ -10090,10 +10090,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N143">
-        <v>61.88484918229447</v>
+        <v>61.88484918229459</v>
       </c>
       <c r="O143">
-        <v>61.4772745944154</v>
+        <v>61.47727459441587</v>
       </c>
       <c r="P143">
         <v>54426</v>
@@ -10158,10 +10158,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N144">
-        <v>61.88484918229447</v>
+        <v>61.88484918229459</v>
       </c>
       <c r="O144">
-        <v>61.4772745944154</v>
+        <v>61.47727459441587</v>
       </c>
       <c r="P144">
         <v>54426</v>
@@ -10172,7 +10172,7 @@
         </is>
       </c>
       <c r="S144">
-        <v>-1.127829715025674</v>
+        <v>-1.127829715025552</v>
       </c>
     </row>
     <row r="145">
@@ -10226,10 +10226,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N145">
-        <v>61.88484918229447</v>
+        <v>61.88484918229459</v>
       </c>
       <c r="O145">
-        <v>61.4772745944154</v>
+        <v>61.47727459441587</v>
       </c>
       <c r="P145">
         <v>54426</v>
@@ -10240,7 +10240,7 @@
         </is>
       </c>
       <c r="S145">
-        <v>-1.535404302904742</v>
+        <v>-1.535404302904275</v>
       </c>
     </row>
     <row r="146">
@@ -10294,10 +10294,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N146">
-        <v>52.10416026488397</v>
+        <v>52.10416026488398</v>
       </c>
       <c r="O146">
-        <v>53.71180101699645</v>
+        <v>53.71180101699651</v>
       </c>
       <c r="P146">
         <v>54535</v>
@@ -10362,10 +10362,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N147">
-        <v>52.10416026488397</v>
+        <v>52.10416026488398</v>
       </c>
       <c r="O147">
-        <v>53.71180101699645</v>
+        <v>53.71180101699651</v>
       </c>
       <c r="P147">
         <v>54535</v>
@@ -10430,10 +10430,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N148">
-        <v>52.10416026488397</v>
+        <v>52.10416026488398</v>
       </c>
       <c r="O148">
-        <v>53.71180101699645</v>
+        <v>53.71180101699651</v>
       </c>
       <c r="P148">
         <v>54535</v>
@@ -10444,7 +10444,7 @@
         </is>
       </c>
       <c r="S148">
-        <v>-0.1882192833705831</v>
+        <v>-0.188219283370572</v>
       </c>
     </row>
     <row r="149">
@@ -10498,10 +10498,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N149">
-        <v>52.10416026488397</v>
+        <v>52.10416026488398</v>
       </c>
       <c r="O149">
-        <v>53.71180101699645</v>
+        <v>53.71180101699651</v>
       </c>
       <c r="P149">
         <v>54535</v>
@@ -10512,7 +10512,7 @@
         </is>
       </c>
       <c r="S149">
-        <v>1.419421468741899</v>
+        <v>1.419421468741955</v>
       </c>
     </row>
     <row r="150">
@@ -10566,10 +10566,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N150">
-        <v>88.10981089169665</v>
+        <v>88.10981089169675</v>
       </c>
       <c r="O150">
-        <v>92.81601489807952</v>
+        <v>92.81601489807957</v>
       </c>
       <c r="P150">
         <v>54281</v>
@@ -10634,10 +10634,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N151">
-        <v>88.10981089169665</v>
+        <v>88.10981089169675</v>
       </c>
       <c r="O151">
-        <v>92.81601489807952</v>
+        <v>92.81601489807957</v>
       </c>
       <c r="P151">
         <v>54281</v>
@@ -10702,10 +10702,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N152">
-        <v>88.10981089169665</v>
+        <v>88.10981089169675</v>
       </c>
       <c r="O152">
-        <v>92.81601489807952</v>
+        <v>92.81601489807957</v>
       </c>
       <c r="P152">
         <v>54281</v>
@@ -10716,7 +10716,7 @@
         </is>
       </c>
       <c r="S152">
-        <v>0.03641639628380045</v>
+        <v>0.03641639628391147</v>
       </c>
     </row>
     <row r="153">
@@ -10770,10 +10770,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N153">
-        <v>88.10981089169665</v>
+        <v>88.10981089169675</v>
       </c>
       <c r="O153">
-        <v>92.81601489807952</v>
+        <v>92.81601489807957</v>
       </c>
       <c r="P153">
         <v>54281</v>
@@ -10784,7 +10784,7 @@
         </is>
       </c>
       <c r="S153">
-        <v>4.742620402666664</v>
+        <v>4.742620402666731</v>
       </c>
     </row>
     <row r="154">
@@ -10838,10 +10838,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N154">
-        <v>90.59641787470704</v>
+        <v>90.59641787470699</v>
       </c>
       <c r="O154">
-        <v>86.4560265318876</v>
+        <v>86.45602653188774</v>
       </c>
       <c r="P154">
         <v>54534</v>
@@ -10906,10 +10906,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N155">
-        <v>90.59641787470704</v>
+        <v>90.59641787470699</v>
       </c>
       <c r="O155">
-        <v>86.4560265318876</v>
+        <v>86.45602653188774</v>
       </c>
       <c r="P155">
         <v>54534</v>
@@ -10974,10 +10974,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N156">
-        <v>90.59641787470704</v>
+        <v>90.59641787470699</v>
       </c>
       <c r="O156">
-        <v>86.4560265318876</v>
+        <v>86.45602653188774</v>
       </c>
       <c r="P156">
         <v>54534</v>
@@ -10988,7 +10988,7 @@
         </is>
       </c>
       <c r="S156">
-        <v>0.6425753431986925</v>
+        <v>0.642575343198637</v>
       </c>
     </row>
     <row r="157">
@@ -11042,10 +11042,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N157">
-        <v>90.59641787470704</v>
+        <v>90.59641787470699</v>
       </c>
       <c r="O157">
-        <v>86.4560265318876</v>
+        <v>86.45602653188774</v>
       </c>
       <c r="P157">
         <v>54534</v>
@@ -11056,7 +11056,7 @@
         </is>
       </c>
       <c r="S157">
-        <v>-3.497815999620746</v>
+        <v>-3.497815999620613</v>
       </c>
     </row>
     <row r="158">
@@ -11110,10 +11110,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N158">
-        <v>81.45050683818823</v>
+        <v>81.45050683818815</v>
       </c>
       <c r="O158">
-        <v>77.4884120909541</v>
+        <v>77.48841209095431</v>
       </c>
       <c r="P158">
         <v>39772</v>
@@ -11178,10 +11178,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N159">
-        <v>81.45050683818823</v>
+        <v>81.45050683818815</v>
       </c>
       <c r="O159">
-        <v>77.4884120909541</v>
+        <v>77.48841209095431</v>
       </c>
       <c r="P159">
         <v>39772</v>
@@ -11246,10 +11246,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N160">
-        <v>81.45050683818823</v>
+        <v>81.45050683818815</v>
       </c>
       <c r="O160">
-        <v>77.4884120909541</v>
+        <v>77.48841209095431</v>
       </c>
       <c r="P160">
         <v>39772</v>
@@ -11260,7 +11260,7 @@
         </is>
       </c>
       <c r="S160">
-        <v>-0.5301548422915192</v>
+        <v>-0.5301548422915969</v>
       </c>
     </row>
     <row r="161">
@@ -11314,10 +11314,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N161">
-        <v>81.45050683818823</v>
+        <v>81.45050683818815</v>
       </c>
       <c r="O161">
-        <v>77.4884120909541</v>
+        <v>77.48841209095431</v>
       </c>
       <c r="P161">
         <v>39772</v>
@@ -11328,7 +11328,7 @@
         </is>
       </c>
       <c r="S161">
-        <v>-4.492249589525644</v>
+        <v>-4.492249589525443</v>
       </c>
     </row>
     <row r="162">
@@ -11382,10 +11382,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N162">
-        <v>53.97907512970576</v>
+        <v>53.97907512970481</v>
       </c>
       <c r="O162">
-        <v>90.77842736117594</v>
+        <v>90.77842736117616</v>
       </c>
       <c r="P162">
         <v>42552</v>
@@ -11450,10 +11450,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N163">
-        <v>53.97907512970576</v>
+        <v>53.97907512970481</v>
       </c>
       <c r="O163">
-        <v>90.77842736117594</v>
+        <v>90.77842736117616</v>
       </c>
       <c r="P163">
         <v>42552</v>
@@ -11518,10 +11518,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N164">
-        <v>53.97907512970576</v>
+        <v>53.97907512970481</v>
       </c>
       <c r="O164">
-        <v>90.77842736117594</v>
+        <v>90.77842736117616</v>
       </c>
       <c r="P164">
         <v>42552</v>
@@ -11532,7 +11532,7 @@
         </is>
       </c>
       <c r="S164">
-        <v>0.0008416705650216016</v>
+        <v>0.0008416705640779121</v>
       </c>
     </row>
     <row r="165">
@@ -11586,10 +11586,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N165">
-        <v>53.97907512970576</v>
+        <v>53.97907512970481</v>
       </c>
       <c r="O165">
-        <v>90.77842736117594</v>
+        <v>90.77842736117616</v>
       </c>
       <c r="P165">
         <v>42552</v>
@@ -11600,7 +11600,7 @@
         </is>
       </c>
       <c r="S165">
-        <v>36.8001939020352</v>
+        <v>36.80019390203542</v>
       </c>
     </row>
     <row r="166">
@@ -20358,10 +20358,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N294">
-        <v>15.41815523864194</v>
+        <v>15.41815523864195</v>
       </c>
       <c r="O294">
-        <v>15.39358401703903</v>
+        <v>15.39358401703959</v>
       </c>
       <c r="P294">
         <v>61000</v>
@@ -20426,10 +20426,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N295">
-        <v>15.41815523864194</v>
+        <v>15.41815523864195</v>
       </c>
       <c r="O295">
-        <v>15.39358401703903</v>
+        <v>15.39358401703959</v>
       </c>
       <c r="P295">
         <v>61000</v>
@@ -20494,10 +20494,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N296">
-        <v>15.41815523864194</v>
+        <v>15.41815523864195</v>
       </c>
       <c r="O296">
-        <v>15.39358401703903</v>
+        <v>15.39358401703959</v>
       </c>
       <c r="P296">
         <v>61000</v>
@@ -20508,7 +20508,7 @@
         </is>
       </c>
       <c r="S296">
-        <v>-2.434066014787231</v>
+        <v>-2.43406601478722</v>
       </c>
     </row>
     <row r="297">
@@ -20562,10 +20562,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N297">
-        <v>15.41815523864194</v>
+        <v>15.41815523864195</v>
       </c>
       <c r="O297">
-        <v>15.39358401703903</v>
+        <v>15.39358401703959</v>
       </c>
       <c r="P297">
         <v>61000</v>
@@ -20576,7 +20576,7 @@
         </is>
       </c>
       <c r="S297">
-        <v>-2.458637236390146</v>
+        <v>-2.458637236389585</v>
       </c>
     </row>
     <row r="298">
@@ -20630,10 +20630,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N298">
-        <v>28.57244554318082</v>
+        <v>28.57244554318077</v>
       </c>
       <c r="O298">
-        <v>28.56364349950706</v>
+        <v>28.56364349950802</v>
       </c>
       <c r="P298">
         <v>61000</v>
@@ -20698,10 +20698,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N299">
-        <v>28.57244554318082</v>
+        <v>28.57244554318077</v>
       </c>
       <c r="O299">
-        <v>28.56364349950706</v>
+        <v>28.56364349950802</v>
       </c>
       <c r="P299">
         <v>61000</v>
@@ -20766,10 +20766,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N300">
-        <v>28.57244554318082</v>
+        <v>28.57244554318077</v>
       </c>
       <c r="O300">
-        <v>28.56364349950706</v>
+        <v>28.56364349950802</v>
       </c>
       <c r="P300">
         <v>61000</v>
@@ -20780,7 +20780,7 @@
         </is>
       </c>
       <c r="S300">
-        <v>-0.5880716505328953</v>
+        <v>-0.5880716505329397</v>
       </c>
     </row>
     <row r="301">
@@ -20834,10 +20834,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N301">
-        <v>28.57244554318082</v>
+        <v>28.57244554318077</v>
       </c>
       <c r="O301">
-        <v>28.56364349950706</v>
+        <v>28.56364349950802</v>
       </c>
       <c r="P301">
         <v>61000</v>
@@ -20848,7 +20848,7 @@
         </is>
       </c>
       <c r="S301">
-        <v>-0.5968736942066566</v>
+        <v>-0.5968736942056962</v>
       </c>
     </row>
     <row r="302">
@@ -20902,10 +20902,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N302">
-        <v>57.98657659676807</v>
+        <v>57.98657659676809</v>
       </c>
       <c r="O302">
-        <v>58.0108328128641</v>
+        <v>58.0108328128659</v>
       </c>
       <c r="P302">
         <v>60966</v>
@@ -20970,10 +20970,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N303">
-        <v>57.98657659676807</v>
+        <v>57.98657659676809</v>
       </c>
       <c r="O303">
-        <v>58.0108328128641</v>
+        <v>58.0108328128659</v>
       </c>
       <c r="P303">
         <v>60966</v>
@@ -21038,10 +21038,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N304">
-        <v>57.98657659676807</v>
+        <v>57.98657659676809</v>
       </c>
       <c r="O304">
-        <v>58.0108328128641</v>
+        <v>58.0108328128659</v>
       </c>
       <c r="P304">
         <v>60966</v>
@@ -21052,7 +21052,7 @@
         </is>
       </c>
       <c r="S304">
-        <v>0.9354526786854334</v>
+        <v>0.9354526786854556</v>
       </c>
     </row>
     <row r="305">
@@ -21106,10 +21106,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N305">
-        <v>57.98657659676807</v>
+        <v>57.98657659676809</v>
       </c>
       <c r="O305">
-        <v>58.0108328128641</v>
+        <v>58.0108328128659</v>
       </c>
       <c r="P305">
         <v>60966</v>
@@ -21120,7 +21120,7 @@
         </is>
       </c>
       <c r="S305">
-        <v>0.9597088947814636</v>
+        <v>0.9597088947832622</v>
       </c>
     </row>
     <row r="306">
@@ -21174,10 +21174,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N306">
-        <v>24.28635160555295</v>
+        <v>24.28635160555294</v>
       </c>
       <c r="O306">
-        <v>24.30807920702731</v>
+        <v>24.30807920702841</v>
       </c>
       <c r="P306">
         <v>54906</v>
@@ -21242,10 +21242,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N307">
-        <v>24.28635160555295</v>
+        <v>24.28635160555294</v>
       </c>
       <c r="O307">
-        <v>24.30807920702731</v>
+        <v>24.30807920702841</v>
       </c>
       <c r="P307">
         <v>54906</v>
@@ -21310,10 +21310,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N308">
-        <v>24.28635160555295</v>
+        <v>24.28635160555294</v>
       </c>
       <c r="O308">
-        <v>24.30807920702731</v>
+        <v>24.30807920702841</v>
       </c>
       <c r="P308">
         <v>54906</v>
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="S308">
-        <v>-0.3936985826528183</v>
+        <v>-0.3936985826528322</v>
       </c>
     </row>
     <row r="309">
@@ -21378,10 +21378,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N309">
-        <v>24.28635160555295</v>
+        <v>24.28635160555294</v>
       </c>
       <c r="O309">
-        <v>24.30807920702731</v>
+        <v>24.30807920702841</v>
       </c>
       <c r="P309">
         <v>54906</v>
@@ -21392,7 +21392,7 @@
         </is>
       </c>
       <c r="S309">
-        <v>-0.3719709811784599</v>
+        <v>-0.3719709811773608</v>
       </c>
     </row>
     <row r="310">
@@ -21446,10 +21446,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N310">
-        <v>86.70056156845874</v>
+        <v>86.70056156845875</v>
       </c>
       <c r="O310">
-        <v>96.82340183287779</v>
+        <v>96.82340183287785</v>
       </c>
       <c r="P310">
         <v>55751</v>
@@ -21514,10 +21514,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N311">
-        <v>86.70056156845874</v>
+        <v>86.70056156845875</v>
       </c>
       <c r="O311">
-        <v>96.82340183287779</v>
+        <v>96.82340183287785</v>
       </c>
       <c r="P311">
         <v>55751</v>
@@ -21582,10 +21582,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N312">
-        <v>86.70056156845874</v>
+        <v>86.70056156845875</v>
       </c>
       <c r="O312">
-        <v>96.82340183287779</v>
+        <v>96.82340183287785</v>
       </c>
       <c r="P312">
         <v>55751</v>
@@ -21596,7 +21596,7 @@
         </is>
       </c>
       <c r="S312">
-        <v>-3.506571111293733</v>
+        <v>-3.50657111129371</v>
       </c>
     </row>
     <row r="313">
@@ -21650,10 +21650,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N313">
-        <v>86.70056156845874</v>
+        <v>86.70056156845875</v>
       </c>
       <c r="O313">
-        <v>96.82340183287779</v>
+        <v>96.82340183287785</v>
       </c>
       <c r="P313">
         <v>55751</v>
@@ -21664,7 +21664,7 @@
         </is>
       </c>
       <c r="S313">
-        <v>6.61626915312532</v>
+        <v>6.616269153125376</v>
       </c>
     </row>
     <row r="314">
@@ -21718,10 +21718,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N314">
-        <v>59.81528043082663</v>
+        <v>59.81528043082665</v>
       </c>
       <c r="O314">
-        <v>60.34381502084364</v>
+        <v>60.34381502084475</v>
       </c>
       <c r="P314">
         <v>60920</v>
@@ -21786,10 +21786,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N315">
-        <v>59.81528043082663</v>
+        <v>59.81528043082665</v>
       </c>
       <c r="O315">
-        <v>60.34381502084364</v>
+        <v>60.34381502084475</v>
       </c>
       <c r="P315">
         <v>60920</v>
@@ -21854,10 +21854,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N316">
-        <v>59.81528043082663</v>
+        <v>59.81528043082665</v>
       </c>
       <c r="O316">
-        <v>60.34381502084364</v>
+        <v>60.34381502084475</v>
       </c>
       <c r="P316">
         <v>60920</v>
@@ -21868,7 +21868,7 @@
         </is>
       </c>
       <c r="S316">
-        <v>-1.367740548997154</v>
+        <v>-1.367740548997121</v>
       </c>
     </row>
     <row r="317">
@@ -21922,10 +21922,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N317">
-        <v>59.81528043082663</v>
+        <v>59.81528043082665</v>
       </c>
       <c r="O317">
-        <v>60.34381502084364</v>
+        <v>60.34381502084475</v>
       </c>
       <c r="P317">
         <v>60920</v>
@@ -21936,7 +21936,7 @@
         </is>
       </c>
       <c r="S317">
-        <v>-0.8392059589801382</v>
+        <v>-0.8392059589790279</v>
       </c>
     </row>
     <row r="318">
@@ -21990,10 +21990,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N318">
-        <v>51.87442533665201</v>
+        <v>51.87442533665195</v>
       </c>
       <c r="O318">
-        <v>55.19320995384727</v>
+        <v>55.19320995384758</v>
       </c>
       <c r="P318">
         <v>61000</v>
@@ -22058,10 +22058,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N319">
-        <v>51.87442533665201</v>
+        <v>51.87442533665195</v>
       </c>
       <c r="O319">
-        <v>55.19320995384727</v>
+        <v>55.19320995384758</v>
       </c>
       <c r="P319">
         <v>61000</v>
@@ -22126,10 +22126,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N320">
-        <v>51.87442533665201</v>
+        <v>51.87442533665195</v>
       </c>
       <c r="O320">
-        <v>55.19320995384727</v>
+        <v>55.19320995384758</v>
       </c>
       <c r="P320">
         <v>61000</v>
@@ -22140,7 +22140,7 @@
         </is>
       </c>
       <c r="S320">
-        <v>-0.2309273630906716</v>
+        <v>-0.2309273630907271</v>
       </c>
     </row>
     <row r="321">
@@ -22194,10 +22194,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N321">
-        <v>51.87442533665201</v>
+        <v>51.87442533665195</v>
       </c>
       <c r="O321">
-        <v>55.19320995384727</v>
+        <v>55.19320995384758</v>
       </c>
       <c r="P321">
         <v>61000</v>
@@ -22208,7 +22208,7 @@
         </is>
       </c>
       <c r="S321">
-        <v>3.087857254104587</v>
+        <v>3.087857254104898</v>
       </c>
     </row>
     <row r="322">
@@ -22262,10 +22262,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N322">
-        <v>88.60775405607029</v>
+        <v>88.60775405607038</v>
       </c>
       <c r="O322">
-        <v>92.81092514217536</v>
+        <v>92.81092514217534</v>
       </c>
       <c r="P322">
         <v>60928</v>
@@ -22330,10 +22330,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N323">
-        <v>88.60775405607029</v>
+        <v>88.60775405607038</v>
       </c>
       <c r="O323">
-        <v>92.81092514217536</v>
+        <v>92.81092514217534</v>
       </c>
       <c r="P323">
         <v>60928</v>
@@ -22398,10 +22398,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N324">
-        <v>88.60775405607029</v>
+        <v>88.60775405607038</v>
       </c>
       <c r="O324">
-        <v>92.81092514217536</v>
+        <v>92.81092514217534</v>
       </c>
       <c r="P324">
         <v>60928</v>
@@ -22412,7 +22412,7 @@
         </is>
       </c>
       <c r="S324">
-        <v>-0.3433119337774126</v>
+        <v>-0.3433119337773349</v>
       </c>
     </row>
     <row r="325">
@@ -22466,10 +22466,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N325">
-        <v>88.60775405607029</v>
+        <v>88.60775405607038</v>
       </c>
       <c r="O325">
-        <v>92.81092514217536</v>
+        <v>92.81092514217534</v>
       </c>
       <c r="P325">
         <v>60928</v>
@@ -22480,7 +22480,7 @@
         </is>
       </c>
       <c r="S325">
-        <v>3.859859152327649</v>
+        <v>3.859859152327627</v>
       </c>
     </row>
     <row r="326">
@@ -22534,10 +22534,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N326">
-        <v>92.49798818801627</v>
+        <v>92.49798818801629</v>
       </c>
       <c r="O326">
-        <v>89.42387194359372</v>
+        <v>89.42387194359381</v>
       </c>
       <c r="P326">
         <v>61000</v>
@@ -22602,10 +22602,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N327">
-        <v>92.49798818801627</v>
+        <v>92.49798818801629</v>
       </c>
       <c r="O327">
-        <v>89.42387194359372</v>
+        <v>89.42387194359381</v>
       </c>
       <c r="P327">
         <v>61000</v>
@@ -22670,10 +22670,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N328">
-        <v>92.49798818801627</v>
+        <v>92.49798818801629</v>
       </c>
       <c r="O328">
-        <v>89.42387194359372</v>
+        <v>89.42387194359381</v>
       </c>
       <c r="P328">
         <v>61000</v>
@@ -22684,7 +22684,7 @@
         </is>
       </c>
       <c r="S328">
-        <v>0.9126431762666365</v>
+        <v>0.9126431762666587</v>
       </c>
     </row>
     <row r="329">
@@ -22738,10 +22738,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N329">
-        <v>92.49798818801627</v>
+        <v>92.49798818801629</v>
       </c>
       <c r="O329">
-        <v>89.42387194359372</v>
+        <v>89.42387194359381</v>
       </c>
       <c r="P329">
         <v>61000</v>
@@ -22752,7 +22752,7 @@
         </is>
       </c>
       <c r="S329">
-        <v>-2.161473068155906</v>
+        <v>-2.161473068155828</v>
       </c>
     </row>
     <row r="330">
@@ -22806,10 +22806,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N330">
-        <v>56.80719956100185</v>
+        <v>56.80719956100195</v>
       </c>
       <c r="O330">
-        <v>53.77092581252928</v>
+        <v>53.77092581252965</v>
       </c>
       <c r="P330">
         <v>45790</v>
@@ -22874,10 +22874,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N331">
-        <v>56.80719956100185</v>
+        <v>56.80719956100195</v>
       </c>
       <c r="O331">
-        <v>53.77092581252928</v>
+        <v>53.77092581252965</v>
       </c>
       <c r="P331">
         <v>45790</v>
@@ -22942,10 +22942,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N332">
-        <v>56.80719956100185</v>
+        <v>56.80719956100195</v>
       </c>
       <c r="O332">
-        <v>53.77092581252928</v>
+        <v>53.77092581252965</v>
       </c>
       <c r="P332">
         <v>45790</v>
@@ -22956,7 +22956,7 @@
         </is>
       </c>
       <c r="S332">
-        <v>0.3061338125184943</v>
+        <v>0.3061338125185942</v>
       </c>
     </row>
     <row r="333">
@@ -23010,10 +23010,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N333">
-        <v>56.80719956100185</v>
+        <v>56.80719956100195</v>
       </c>
       <c r="O333">
-        <v>53.77092581252928</v>
+        <v>53.77092581252965</v>
       </c>
       <c r="P333">
         <v>45790</v>
@@ -23024,7 +23024,7 @@
         </is>
       </c>
       <c r="S333">
-        <v>-2.730139935954079</v>
+        <v>-2.730139935953713</v>
       </c>
     </row>
     <row r="334">
@@ -23078,10 +23078,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N334">
-        <v>62.0772182760082</v>
+        <v>62.07721827600816</v>
       </c>
       <c r="O334">
-        <v>94.75407612852116</v>
+        <v>94.75407612852125</v>
       </c>
       <c r="P334">
         <v>48462</v>
@@ -23146,10 +23146,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N335">
-        <v>62.0772182760082</v>
+        <v>62.07721827600816</v>
       </c>
       <c r="O335">
-        <v>94.75407612852116</v>
+        <v>94.75407612852125</v>
       </c>
       <c r="P335">
         <v>48462</v>
@@ -23214,10 +23214,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N336">
-        <v>62.0772182760082</v>
+        <v>62.07721827600816</v>
       </c>
       <c r="O336">
-        <v>94.75407612852116</v>
+        <v>94.75407612852125</v>
       </c>
       <c r="P336">
         <v>48462</v>
@@ -23228,7 +23228,7 @@
         </is>
       </c>
       <c r="S336">
-        <v>0.2443851464968394</v>
+        <v>0.244385146496795</v>
       </c>
     </row>
     <row r="337">
@@ -23282,10 +23282,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N337">
-        <v>62.0772182760082</v>
+        <v>62.07721827600816</v>
       </c>
       <c r="O337">
-        <v>94.75407612852116</v>
+        <v>94.75407612852125</v>
       </c>
       <c r="P337">
         <v>48462</v>
@@ -23296,7 +23296,7 @@
         </is>
       </c>
       <c r="S337">
-        <v>32.92124299900981</v>
+        <v>32.92124299900988</v>
       </c>
     </row>
     <row r="338">
@@ -23350,10 +23350,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N338">
-        <v>15.79902661390823</v>
+        <v>15.79903111329061</v>
       </c>
       <c r="O338">
-        <v>15.7990265685755</v>
+        <v>15.79902656857579</v>
       </c>
       <c r="P338">
         <v>60000</v>
@@ -23418,10 +23418,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N339">
-        <v>15.79902661390823</v>
+        <v>15.79903111329061</v>
       </c>
       <c r="O339">
-        <v>15.7990265685755</v>
+        <v>15.79902656857579</v>
       </c>
       <c r="P339">
         <v>60000</v>
@@ -23486,10 +23486,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N340">
-        <v>15.79902661390823</v>
+        <v>15.79903111329061</v>
       </c>
       <c r="O340">
-        <v>15.7990265685755</v>
+        <v>15.79902656857579</v>
       </c>
       <c r="P340">
         <v>60000</v>
@@ -23500,7 +23500,7 @@
         </is>
       </c>
       <c r="S340">
-        <v>-2.973347407419533</v>
+        <v>-2.973342908037155</v>
       </c>
     </row>
     <row r="341">
@@ -23554,10 +23554,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N341">
-        <v>15.79902661390823</v>
+        <v>15.79903111329061</v>
       </c>
       <c r="O341">
-        <v>15.7990265685755</v>
+        <v>15.79902656857579</v>
       </c>
       <c r="P341">
         <v>60000</v>
@@ -23568,7 +23568,7 @@
         </is>
       </c>
       <c r="S341">
-        <v>-2.97334745275227</v>
+        <v>-2.973347452751979</v>
       </c>
     </row>
     <row r="342">
@@ -23622,10 +23622,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N342">
-        <v>29.12343032366759</v>
+        <v>29.1234330717829</v>
       </c>
       <c r="O342">
-        <v>29.12342358088552</v>
+        <v>29.12342358088578</v>
       </c>
       <c r="P342">
         <v>60000</v>
@@ -23690,10 +23690,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N343">
-        <v>29.12343032366759</v>
+        <v>29.1234330717829</v>
       </c>
       <c r="O343">
-        <v>29.12342358088552</v>
+        <v>29.12342358088578</v>
       </c>
       <c r="P343">
         <v>60000</v>
@@ -23758,10 +23758,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N344">
-        <v>29.12343032366759</v>
+        <v>29.1234330717829</v>
       </c>
       <c r="O344">
-        <v>29.12342358088552</v>
+        <v>29.12342358088578</v>
       </c>
       <c r="P344">
         <v>60000</v>
@@ -23772,7 +23772,7 @@
         </is>
       </c>
       <c r="S344">
-        <v>-0.3447549026368069</v>
+        <v>-0.3447521545214938</v>
       </c>
     </row>
     <row r="345">
@@ -23826,10 +23826,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N345">
-        <v>29.12343032366759</v>
+        <v>29.1234330717829</v>
       </c>
       <c r="O345">
-        <v>29.12342358088552</v>
+        <v>29.12342358088578</v>
       </c>
       <c r="P345">
         <v>60000</v>
@@ -23840,7 +23840,7 @@
         </is>
       </c>
       <c r="S345">
-        <v>-0.3447616454188729</v>
+        <v>-0.3447616454186175</v>
       </c>
     </row>
     <row r="346">
@@ -23894,10 +23894,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N346">
-        <v>60.91533786695899</v>
+        <v>60.91535036081953</v>
       </c>
       <c r="O346">
-        <v>60.91538488022654</v>
+        <v>60.91538488022671</v>
       </c>
       <c r="P346">
         <v>59952</v>
@@ -23962,10 +23962,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N347">
-        <v>60.91533786695899</v>
+        <v>60.91535036081953</v>
       </c>
       <c r="O347">
-        <v>60.91538488022654</v>
+        <v>60.91538488022671</v>
       </c>
       <c r="P347">
         <v>59952</v>
@@ -24030,10 +24030,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N348">
-        <v>60.91533786695899</v>
+        <v>60.91535036081953</v>
       </c>
       <c r="O348">
-        <v>60.91538488022654</v>
+        <v>60.91538488022671</v>
       </c>
       <c r="P348">
         <v>59952</v>
@@ -24044,7 +24044,7 @@
         </is>
       </c>
       <c r="S348">
-        <v>2.019571604702652</v>
+        <v>2.019584098563187</v>
       </c>
     </row>
     <row r="349">
@@ -24098,10 +24098,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N349">
-        <v>60.91533786695899</v>
+        <v>60.91535036081953</v>
       </c>
       <c r="O349">
-        <v>60.91538488022654</v>
+        <v>60.91538488022671</v>
       </c>
       <c r="P349">
         <v>59952</v>
@@ -24112,7 +24112,7 @@
         </is>
       </c>
       <c r="S349">
-        <v>2.019618617970198</v>
+        <v>2.019618617970365</v>
       </c>
     </row>
     <row r="350">
@@ -24166,10 +24166,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N350">
-        <v>23.77362719719695</v>
+        <v>23.77362779864108</v>
       </c>
       <c r="O350">
-        <v>23.77362873790585</v>
+        <v>23.77362873790611</v>
       </c>
       <c r="P350">
         <v>55143</v>
@@ -24234,10 +24234,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N351">
-        <v>23.77362719719695</v>
+        <v>23.77362779864108</v>
       </c>
       <c r="O351">
-        <v>23.77362873790585</v>
+        <v>23.77362873790611</v>
       </c>
       <c r="P351">
         <v>55143</v>
@@ -24302,10 +24302,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N352">
-        <v>23.77362719719695</v>
+        <v>23.77362779864108</v>
       </c>
       <c r="O352">
-        <v>23.77362873790585</v>
+        <v>23.77362873790611</v>
       </c>
       <c r="P352">
         <v>55143</v>
@@ -24316,7 +24316,7 @@
         </is>
       </c>
       <c r="S352">
-        <v>-0.3448168947264851</v>
+        <v>-0.3448162932823545</v>
       </c>
     </row>
     <row r="353">
@@ -24370,10 +24370,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N353">
-        <v>23.77362719719695</v>
+        <v>23.77362779864108</v>
       </c>
       <c r="O353">
-        <v>23.77362873790585</v>
+        <v>23.77362873790611</v>
       </c>
       <c r="P353">
         <v>55143</v>
@@ -24384,7 +24384,7 @@
         </is>
       </c>
       <c r="S353">
-        <v>-0.3448153540175858</v>
+        <v>-0.3448153540173249</v>
       </c>
     </row>
     <row r="354">
@@ -24438,10 +24438,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N354">
-        <v>86.61759446798273</v>
+        <v>86.61759427225223</v>
       </c>
       <c r="O354">
-        <v>90.83563195911086</v>
+        <v>90.83563195911087</v>
       </c>
       <c r="P354">
         <v>57277</v>
@@ -24506,10 +24506,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N355">
-        <v>86.61759446798273</v>
+        <v>86.61759427225223</v>
       </c>
       <c r="O355">
-        <v>90.83563195911086</v>
+        <v>90.83563195911087</v>
       </c>
       <c r="P355">
         <v>57277</v>
@@ -24574,10 +24574,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N356">
-        <v>86.61759446798273</v>
+        <v>86.61759427225223</v>
       </c>
       <c r="O356">
-        <v>90.83563195911086</v>
+        <v>90.83563195911087</v>
       </c>
       <c r="P356">
         <v>57277</v>
@@ -24588,7 +24588,7 @@
         </is>
       </c>
       <c r="S356">
-        <v>-2.943012570225256</v>
+        <v>-2.943012765955744</v>
       </c>
     </row>
     <row r="357">
@@ -24642,10 +24642,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N357">
-        <v>86.61759446798273</v>
+        <v>86.61759427225223</v>
       </c>
       <c r="O357">
-        <v>90.83563195911086</v>
+        <v>90.83563195911087</v>
       </c>
       <c r="P357">
         <v>57277</v>
@@ -24656,7 +24656,7 @@
         </is>
       </c>
       <c r="S357">
-        <v>1.275024920902879</v>
+        <v>1.27502492090289</v>
       </c>
     </row>
     <row r="358">
@@ -24675,17 +24675,17 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Residence Duration</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>5 years or longer</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Secondary</t>
         </is>
       </c>
       <c r="G358" t="b">
@@ -24698,25 +24698,25 @@
         <v>0</v>
       </c>
       <c r="J358" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K358">
-        <v>52.08816782768694</v>
+        <v>62.78175698310654</v>
       </c>
       <c r="L358">
-        <v>53.54498598122996</v>
+        <v>61.71963677639047</v>
       </c>
       <c r="M358">
-        <v>52.20547113980047</v>
+        <v>60.99375995409059</v>
       </c>
       <c r="N358">
-        <v>51.5832883890784</v>
+        <v>61.01690685229683</v>
       </c>
       <c r="O358">
-        <v>51.69280674241715</v>
+        <v>60.71393243350647</v>
       </c>
       <c r="P358">
-        <v>59563</v>
+        <v>59908</v>
       </c>
       <c r="R358" t="inlineStr">
         <is>
@@ -24724,7 +24724,7 @@
         </is>
       </c>
       <c r="S358">
-        <v>1.456818153543016</v>
+        <v>-1.062120206716077</v>
       </c>
     </row>
     <row r="359">
@@ -24743,17 +24743,17 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Residence Duration</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>5 years or longer</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Secondary</t>
         </is>
       </c>
       <c r="G359" t="b">
@@ -24766,25 +24766,25 @@
         <v>0</v>
       </c>
       <c r="J359" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K359">
-        <v>52.08816782768694</v>
+        <v>62.78175698310654</v>
       </c>
       <c r="L359">
-        <v>53.54498598122996</v>
+        <v>61.71963677639047</v>
       </c>
       <c r="M359">
-        <v>52.20547113980047</v>
+        <v>60.99375995409059</v>
       </c>
       <c r="N359">
-        <v>51.5832883890784</v>
+        <v>61.01690685229683</v>
       </c>
       <c r="O359">
-        <v>51.69280674241715</v>
+        <v>60.71393243350647</v>
       </c>
       <c r="P359">
-        <v>59563</v>
+        <v>59908</v>
       </c>
       <c r="R359" t="inlineStr">
         <is>
@@ -24792,7 +24792,7 @@
         </is>
       </c>
       <c r="S359">
-        <v>0.1173033121135258</v>
+        <v>-1.787997029015953</v>
       </c>
     </row>
     <row r="360">
@@ -24811,17 +24811,17 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Residence Duration</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>5 years or longer</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Secondary</t>
         </is>
       </c>
       <c r="G360" t="b">
@@ -24834,25 +24834,25 @@
         <v>0</v>
       </c>
       <c r="J360" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K360">
-        <v>52.08816782768694</v>
+        <v>62.78175698310654</v>
       </c>
       <c r="L360">
-        <v>53.54498598122996</v>
+        <v>61.71963677639047</v>
       </c>
       <c r="M360">
-        <v>52.20547113980047</v>
+        <v>60.99375995409059</v>
       </c>
       <c r="N360">
-        <v>51.5832883890784</v>
+        <v>61.01690685229683</v>
       </c>
       <c r="O360">
-        <v>51.69280674241715</v>
+        <v>60.71393243350647</v>
       </c>
       <c r="P360">
-        <v>59563</v>
+        <v>59908</v>
       </c>
       <c r="R360" t="inlineStr">
         <is>
@@ -24860,7 +24860,7 @@
         </is>
       </c>
       <c r="S360">
-        <v>-0.5048794386085298</v>
+        <v>-1.764850130809714</v>
       </c>
     </row>
     <row r="361">
@@ -24879,17 +24879,17 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Residence Duration</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>5 years or longer</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Secondary</t>
         </is>
       </c>
       <c r="G361" t="b">
@@ -24902,25 +24902,25 @@
         <v>0</v>
       </c>
       <c r="J361" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K361">
-        <v>52.08816782768694</v>
+        <v>62.78175698310654</v>
       </c>
       <c r="L361">
-        <v>53.54498598122996</v>
+        <v>61.71963677639047</v>
       </c>
       <c r="M361">
-        <v>52.20547113980047</v>
+        <v>60.99375995409059</v>
       </c>
       <c r="N361">
-        <v>51.5832883890784</v>
+        <v>61.01690685229683</v>
       </c>
       <c r="O361">
-        <v>51.69280674241715</v>
+        <v>60.71393243350647</v>
       </c>
       <c r="P361">
-        <v>59563</v>
+        <v>59908</v>
       </c>
       <c r="R361" t="inlineStr">
         <is>
@@ -24928,7 +24928,7 @@
         </is>
       </c>
       <c r="S361">
-        <v>-0.3953610852697853</v>
+        <v>-2.067824549600072</v>
       </c>
     </row>
     <row r="362">
@@ -24947,17 +24947,17 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>Union Membership</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Not current union member</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G362" t="b">
@@ -24970,25 +24970,25 @@
         <v>0</v>
       </c>
       <c r="J362" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K362">
-        <v>89.75011666878791</v>
+        <v>52.08816782768694</v>
       </c>
       <c r="L362">
-        <v>93.26294368828397</v>
+        <v>53.54498598122996</v>
       </c>
       <c r="M362">
-        <v>94.03545595788032</v>
+        <v>52.20547113980047</v>
       </c>
       <c r="N362">
-        <v>89.30448547879433</v>
+        <v>51.58328699371187</v>
       </c>
       <c r="O362">
-        <v>92.04660792596596</v>
+        <v>51.69280674241718</v>
       </c>
       <c r="P362">
-        <v>59952</v>
+        <v>59563</v>
       </c>
       <c r="R362" t="inlineStr">
         <is>
@@ -24996,7 +24996,7 @@
         </is>
       </c>
       <c r="S362">
-        <v>3.512827019496045</v>
+        <v>1.456818153543016</v>
       </c>
     </row>
     <row r="363">
@@ -25015,17 +25015,17 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>Union Membership</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Not current union member</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G363" t="b">
@@ -25038,25 +25038,25 @@
         <v>0</v>
       </c>
       <c r="J363" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K363">
-        <v>89.75011666878791</v>
+        <v>52.08816782768694</v>
       </c>
       <c r="L363">
-        <v>93.26294368828397</v>
+        <v>53.54498598122996</v>
       </c>
       <c r="M363">
-        <v>94.03545595788032</v>
+        <v>52.20547113980047</v>
       </c>
       <c r="N363">
-        <v>89.30448547879433</v>
+        <v>51.58328699371187</v>
       </c>
       <c r="O363">
-        <v>92.04660792596596</v>
+        <v>51.69280674241718</v>
       </c>
       <c r="P363">
-        <v>59952</v>
+        <v>59563</v>
       </c>
       <c r="R363" t="inlineStr">
         <is>
@@ -25064,7 +25064,7 @@
         </is>
       </c>
       <c r="S363">
-        <v>4.285339289092393</v>
+        <v>0.1173033121135258</v>
       </c>
     </row>
     <row r="364">
@@ -25083,17 +25083,17 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>Union Membership</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Not current union member</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G364" t="b">
@@ -25106,25 +25106,25 @@
         <v>0</v>
       </c>
       <c r="J364" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K364">
-        <v>89.75011666878791</v>
+        <v>52.08816782768694</v>
       </c>
       <c r="L364">
-        <v>93.26294368828397</v>
+        <v>53.54498598122996</v>
       </c>
       <c r="M364">
-        <v>94.03545595788032</v>
+        <v>52.20547113980047</v>
       </c>
       <c r="N364">
-        <v>89.30448547879433</v>
+        <v>51.58328699371187</v>
       </c>
       <c r="O364">
-        <v>92.04660792596596</v>
+        <v>51.69280674241718</v>
       </c>
       <c r="P364">
-        <v>59952</v>
+        <v>59563</v>
       </c>
       <c r="R364" t="inlineStr">
         <is>
@@ -25132,7 +25132,7 @@
         </is>
       </c>
       <c r="S364">
-        <v>-0.4456311899935783</v>
+        <v>-0.5048808339750743</v>
       </c>
     </row>
     <row r="365">
@@ -25151,17 +25151,17 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>Union Membership</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>Not current union member</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G365" t="b">
@@ -25174,25 +25174,25 @@
         <v>0</v>
       </c>
       <c r="J365" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K365">
-        <v>89.75011666878791</v>
+        <v>52.08816782768694</v>
       </c>
       <c r="L365">
-        <v>93.26294368828397</v>
+        <v>53.54498598122996</v>
       </c>
       <c r="M365">
-        <v>94.03545595788032</v>
+        <v>52.20547113980047</v>
       </c>
       <c r="N365">
-        <v>89.30448547879433</v>
+        <v>51.58328699371187</v>
       </c>
       <c r="O365">
-        <v>92.04660792596596</v>
+        <v>51.69280674241718</v>
       </c>
       <c r="P365">
-        <v>59952</v>
+        <v>59563</v>
       </c>
       <c r="R365" t="inlineStr">
         <is>
@@ -25200,7 +25200,7 @@
         </is>
       </c>
       <c r="S365">
-        <v>2.296491257178046</v>
+        <v>-0.395361085269752</v>
       </c>
     </row>
     <row r="366">
@@ -25219,12 +25219,12 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>Veteran Status</t>
+          <t>Union Membership</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>Non-veteran</t>
+          <t>Not current union member</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
@@ -25245,22 +25245,22 @@
         <v>1</v>
       </c>
       <c r="K366">
-        <v>92.01159398266043</v>
+        <v>89.75011666878791</v>
       </c>
       <c r="L366">
-        <v>89.36833333333334</v>
+        <v>93.26294368828397</v>
       </c>
       <c r="M366">
-        <v>90.81416282496983</v>
+        <v>94.03545595788032</v>
       </c>
       <c r="N366">
-        <v>92.88968287704053</v>
+        <v>89.30448482920681</v>
       </c>
       <c r="O366">
-        <v>89.6150820305524</v>
+        <v>92.04660792596593</v>
       </c>
       <c r="P366">
-        <v>60000</v>
+        <v>59952</v>
       </c>
       <c r="R366" t="inlineStr">
         <is>
@@ -25268,7 +25268,7 @@
         </is>
       </c>
       <c r="S366">
-        <v>-2.643260649327084</v>
+        <v>3.512827019496045</v>
       </c>
     </row>
     <row r="367">
@@ -25287,12 +25287,12 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>Veteran Status</t>
+          <t>Union Membership</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>Non-veteran</t>
+          <t>Not current union member</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
@@ -25313,22 +25313,22 @@
         <v>1</v>
       </c>
       <c r="K367">
-        <v>92.01159398266043</v>
+        <v>89.75011666878791</v>
       </c>
       <c r="L367">
-        <v>89.36833333333334</v>
+        <v>93.26294368828397</v>
       </c>
       <c r="M367">
-        <v>90.81416282496983</v>
+        <v>94.03545595788032</v>
       </c>
       <c r="N367">
-        <v>92.88968287704053</v>
+        <v>89.30448482920681</v>
       </c>
       <c r="O367">
-        <v>89.6150820305524</v>
+        <v>92.04660792596593</v>
       </c>
       <c r="P367">
-        <v>60000</v>
+        <v>59952</v>
       </c>
       <c r="R367" t="inlineStr">
         <is>
@@ -25336,7 +25336,7 @@
         </is>
       </c>
       <c r="S367">
-        <v>-1.197431157690598</v>
+        <v>4.285339289092393</v>
       </c>
     </row>
     <row r="368">
@@ -25355,12 +25355,12 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Veteran Status</t>
+          <t>Union Membership</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>Non-veteran</t>
+          <t>Not current union member</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
@@ -25381,22 +25381,22 @@
         <v>1</v>
       </c>
       <c r="K368">
-        <v>92.01159398266043</v>
+        <v>89.75011666878791</v>
       </c>
       <c r="L368">
-        <v>89.36833333333334</v>
+        <v>93.26294368828397</v>
       </c>
       <c r="M368">
-        <v>90.81416282496983</v>
+        <v>94.03545595788032</v>
       </c>
       <c r="N368">
-        <v>92.88968287704053</v>
+        <v>89.30448482920681</v>
       </c>
       <c r="O368">
-        <v>89.6150820305524</v>
+        <v>92.04660792596593</v>
       </c>
       <c r="P368">
-        <v>60000</v>
+        <v>59952</v>
       </c>
       <c r="R368" t="inlineStr">
         <is>
@@ -25404,7 +25404,7 @@
         </is>
       </c>
       <c r="S368">
-        <v>0.8780888943801024</v>
+        <v>-0.4456318395810954</v>
       </c>
     </row>
     <row r="369">
@@ -25423,12 +25423,12 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>Veteran Status</t>
+          <t>Union Membership</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Non-veteran</t>
+          <t>Not current union member</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
@@ -25449,22 +25449,22 @@
         <v>1</v>
       </c>
       <c r="K369">
-        <v>92.01159398266043</v>
+        <v>89.75011666878791</v>
       </c>
       <c r="L369">
-        <v>89.36833333333334</v>
+        <v>93.26294368828397</v>
       </c>
       <c r="M369">
-        <v>90.81416282496983</v>
+        <v>94.03545595788032</v>
       </c>
       <c r="N369">
-        <v>92.88968287704053</v>
+        <v>89.30448482920681</v>
       </c>
       <c r="O369">
-        <v>89.6150820305524</v>
+        <v>92.04660792596593</v>
       </c>
       <c r="P369">
-        <v>60000</v>
+        <v>59952</v>
       </c>
       <c r="R369" t="inlineStr">
         <is>
@@ -25472,7 +25472,7 @@
         </is>
       </c>
       <c r="S369">
-        <v>-2.396511952108016</v>
+        <v>2.296491257178013</v>
       </c>
     </row>
     <row r="370">
@@ -25486,17 +25486,17 @@
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>Voting Administration</t>
+          <t>Demographic</t>
         </is>
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>Voting Method</t>
+          <t>Veteran Status</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>In person</t>
+          <t>Non-veteran</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
@@ -25517,22 +25517,22 @@
         <v>1</v>
       </c>
       <c r="K370">
-        <v>67.38796807857581</v>
+        <v>92.01159398266043</v>
       </c>
       <c r="L370">
-        <v>64.47793326157158</v>
+        <v>89.36833333333334</v>
       </c>
       <c r="M370">
-        <v>66.36932631856995</v>
+        <v>90.81416282496983</v>
       </c>
       <c r="N370">
-        <v>68.08470929799424</v>
+        <v>92.88968438627357</v>
       </c>
       <c r="O370">
-        <v>65.01271796233409</v>
+        <v>89.61508203055229</v>
       </c>
       <c r="P370">
-        <v>40876</v>
+        <v>60000</v>
       </c>
       <c r="R370" t="inlineStr">
         <is>
@@ -25540,7 +25540,7 @@
         </is>
       </c>
       <c r="S370">
-        <v>-2.910034817004226</v>
+        <v>-2.643260649327084</v>
       </c>
     </row>
     <row r="371">
@@ -25554,17 +25554,17 @@
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Voting Administration</t>
+          <t>Demographic</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>Voting Method</t>
+          <t>Veteran Status</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>In person</t>
+          <t>Non-veteran</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
@@ -25585,22 +25585,22 @@
         <v>1</v>
       </c>
       <c r="K371">
-        <v>67.38796807857581</v>
+        <v>92.01159398266043</v>
       </c>
       <c r="L371">
-        <v>64.47793326157158</v>
+        <v>89.36833333333334</v>
       </c>
       <c r="M371">
-        <v>66.36932631856995</v>
+        <v>90.81416282496983</v>
       </c>
       <c r="N371">
-        <v>68.08470929799424</v>
+        <v>92.88968438627357</v>
       </c>
       <c r="O371">
-        <v>65.01271796233409</v>
+        <v>89.61508203055229</v>
       </c>
       <c r="P371">
-        <v>40876</v>
+        <v>60000</v>
       </c>
       <c r="R371" t="inlineStr">
         <is>
@@ -25608,7 +25608,7 @@
         </is>
       </c>
       <c r="S371">
-        <v>-1.018641760005867</v>
+        <v>-1.197431157690598</v>
       </c>
     </row>
     <row r="372">
@@ -25622,17 +25622,17 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Voting Administration</t>
+          <t>Demographic</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>Voting Method</t>
+          <t>Veteran Status</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>In person</t>
+          <t>Non-veteran</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
@@ -25653,22 +25653,22 @@
         <v>1</v>
       </c>
       <c r="K372">
-        <v>67.38796807857581</v>
+        <v>92.01159398266043</v>
       </c>
       <c r="L372">
-        <v>64.47793326157158</v>
+        <v>89.36833333333334</v>
       </c>
       <c r="M372">
-        <v>66.36932631856995</v>
+        <v>90.81416282496983</v>
       </c>
       <c r="N372">
-        <v>68.08470929799424</v>
+        <v>92.88968438627357</v>
       </c>
       <c r="O372">
-        <v>65.01271796233409</v>
+        <v>89.61508203055229</v>
       </c>
       <c r="P372">
-        <v>40876</v>
+        <v>60000</v>
       </c>
       <c r="R372" t="inlineStr">
         <is>
@@ -25676,7 +25676,7 @@
         </is>
       </c>
       <c r="S372">
-        <v>0.6967412194184286</v>
+        <v>0.878090403613152</v>
       </c>
     </row>
     <row r="373">
@@ -25690,17 +25690,17 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>Voting Administration</t>
+          <t>Demographic</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>Voting Method</t>
+          <t>Veteran Status</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>In person</t>
+          <t>Non-veteran</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
@@ -25721,22 +25721,22 @@
         <v>1</v>
       </c>
       <c r="K373">
-        <v>67.38796807857581</v>
+        <v>92.01159398266043</v>
       </c>
       <c r="L373">
-        <v>64.47793326157158</v>
+        <v>89.36833333333334</v>
       </c>
       <c r="M373">
-        <v>66.36932631856995</v>
+        <v>90.81416282496983</v>
       </c>
       <c r="N373">
-        <v>68.08470929799424</v>
+        <v>92.88968438627357</v>
       </c>
       <c r="O373">
-        <v>65.01271796233409</v>
+        <v>89.61508203055229</v>
       </c>
       <c r="P373">
-        <v>40876</v>
+        <v>60000</v>
       </c>
       <c r="R373" t="inlineStr">
         <is>
@@ -25744,7 +25744,7 @@
         </is>
       </c>
       <c r="S373">
-        <v>-2.375250116241723</v>
+        <v>-2.396511952108138</v>
       </c>
     </row>
     <row r="374">
@@ -25763,12 +25763,12 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>Voting Turnout</t>
+          <t>Voting Method</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Did not vote</t>
+          <t>In person</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
@@ -25789,22 +25789,22 @@
         <v>1</v>
       </c>
       <c r="K374">
-        <v>57.1867220532585</v>
+        <v>67.38796807857581</v>
       </c>
       <c r="L374">
-        <v>15.30204431796782</v>
+        <v>64.47793326157158</v>
       </c>
       <c r="M374">
-        <v>7.294531710394677</v>
+        <v>66.36932631856995</v>
       </c>
       <c r="N374">
-        <v>57.18662972561633</v>
+        <v>68.08470983266751</v>
       </c>
       <c r="O374">
-        <v>14.73483535187088</v>
+        <v>65.01271796233431</v>
       </c>
       <c r="P374">
-        <v>47791</v>
+        <v>40876</v>
       </c>
       <c r="R374" t="inlineStr">
         <is>
@@ -25812,7 +25812,7 @@
         </is>
       </c>
       <c r="S374">
-        <v>-41.88467773529068</v>
+        <v>-2.910034817004226</v>
       </c>
     </row>
     <row r="375">
@@ -25831,12 +25831,12 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>Voting Turnout</t>
+          <t>Voting Method</t>
         </is>
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Did not vote</t>
+          <t>In person</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
@@ -25857,22 +25857,22 @@
         <v>1</v>
       </c>
       <c r="K375">
-        <v>57.1867220532585</v>
+        <v>67.38796807857581</v>
       </c>
       <c r="L375">
-        <v>15.30204431796782</v>
+        <v>64.47793326157158</v>
       </c>
       <c r="M375">
-        <v>7.294531710394677</v>
+        <v>66.36932631856995</v>
       </c>
       <c r="N375">
-        <v>57.18662972561633</v>
+        <v>68.08470983266751</v>
       </c>
       <c r="O375">
-        <v>14.73483535187088</v>
+        <v>65.01271796233431</v>
       </c>
       <c r="P375">
-        <v>47791</v>
+        <v>40876</v>
       </c>
       <c r="R375" t="inlineStr">
         <is>
@@ -25880,7 +25880,7 @@
         </is>
       </c>
       <c r="S375">
-        <v>-49.89219034286382</v>
+        <v>-1.018641760005867</v>
       </c>
     </row>
     <row r="376">
@@ -25899,12 +25899,12 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>Voting Turnout</t>
+          <t>Voting Method</t>
         </is>
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Did not vote</t>
+          <t>In person</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
@@ -25925,22 +25925,22 @@
         <v>1</v>
       </c>
       <c r="K376">
-        <v>57.1867220532585</v>
+        <v>67.38796807857581</v>
       </c>
       <c r="L376">
-        <v>15.30204431796782</v>
+        <v>64.47793326157158</v>
       </c>
       <c r="M376">
-        <v>7.294531710394677</v>
+        <v>66.36932631856995</v>
       </c>
       <c r="N376">
-        <v>57.18662972561633</v>
+        <v>68.08470983266751</v>
       </c>
       <c r="O376">
-        <v>14.73483535187088</v>
+        <v>65.01271796233431</v>
       </c>
       <c r="P376">
-        <v>47791</v>
+        <v>40876</v>
       </c>
       <c r="R376" t="inlineStr">
         <is>
@@ -25948,7 +25948,7 @@
         </is>
       </c>
       <c r="S376">
-        <v>-9.23276421649355E-05</v>
+        <v>0.6967417540917009</v>
       </c>
     </row>
     <row r="377">
@@ -25967,56 +25967,328 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
+          <t>Voting Method</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>In person</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="G377" t="b">
+        <v>1</v>
+      </c>
+      <c r="H377" t="b">
+        <v>0</v>
+      </c>
+      <c r="I377" t="b">
+        <v>0</v>
+      </c>
+      <c r="J377" t="b">
+        <v>1</v>
+      </c>
+      <c r="K377">
+        <v>67.38796807857581</v>
+      </c>
+      <c r="L377">
+        <v>64.47793326157158</v>
+      </c>
+      <c r="M377">
+        <v>66.36932631856995</v>
+      </c>
+      <c r="N377">
+        <v>68.08470983266751</v>
+      </c>
+      <c r="O377">
+        <v>65.01271796233431</v>
+      </c>
+      <c r="P377">
+        <v>40876</v>
+      </c>
+      <c r="R377" t="inlineStr">
+        <is>
+          <t>ANESRake-Restricted</t>
+        </is>
+      </c>
+      <c r="S377">
+        <v>-2.375250116241501</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378">
+        <v>2022</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>NATIONAL</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Voting Administration</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
           <t>Voting Turnout</t>
         </is>
       </c>
-      <c r="E377" t="inlineStr">
+      <c r="E378" t="inlineStr">
         <is>
           <t>Did not vote</t>
         </is>
       </c>
-      <c r="F377" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
-      <c r="G377" t="b">
-        <v>1</v>
-      </c>
-      <c r="H377" t="b">
-        <v>0</v>
-      </c>
-      <c r="I377" t="b">
-        <v>0</v>
-      </c>
-      <c r="J377" t="b">
-        <v>1</v>
-      </c>
-      <c r="K377">
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="G378" t="b">
+        <v>1</v>
+      </c>
+      <c r="H378" t="b">
+        <v>0</v>
+      </c>
+      <c r="I378" t="b">
+        <v>0</v>
+      </c>
+      <c r="J378" t="b">
+        <v>1</v>
+      </c>
+      <c r="K378">
         <v>57.1867220532585</v>
       </c>
-      <c r="L377">
+      <c r="L378">
         <v>15.30204431796782</v>
       </c>
-      <c r="M377">
+      <c r="M378">
         <v>7.294531710394677</v>
       </c>
-      <c r="N377">
-        <v>57.18662972561633</v>
-      </c>
-      <c r="O377">
-        <v>14.73483535187088</v>
-      </c>
-      <c r="P377">
+      <c r="N378">
+        <v>57.18663105574594</v>
+      </c>
+      <c r="O378">
+        <v>14.7348353518708</v>
+      </c>
+      <c r="P378">
         <v>47791</v>
       </c>
-      <c r="R377" t="inlineStr">
+      <c r="R378" t="inlineStr">
+        <is>
+          <t>CES-Unweighted</t>
+        </is>
+      </c>
+      <c r="S378">
+        <v>-41.88467773529068</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379">
+        <v>2022</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>NATIONAL</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Voting Administration</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Voting Turnout</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Did not vote</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="G379" t="b">
+        <v>1</v>
+      </c>
+      <c r="H379" t="b">
+        <v>0</v>
+      </c>
+      <c r="I379" t="b">
+        <v>0</v>
+      </c>
+      <c r="J379" t="b">
+        <v>1</v>
+      </c>
+      <c r="K379">
+        <v>57.1867220532585</v>
+      </c>
+      <c r="L379">
+        <v>15.30204431796782</v>
+      </c>
+      <c r="M379">
+        <v>7.294531710394677</v>
+      </c>
+      <c r="N379">
+        <v>57.18663105574594</v>
+      </c>
+      <c r="O379">
+        <v>14.7348353518708</v>
+      </c>
+      <c r="P379">
+        <v>47791</v>
+      </c>
+      <c r="R379" t="inlineStr">
+        <is>
+          <t>CES-Provided Weights</t>
+        </is>
+      </c>
+      <c r="S379">
+        <v>-49.89219034286382</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380">
+        <v>2022</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>NATIONAL</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Voting Administration</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Voting Turnout</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Did not vote</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="G380" t="b">
+        <v>1</v>
+      </c>
+      <c r="H380" t="b">
+        <v>0</v>
+      </c>
+      <c r="I380" t="b">
+        <v>0</v>
+      </c>
+      <c r="J380" t="b">
+        <v>1</v>
+      </c>
+      <c r="K380">
+        <v>57.1867220532585</v>
+      </c>
+      <c r="L380">
+        <v>15.30204431796782</v>
+      </c>
+      <c r="M380">
+        <v>7.294531710394677</v>
+      </c>
+      <c r="N380">
+        <v>57.18663105574594</v>
+      </c>
+      <c r="O380">
+        <v>14.7348353518708</v>
+      </c>
+      <c r="P380">
+        <v>47791</v>
+      </c>
+      <c r="R380" t="inlineStr">
+        <is>
+          <t>ANESRake-Full</t>
+        </is>
+      </c>
+      <c r="S380">
+        <v>-9.099751255847721E-05</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381">
+        <v>2022</v>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>NATIONAL</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Voting Administration</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Voting Turnout</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Did not vote</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="G381" t="b">
+        <v>1</v>
+      </c>
+      <c r="H381" t="b">
+        <v>0</v>
+      </c>
+      <c r="I381" t="b">
+        <v>0</v>
+      </c>
+      <c r="J381" t="b">
+        <v>1</v>
+      </c>
+      <c r="K381">
+        <v>57.1867220532585</v>
+      </c>
+      <c r="L381">
+        <v>15.30204431796782</v>
+      </c>
+      <c r="M381">
+        <v>7.294531710394677</v>
+      </c>
+      <c r="N381">
+        <v>57.18663105574594</v>
+      </c>
+      <c r="O381">
+        <v>14.7348353518708</v>
+      </c>
+      <c r="P381">
+        <v>47791</v>
+      </c>
+      <c r="R381" t="inlineStr">
         <is>
           <t>ANESRake-Restricted</t>
         </is>
       </c>
-      <c r="S377">
-        <v>-42.45188670138761</v>
+      <c r="S381">
+        <v>-42.4518867013877</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update analysisHQ, special election candidates, and input tables
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/tables_and_figures/input_tables/national_errors.xlsx
+++ b/tables_and_figures/input_tables/national_errors.xlsx
@@ -5670,10 +5670,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N78">
-        <v>21.68983558756369</v>
+        <v>21.68983558756392</v>
       </c>
       <c r="O78">
-        <v>21.68983558756393</v>
+        <v>21.68983558756405</v>
       </c>
       <c r="P78">
         <v>55400</v>
@@ -5738,10 +5738,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N79">
-        <v>21.68983558756369</v>
+        <v>21.68983558756392</v>
       </c>
       <c r="O79">
-        <v>21.68983558756393</v>
+        <v>21.68983558756405</v>
       </c>
       <c r="P79">
         <v>55400</v>
@@ -5806,10 +5806,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N80">
-        <v>21.68983558756369</v>
+        <v>21.68983558756392</v>
       </c>
       <c r="O80">
-        <v>21.68983558756393</v>
+        <v>21.68983558756405</v>
       </c>
       <c r="P80">
         <v>55400</v>
@@ -5820,7 +5820,7 @@
         </is>
       </c>
       <c r="S80">
-        <v>1.936748087924511</v>
+        <v>1.936748087924742</v>
       </c>
     </row>
     <row r="81">
@@ -5874,10 +5874,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N81">
-        <v>21.68983558756369</v>
+        <v>21.68983558756392</v>
       </c>
       <c r="O81">
-        <v>21.68983558756393</v>
+        <v>21.68983558756405</v>
       </c>
       <c r="P81">
         <v>55400</v>
@@ -5888,7 +5888,7 @@
         </is>
       </c>
       <c r="S81">
-        <v>1.936748087924747</v>
+        <v>1.936748087924864</v>
       </c>
     </row>
     <row r="82">
@@ -5942,10 +5942,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N82">
-        <v>32.131084023464</v>
+        <v>32.13108402346401</v>
       </c>
       <c r="O82">
-        <v>32.13108402346392</v>
+        <v>32.13108402346418</v>
       </c>
       <c r="P82">
         <v>55400</v>
@@ -6010,10 +6010,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N83">
-        <v>32.131084023464</v>
+        <v>32.13108402346401</v>
       </c>
       <c r="O83">
-        <v>32.13108402346392</v>
+        <v>32.13108402346418</v>
       </c>
       <c r="P83">
         <v>55400</v>
@@ -6078,10 +6078,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N84">
-        <v>32.131084023464</v>
+        <v>32.13108402346401</v>
       </c>
       <c r="O84">
-        <v>32.13108402346392</v>
+        <v>32.13108402346418</v>
       </c>
       <c r="P84">
         <v>55400</v>
@@ -6092,7 +6092,7 @@
         </is>
       </c>
       <c r="S84">
-        <v>0.44453379206007</v>
+        <v>0.4445337920600756</v>
       </c>
     </row>
     <row r="85">
@@ -6146,10 +6146,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N85">
-        <v>32.131084023464</v>
+        <v>32.13108402346401</v>
       </c>
       <c r="O85">
-        <v>32.13108402346392</v>
+        <v>32.13108402346418</v>
       </c>
       <c r="P85">
         <v>55400</v>
@@ -6160,7 +6160,7 @@
         </is>
       </c>
       <c r="S85">
-        <v>0.4445337920599868</v>
+        <v>0.4445337920602477</v>
       </c>
     </row>
     <row r="86">
@@ -6214,10 +6214,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N86">
-        <v>60.64538348495072</v>
+        <v>60.64538348494989</v>
       </c>
       <c r="O86">
-        <v>60.64538348495044</v>
+        <v>60.64538348495076</v>
       </c>
       <c r="P86">
         <v>55400</v>
@@ -6282,10 +6282,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N87">
-        <v>60.64538348495072</v>
+        <v>60.64538348494989</v>
       </c>
       <c r="O87">
-        <v>60.64538348495044</v>
+        <v>60.64538348495076</v>
       </c>
       <c r="P87">
         <v>55400</v>
@@ -6350,10 +6350,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N88">
-        <v>60.64538348495072</v>
+        <v>60.64538348494989</v>
       </c>
       <c r="O88">
-        <v>60.64538348495044</v>
+        <v>60.64538348495076</v>
       </c>
       <c r="P88">
         <v>55400</v>
@@ -6364,7 +6364,7 @@
         </is>
       </c>
       <c r="S88">
-        <v>-0.2387361085900874</v>
+        <v>-0.2387361085909201</v>
       </c>
     </row>
     <row r="89">
@@ -6418,10 +6418,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N89">
-        <v>60.64538348495072</v>
+        <v>60.64538348494989</v>
       </c>
       <c r="O89">
-        <v>60.64538348495044</v>
+        <v>60.64538348495076</v>
       </c>
       <c r="P89">
         <v>55400</v>
@@ -6432,7 +6432,7 @@
         </is>
       </c>
       <c r="S89">
-        <v>-0.238736108590365</v>
+        <v>-0.238736108590043</v>
       </c>
     </row>
     <row r="90">
@@ -6486,10 +6486,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N90">
-        <v>23.19167199619718</v>
+        <v>23.19167199619754</v>
       </c>
       <c r="O90">
-        <v>23.19287782028157</v>
+        <v>23.19287782028184</v>
       </c>
       <c r="P90">
         <v>48612</v>
@@ -6554,10 +6554,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N91">
-        <v>23.19167199619718</v>
+        <v>23.19167199619754</v>
       </c>
       <c r="O91">
-        <v>23.19287782028157</v>
+        <v>23.19287782028184</v>
       </c>
       <c r="P91">
         <v>48612</v>
@@ -6622,10 +6622,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N92">
-        <v>23.19167199619718</v>
+        <v>23.19167199619754</v>
       </c>
       <c r="O92">
-        <v>23.19287782028157</v>
+        <v>23.19287782028184</v>
       </c>
       <c r="P92">
         <v>48612</v>
@@ -6636,7 +6636,7 @@
         </is>
       </c>
       <c r="S92">
-        <v>-0.2830345174889337</v>
+        <v>-0.2830345174885757</v>
       </c>
     </row>
     <row r="93">
@@ -6690,10 +6690,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N93">
-        <v>23.19167199619718</v>
+        <v>23.19167199619754</v>
       </c>
       <c r="O93">
-        <v>23.19287782028157</v>
+        <v>23.19287782028184</v>
       </c>
       <c r="P93">
         <v>48612</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="S93">
-        <v>-0.2818286934045483</v>
+        <v>-0.2818286934042763</v>
       </c>
     </row>
     <row r="94">
@@ -6758,10 +6758,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N94">
-        <v>90.07772910426878</v>
+        <v>90.07772910426883</v>
       </c>
       <c r="O94">
-        <v>95.5694528334882</v>
+        <v>95.56945283348823</v>
       </c>
       <c r="P94">
         <v>49058</v>
@@ -6826,10 +6826,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N95">
-        <v>90.07772910426878</v>
+        <v>90.07772910426883</v>
       </c>
       <c r="O95">
-        <v>95.5694528334882</v>
+        <v>95.56945283348823</v>
       </c>
       <c r="P95">
         <v>49058</v>
@@ -6894,10 +6894,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N96">
-        <v>90.07772910426878</v>
+        <v>90.07772910426883</v>
       </c>
       <c r="O96">
-        <v>95.5694528334882</v>
+        <v>95.56945283348823</v>
       </c>
       <c r="P96">
         <v>49058</v>
@@ -6908,7 +6908,7 @@
         </is>
       </c>
       <c r="S96">
-        <v>-2.0360808689739</v>
+        <v>-2.036080868973866</v>
       </c>
     </row>
     <row r="97">
@@ -6962,10 +6962,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N97">
-        <v>90.07772910426878</v>
+        <v>90.07772910426883</v>
       </c>
       <c r="O97">
-        <v>95.5694528334882</v>
+        <v>95.56945283348823</v>
       </c>
       <c r="P97">
         <v>49058</v>
@@ -6976,7 +6976,7 @@
         </is>
       </c>
       <c r="S97">
-        <v>3.455642860245511</v>
+        <v>3.455642860245545</v>
       </c>
     </row>
     <row r="98">
@@ -7030,10 +7030,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N98">
-        <v>60.39792154911988</v>
+        <v>60.39792154911977</v>
       </c>
       <c r="O98">
-        <v>61.38848427025866</v>
+        <v>61.3884842702589</v>
       </c>
       <c r="P98">
         <v>55325</v>
@@ -7098,10 +7098,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N99">
-        <v>60.39792154911988</v>
+        <v>60.39792154911977</v>
       </c>
       <c r="O99">
-        <v>61.38848427025866</v>
+        <v>61.3884842702589</v>
       </c>
       <c r="P99">
         <v>55325</v>
@@ -7166,10 +7166,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N100">
-        <v>60.39792154911988</v>
+        <v>60.39792154911977</v>
       </c>
       <c r="O100">
-        <v>61.38848427025866</v>
+        <v>61.3884842702589</v>
       </c>
       <c r="P100">
         <v>55325</v>
@@ -7180,7 +7180,7 @@
         </is>
       </c>
       <c r="S100">
-        <v>-1.44705391069867</v>
+        <v>-1.447053910698781</v>
       </c>
     </row>
     <row r="101">
@@ -7234,10 +7234,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N101">
-        <v>60.39792154911988</v>
+        <v>60.39792154911977</v>
       </c>
       <c r="O101">
-        <v>61.38848427025866</v>
+        <v>61.3884842702589</v>
       </c>
       <c r="P101">
         <v>55325</v>
@@ -7248,7 +7248,7 @@
         </is>
       </c>
       <c r="S101">
-        <v>-0.4564911895598933</v>
+        <v>-0.4564911895596491</v>
       </c>
     </row>
     <row r="102">
@@ -7302,10 +7302,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N102">
-        <v>51.96851035400858</v>
+        <v>51.9685103540086</v>
       </c>
       <c r="O102">
-        <v>55.16820532599596</v>
+        <v>55.16820532599615</v>
       </c>
       <c r="P102">
         <v>55400</v>
@@ -7370,10 +7370,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N103">
-        <v>51.96851035400858</v>
+        <v>51.9685103540086</v>
       </c>
       <c r="O103">
-        <v>55.16820532599596</v>
+        <v>55.16820532599615</v>
       </c>
       <c r="P103">
         <v>55400</v>
@@ -7438,10 +7438,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N104">
-        <v>51.96851035400858</v>
+        <v>51.9685103540086</v>
       </c>
       <c r="O104">
-        <v>55.16820532599596</v>
+        <v>55.16820532599615</v>
       </c>
       <c r="P104">
         <v>55400</v>
@@ -7452,7 +7452,7 @@
         </is>
       </c>
       <c r="S104">
-        <v>-0.4053152415143146</v>
+        <v>-0.4053152415142924</v>
       </c>
     </row>
     <row r="105">
@@ -7506,10 +7506,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N105">
-        <v>51.96851035400858</v>
+        <v>51.9685103540086</v>
       </c>
       <c r="O105">
-        <v>55.16820532599596</v>
+        <v>55.16820532599615</v>
       </c>
       <c r="P105">
         <v>55400</v>
@@ -7520,7 +7520,7 @@
         </is>
       </c>
       <c r="S105">
-        <v>2.794379730473062</v>
+        <v>2.794379730473251</v>
       </c>
     </row>
     <row r="106">
@@ -7574,10 +7574,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N106">
-        <v>87.32994267910654</v>
+        <v>87.32994267910608</v>
       </c>
       <c r="O106">
-        <v>92.33804839648147</v>
+        <v>92.33804839648158</v>
       </c>
       <c r="P106">
         <v>55242</v>
@@ -7642,10 +7642,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N107">
-        <v>87.32994267910654</v>
+        <v>87.32994267910608</v>
       </c>
       <c r="O107">
-        <v>92.33804839648147</v>
+        <v>92.33804839648158</v>
       </c>
       <c r="P107">
         <v>55242</v>
@@ -7710,10 +7710,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N108">
-        <v>87.32994267910654</v>
+        <v>87.32994267910608</v>
       </c>
       <c r="O108">
-        <v>92.33804839648147</v>
+        <v>92.33804839648158</v>
       </c>
       <c r="P108">
         <v>55242</v>
@@ -7724,7 +7724,7 @@
         </is>
       </c>
       <c r="S108">
-        <v>-0.1009559809638128</v>
+        <v>-0.1009559809642679</v>
       </c>
     </row>
     <row r="109">
@@ -7778,10 +7778,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N109">
-        <v>87.32994267910654</v>
+        <v>87.32994267910608</v>
       </c>
       <c r="O109">
-        <v>92.33804839648147</v>
+        <v>92.33804839648158</v>
       </c>
       <c r="P109">
         <v>55242</v>
@@ -7792,7 +7792,7 @@
         </is>
       </c>
       <c r="S109">
-        <v>4.907149736411109</v>
+        <v>4.907149736411231</v>
       </c>
     </row>
     <row r="110">
@@ -7846,10 +7846,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N110">
-        <v>90.29738719024533</v>
+        <v>90.29738719024508</v>
       </c>
       <c r="O110">
-        <v>85.14002215874858</v>
+        <v>85.14002215874885</v>
       </c>
       <c r="P110">
         <v>55400</v>
@@ -7914,10 +7914,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N111">
-        <v>90.29738719024533</v>
+        <v>90.29738719024508</v>
       </c>
       <c r="O111">
-        <v>85.14002215874858</v>
+        <v>85.14002215874885</v>
       </c>
       <c r="P111">
         <v>55400</v>
@@ -7982,10 +7982,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N112">
-        <v>90.29738719024533</v>
+        <v>90.29738719024508</v>
       </c>
       <c r="O112">
-        <v>85.14002215874858</v>
+        <v>85.14002215874885</v>
       </c>
       <c r="P112">
         <v>55400</v>
@@ -7996,7 +7996,7 @@
         </is>
       </c>
       <c r="S112">
-        <v>0.7294136856202504</v>
+        <v>0.729413685619984</v>
       </c>
     </row>
     <row r="113">
@@ -8050,10 +8050,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N113">
-        <v>90.29738719024533</v>
+        <v>90.29738719024508</v>
       </c>
       <c r="O113">
-        <v>85.14002215874858</v>
+        <v>85.14002215874885</v>
       </c>
       <c r="P113">
         <v>55400</v>
@@ -8064,7 +8064,7 @@
         </is>
       </c>
       <c r="S113">
-        <v>-4.427951345876502</v>
+        <v>-4.427951345876235</v>
       </c>
     </row>
     <row r="114">
@@ -8118,10 +8118,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N114">
-        <v>81.97678428265843</v>
+        <v>81.97678428265853</v>
       </c>
       <c r="O114">
-        <v>78.85814310205271</v>
+        <v>78.85814310205289</v>
       </c>
       <c r="P114">
         <v>37859</v>
@@ -8186,10 +8186,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N115">
-        <v>81.97678428265843</v>
+        <v>81.97678428265853</v>
       </c>
       <c r="O115">
-        <v>78.85814310205271</v>
+        <v>78.85814310205289</v>
       </c>
       <c r="P115">
         <v>37859</v>
@@ -8254,10 +8254,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N116">
-        <v>81.97678428265843</v>
+        <v>81.97678428265853</v>
       </c>
       <c r="O116">
-        <v>78.85814310205271</v>
+        <v>78.85814310205289</v>
       </c>
       <c r="P116">
         <v>37859</v>
@@ -8268,7 +8268,7 @@
         </is>
       </c>
       <c r="S116">
-        <v>-0.8086498910110373</v>
+        <v>-0.8086498910109485</v>
       </c>
     </row>
     <row r="117">
@@ -8322,10 +8322,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N117">
-        <v>81.97678428265843</v>
+        <v>81.97678428265853</v>
       </c>
       <c r="O117">
-        <v>78.85814310205271</v>
+        <v>78.85814310205289</v>
       </c>
       <c r="P117">
         <v>37859</v>
@@ -8336,7 +8336,7 @@
         </is>
       </c>
       <c r="S117">
-        <v>-3.927291071616756</v>
+        <v>-3.927291071616579</v>
       </c>
     </row>
     <row r="118">
@@ -8390,10 +8390,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N118">
-        <v>61.84561105159537</v>
+        <v>61.84561105159655</v>
       </c>
       <c r="O118">
-        <v>26.29907721541595</v>
+        <v>26.29907721541566</v>
       </c>
       <c r="P118">
         <v>44776</v>
@@ -8458,10 +8458,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N119">
-        <v>61.84561105159537</v>
+        <v>61.84561105159655</v>
       </c>
       <c r="O119">
-        <v>26.29907721541595</v>
+        <v>26.29907721541566</v>
       </c>
       <c r="P119">
         <v>44776</v>
@@ -8526,10 +8526,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N120">
-        <v>61.84561105159537</v>
+        <v>61.84561105159655</v>
       </c>
       <c r="O120">
-        <v>26.29907721541595</v>
+        <v>26.29907721541566</v>
       </c>
       <c r="P120">
         <v>44776</v>
@@ -8540,7 +8540,7 @@
         </is>
       </c>
       <c r="S120">
-        <v>0.3570698780789416</v>
+        <v>0.3570698780801185</v>
       </c>
     </row>
     <row r="121">
@@ -8594,10 +8594,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N121">
-        <v>61.84561105159537</v>
+        <v>61.84561105159655</v>
       </c>
       <c r="O121">
-        <v>26.29907721541595</v>
+        <v>26.29907721541566</v>
       </c>
       <c r="P121">
         <v>44776</v>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="S121">
-        <v>-35.18946395810048</v>
+        <v>-35.18946395810077</v>
       </c>
     </row>
     <row r="122">
@@ -8662,10 +8662,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N122">
-        <v>18.78381922591102</v>
+        <v>18.78381922591106</v>
       </c>
       <c r="O122">
-        <v>18.78376405592434</v>
+        <v>18.78376405592467</v>
       </c>
       <c r="P122">
         <v>54535</v>
@@ -8730,10 +8730,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N123">
-        <v>18.78381922591102</v>
+        <v>18.78381922591106</v>
       </c>
       <c r="O123">
-        <v>18.78376405592434</v>
+        <v>18.78376405592467</v>
       </c>
       <c r="P123">
         <v>54535</v>
@@ -8798,10 +8798,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N124">
-        <v>18.78381922591102</v>
+        <v>18.78381922591106</v>
       </c>
       <c r="O124">
-        <v>18.78376405592434</v>
+        <v>18.78376405592467</v>
       </c>
       <c r="P124">
         <v>54535</v>
@@ -8812,7 +8812,7 @@
         </is>
       </c>
       <c r="S124">
-        <v>-0.5877807213773845</v>
+        <v>-0.5877807213773428</v>
       </c>
     </row>
     <row r="125">
@@ -8866,10 +8866,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N125">
-        <v>18.78381922591102</v>
+        <v>18.78381922591106</v>
       </c>
       <c r="O125">
-        <v>18.78376405592434</v>
+        <v>18.78376405592467</v>
       </c>
       <c r="P125">
         <v>54535</v>
@@ -8880,7 +8880,7 @@
         </is>
       </c>
       <c r="S125">
-        <v>-0.5878358913640636</v>
+        <v>-0.587835891363736</v>
       </c>
     </row>
     <row r="126">
@@ -8934,10 +8934,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N126">
-        <v>30.53786279215657</v>
+        <v>30.53786279215646</v>
       </c>
       <c r="O126">
-        <v>30.53774451303544</v>
+        <v>30.53774451303555</v>
       </c>
       <c r="P126">
         <v>54535</v>
@@ -9002,10 +9002,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N127">
-        <v>30.53786279215657</v>
+        <v>30.53786279215646</v>
       </c>
       <c r="O127">
-        <v>30.53774451303544</v>
+        <v>30.53774451303555</v>
       </c>
       <c r="P127">
         <v>54535</v>
@@ -9070,10 +9070,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N128">
-        <v>30.53786279215657</v>
+        <v>30.53786279215646</v>
       </c>
       <c r="O128">
-        <v>30.53774451303544</v>
+        <v>30.53774451303555</v>
       </c>
       <c r="P128">
         <v>54535</v>
@@ -9084,7 +9084,7 @@
         </is>
       </c>
       <c r="S128">
-        <v>-0.1367483492705823</v>
+        <v>-0.1367483492706933</v>
       </c>
     </row>
     <row r="129">
@@ -9138,10 +9138,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N129">
-        <v>30.53786279215657</v>
+        <v>30.53786279215646</v>
       </c>
       <c r="O129">
-        <v>30.53774451303544</v>
+        <v>30.53774451303555</v>
       </c>
       <c r="P129">
         <v>54535</v>
@@ -9152,7 +9152,7 @@
         </is>
       </c>
       <c r="S129">
-        <v>-0.136866628391713</v>
+        <v>-0.136866628391602</v>
       </c>
     </row>
     <row r="130">
@@ -9206,10 +9206,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N130">
-        <v>60.07048159861138</v>
+        <v>60.0704815986113</v>
       </c>
       <c r="O130">
-        <v>60.07051969567385</v>
+        <v>60.07051969567441</v>
       </c>
       <c r="P130">
         <v>54535</v>
@@ -9274,10 +9274,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N131">
-        <v>60.07048159861138</v>
+        <v>60.0704815986113</v>
       </c>
       <c r="O131">
-        <v>60.07051969567385</v>
+        <v>60.07051969567441</v>
       </c>
       <c r="P131">
         <v>54535</v>
@@ -9342,10 +9342,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N132">
-        <v>60.07048159861138</v>
+        <v>60.0704815986113</v>
       </c>
       <c r="O132">
-        <v>60.07051969567385</v>
+        <v>60.07051969567441</v>
       </c>
       <c r="P132">
         <v>54535</v>
@@ -9356,7 +9356,7 @@
         </is>
       </c>
       <c r="S132">
-        <v>-0.7931925941980889</v>
+        <v>-0.7931925941981666</v>
       </c>
     </row>
     <row r="133">
@@ -9410,10 +9410,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N133">
-        <v>60.07048159861138</v>
+        <v>60.0704815986113</v>
       </c>
       <c r="O133">
-        <v>60.07051969567385</v>
+        <v>60.07051969567441</v>
       </c>
       <c r="P133">
         <v>54535</v>
@@ -9424,7 +9424,7 @@
         </is>
       </c>
       <c r="S133">
-        <v>-0.7931544971356175</v>
+        <v>-0.7931544971350624</v>
       </c>
     </row>
     <row r="134">
@@ -9478,10 +9478,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N134">
-        <v>22.80752813266336</v>
+        <v>22.8075281326633</v>
       </c>
       <c r="O134">
-        <v>22.80764277056756</v>
+        <v>22.80764277056721</v>
       </c>
       <c r="P134">
         <v>47918</v>
@@ -9546,10 +9546,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N135">
-        <v>22.80752813266336</v>
+        <v>22.8075281326633</v>
       </c>
       <c r="O135">
-        <v>22.80764277056756</v>
+        <v>22.80764277056721</v>
       </c>
       <c r="P135">
         <v>47918</v>
@@ -9614,10 +9614,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N136">
-        <v>22.80752813266336</v>
+        <v>22.8075281326633</v>
       </c>
       <c r="O136">
-        <v>22.80764277056756</v>
+        <v>22.80764277056721</v>
       </c>
       <c r="P136">
         <v>47918</v>
@@ -9628,7 +9628,7 @@
         </is>
       </c>
       <c r="S136">
-        <v>-0.6564727659101488</v>
+        <v>-0.6564727659102182</v>
       </c>
     </row>
     <row r="137">
@@ -9682,10 +9682,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N137">
-        <v>22.80752813266336</v>
+        <v>22.8075281326633</v>
       </c>
       <c r="O137">
-        <v>22.80764277056756</v>
+        <v>22.80764277056721</v>
       </c>
       <c r="P137">
         <v>47918</v>
@@ -9696,7 +9696,7 @@
         </is>
       </c>
       <c r="S137">
-        <v>-0.6563581280059488</v>
+        <v>-0.6563581280063013</v>
       </c>
     </row>
     <row r="138">
@@ -9750,7 +9750,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N138">
-        <v>89.05764683702921</v>
+        <v>89.057646837029</v>
       </c>
       <c r="O138">
         <v>96.53969112716689</v>
@@ -9818,7 +9818,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N139">
-        <v>89.05764683702921</v>
+        <v>89.057646837029</v>
       </c>
       <c r="O139">
         <v>96.53969112716689</v>
@@ -9886,7 +9886,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N140">
-        <v>89.05764683702921</v>
+        <v>89.057646837029</v>
       </c>
       <c r="O140">
         <v>96.53969112716689</v>
@@ -9900,7 +9900,7 @@
         </is>
       </c>
       <c r="S140">
-        <v>-2.609675776510767</v>
+        <v>-2.609675776510978</v>
       </c>
     </row>
     <row r="141">
@@ -9954,7 +9954,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N141">
-        <v>89.05764683702921</v>
+        <v>89.057646837029</v>
       </c>
       <c r="O141">
         <v>96.53969112716689</v>
@@ -10022,10 +10022,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N142">
-        <v>61.88484918229459</v>
+        <v>61.88484918229447</v>
       </c>
       <c r="O142">
-        <v>61.47727459441587</v>
+        <v>61.4772745944154</v>
       </c>
       <c r="P142">
         <v>54426</v>
@@ -10090,10 +10090,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N143">
-        <v>61.88484918229459</v>
+        <v>61.88484918229447</v>
       </c>
       <c r="O143">
-        <v>61.47727459441587</v>
+        <v>61.4772745944154</v>
       </c>
       <c r="P143">
         <v>54426</v>
@@ -10158,10 +10158,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N144">
-        <v>61.88484918229459</v>
+        <v>61.88484918229447</v>
       </c>
       <c r="O144">
-        <v>61.47727459441587</v>
+        <v>61.4772745944154</v>
       </c>
       <c r="P144">
         <v>54426</v>
@@ -10172,7 +10172,7 @@
         </is>
       </c>
       <c r="S144">
-        <v>-1.127829715025552</v>
+        <v>-1.127829715025674</v>
       </c>
     </row>
     <row r="145">
@@ -10226,10 +10226,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N145">
-        <v>61.88484918229459</v>
+        <v>61.88484918229447</v>
       </c>
       <c r="O145">
-        <v>61.47727459441587</v>
+        <v>61.4772745944154</v>
       </c>
       <c r="P145">
         <v>54426</v>
@@ -10240,7 +10240,7 @@
         </is>
       </c>
       <c r="S145">
-        <v>-1.535404302904275</v>
+        <v>-1.535404302904742</v>
       </c>
     </row>
     <row r="146">
@@ -10294,10 +10294,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N146">
-        <v>52.10416026488398</v>
+        <v>52.10416026488397</v>
       </c>
       <c r="O146">
-        <v>53.71180101699651</v>
+        <v>53.71180101699645</v>
       </c>
       <c r="P146">
         <v>54535</v>
@@ -10362,10 +10362,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N147">
-        <v>52.10416026488398</v>
+        <v>52.10416026488397</v>
       </c>
       <c r="O147">
-        <v>53.71180101699651</v>
+        <v>53.71180101699645</v>
       </c>
       <c r="P147">
         <v>54535</v>
@@ -10430,10 +10430,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N148">
-        <v>52.10416026488398</v>
+        <v>52.10416026488397</v>
       </c>
       <c r="O148">
-        <v>53.71180101699651</v>
+        <v>53.71180101699645</v>
       </c>
       <c r="P148">
         <v>54535</v>
@@ -10444,7 +10444,7 @@
         </is>
       </c>
       <c r="S148">
-        <v>-0.188219283370572</v>
+        <v>-0.1882192833705831</v>
       </c>
     </row>
     <row r="149">
@@ -10498,10 +10498,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N149">
-        <v>52.10416026488398</v>
+        <v>52.10416026488397</v>
       </c>
       <c r="O149">
-        <v>53.71180101699651</v>
+        <v>53.71180101699645</v>
       </c>
       <c r="P149">
         <v>54535</v>
@@ -10512,7 +10512,7 @@
         </is>
       </c>
       <c r="S149">
-        <v>1.419421468741955</v>
+        <v>1.419421468741899</v>
       </c>
     </row>
     <row r="150">
@@ -10566,10 +10566,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N150">
-        <v>88.10981089169675</v>
+        <v>88.10981089169665</v>
       </c>
       <c r="O150">
-        <v>92.81601489807957</v>
+        <v>92.81601489807952</v>
       </c>
       <c r="P150">
         <v>54281</v>
@@ -10634,10 +10634,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N151">
-        <v>88.10981089169675</v>
+        <v>88.10981089169665</v>
       </c>
       <c r="O151">
-        <v>92.81601489807957</v>
+        <v>92.81601489807952</v>
       </c>
       <c r="P151">
         <v>54281</v>
@@ -10702,10 +10702,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N152">
-        <v>88.10981089169675</v>
+        <v>88.10981089169665</v>
       </c>
       <c r="O152">
-        <v>92.81601489807957</v>
+        <v>92.81601489807952</v>
       </c>
       <c r="P152">
         <v>54281</v>
@@ -10716,7 +10716,7 @@
         </is>
       </c>
       <c r="S152">
-        <v>0.03641639628391147</v>
+        <v>0.03641639628380045</v>
       </c>
     </row>
     <row r="153">
@@ -10770,10 +10770,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N153">
-        <v>88.10981089169675</v>
+        <v>88.10981089169665</v>
       </c>
       <c r="O153">
-        <v>92.81601489807957</v>
+        <v>92.81601489807952</v>
       </c>
       <c r="P153">
         <v>54281</v>
@@ -10784,7 +10784,7 @@
         </is>
       </c>
       <c r="S153">
-        <v>4.742620402666731</v>
+        <v>4.742620402666664</v>
       </c>
     </row>
     <row r="154">
@@ -10838,10 +10838,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N154">
-        <v>90.59641787470699</v>
+        <v>90.59641787470704</v>
       </c>
       <c r="O154">
-        <v>86.45602653188774</v>
+        <v>86.4560265318876</v>
       </c>
       <c r="P154">
         <v>54534</v>
@@ -10906,10 +10906,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N155">
-        <v>90.59641787470699</v>
+        <v>90.59641787470704</v>
       </c>
       <c r="O155">
-        <v>86.45602653188774</v>
+        <v>86.4560265318876</v>
       </c>
       <c r="P155">
         <v>54534</v>
@@ -10974,10 +10974,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N156">
-        <v>90.59641787470699</v>
+        <v>90.59641787470704</v>
       </c>
       <c r="O156">
-        <v>86.45602653188774</v>
+        <v>86.4560265318876</v>
       </c>
       <c r="P156">
         <v>54534</v>
@@ -10988,7 +10988,7 @@
         </is>
       </c>
       <c r="S156">
-        <v>0.642575343198637</v>
+        <v>0.6425753431986925</v>
       </c>
     </row>
     <row r="157">
@@ -11042,10 +11042,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N157">
-        <v>90.59641787470699</v>
+        <v>90.59641787470704</v>
       </c>
       <c r="O157">
-        <v>86.45602653188774</v>
+        <v>86.4560265318876</v>
       </c>
       <c r="P157">
         <v>54534</v>
@@ -11056,7 +11056,7 @@
         </is>
       </c>
       <c r="S157">
-        <v>-3.497815999620613</v>
+        <v>-3.497815999620746</v>
       </c>
     </row>
     <row r="158">
@@ -11110,10 +11110,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N158">
-        <v>81.45050683818815</v>
+        <v>81.45050683818823</v>
       </c>
       <c r="O158">
-        <v>77.48841209095431</v>
+        <v>77.4884120909541</v>
       </c>
       <c r="P158">
         <v>39772</v>
@@ -11178,10 +11178,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N159">
-        <v>81.45050683818815</v>
+        <v>81.45050683818823</v>
       </c>
       <c r="O159">
-        <v>77.48841209095431</v>
+        <v>77.4884120909541</v>
       </c>
       <c r="P159">
         <v>39772</v>
@@ -11246,10 +11246,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N160">
-        <v>81.45050683818815</v>
+        <v>81.45050683818823</v>
       </c>
       <c r="O160">
-        <v>77.48841209095431</v>
+        <v>77.4884120909541</v>
       </c>
       <c r="P160">
         <v>39772</v>
@@ -11260,7 +11260,7 @@
         </is>
       </c>
       <c r="S160">
-        <v>-0.5301548422915969</v>
+        <v>-0.5301548422915192</v>
       </c>
     </row>
     <row r="161">
@@ -11314,10 +11314,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N161">
-        <v>81.45050683818815</v>
+        <v>81.45050683818823</v>
       </c>
       <c r="O161">
-        <v>77.48841209095431</v>
+        <v>77.4884120909541</v>
       </c>
       <c r="P161">
         <v>39772</v>
@@ -11328,7 +11328,7 @@
         </is>
       </c>
       <c r="S161">
-        <v>-4.492249589525443</v>
+        <v>-4.492249589525644</v>
       </c>
     </row>
     <row r="162">
@@ -11382,10 +11382,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N162">
-        <v>53.97907512970481</v>
+        <v>53.97907512970576</v>
       </c>
       <c r="O162">
-        <v>90.77842736117616</v>
+        <v>90.77842736117594</v>
       </c>
       <c r="P162">
         <v>42552</v>
@@ -11450,10 +11450,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N163">
-        <v>53.97907512970481</v>
+        <v>53.97907512970576</v>
       </c>
       <c r="O163">
-        <v>90.77842736117616</v>
+        <v>90.77842736117594</v>
       </c>
       <c r="P163">
         <v>42552</v>
@@ -11518,10 +11518,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N164">
-        <v>53.97907512970481</v>
+        <v>53.97907512970576</v>
       </c>
       <c r="O164">
-        <v>90.77842736117616</v>
+        <v>90.77842736117594</v>
       </c>
       <c r="P164">
         <v>42552</v>
@@ -11532,7 +11532,7 @@
         </is>
       </c>
       <c r="S164">
-        <v>0.0008416705640779121</v>
+        <v>0.0008416705650216016</v>
       </c>
     </row>
     <row r="165">
@@ -11586,10 +11586,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N165">
-        <v>53.97907512970481</v>
+        <v>53.97907512970576</v>
       </c>
       <c r="O165">
-        <v>90.77842736117616</v>
+        <v>90.77842736117594</v>
       </c>
       <c r="P165">
         <v>42552</v>
@@ -11600,7 +11600,7 @@
         </is>
       </c>
       <c r="S165">
-        <v>36.80019390203542</v>
+        <v>36.8001939020352</v>
       </c>
     </row>
     <row r="166">
@@ -20358,10 +20358,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N294">
-        <v>15.41815523864195</v>
+        <v>15.41815523864194</v>
       </c>
       <c r="O294">
-        <v>15.39358401703959</v>
+        <v>15.39358401703903</v>
       </c>
       <c r="P294">
         <v>61000</v>
@@ -20426,10 +20426,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N295">
-        <v>15.41815523864195</v>
+        <v>15.41815523864194</v>
       </c>
       <c r="O295">
-        <v>15.39358401703959</v>
+        <v>15.39358401703903</v>
       </c>
       <c r="P295">
         <v>61000</v>
@@ -20494,10 +20494,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N296">
-        <v>15.41815523864195</v>
+        <v>15.41815523864194</v>
       </c>
       <c r="O296">
-        <v>15.39358401703959</v>
+        <v>15.39358401703903</v>
       </c>
       <c r="P296">
         <v>61000</v>
@@ -20508,7 +20508,7 @@
         </is>
       </c>
       <c r="S296">
-        <v>-2.43406601478722</v>
+        <v>-2.434066014787231</v>
       </c>
     </row>
     <row r="297">
@@ -20562,10 +20562,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N297">
-        <v>15.41815523864195</v>
+        <v>15.41815523864194</v>
       </c>
       <c r="O297">
-        <v>15.39358401703959</v>
+        <v>15.39358401703903</v>
       </c>
       <c r="P297">
         <v>61000</v>
@@ -20576,7 +20576,7 @@
         </is>
       </c>
       <c r="S297">
-        <v>-2.458637236389585</v>
+        <v>-2.458637236390146</v>
       </c>
     </row>
     <row r="298">
@@ -20630,10 +20630,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N298">
-        <v>28.57244554318077</v>
+        <v>28.57244554318082</v>
       </c>
       <c r="O298">
-        <v>28.56364349950802</v>
+        <v>28.56364349950706</v>
       </c>
       <c r="P298">
         <v>61000</v>
@@ -20698,10 +20698,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N299">
-        <v>28.57244554318077</v>
+        <v>28.57244554318082</v>
       </c>
       <c r="O299">
-        <v>28.56364349950802</v>
+        <v>28.56364349950706</v>
       </c>
       <c r="P299">
         <v>61000</v>
@@ -20766,10 +20766,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N300">
-        <v>28.57244554318077</v>
+        <v>28.57244554318082</v>
       </c>
       <c r="O300">
-        <v>28.56364349950802</v>
+        <v>28.56364349950706</v>
       </c>
       <c r="P300">
         <v>61000</v>
@@ -20780,7 +20780,7 @@
         </is>
       </c>
       <c r="S300">
-        <v>-0.5880716505329397</v>
+        <v>-0.5880716505328953</v>
       </c>
     </row>
     <row r="301">
@@ -20834,10 +20834,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N301">
-        <v>28.57244554318077</v>
+        <v>28.57244554318082</v>
       </c>
       <c r="O301">
-        <v>28.56364349950802</v>
+        <v>28.56364349950706</v>
       </c>
       <c r="P301">
         <v>61000</v>
@@ -20848,7 +20848,7 @@
         </is>
       </c>
       <c r="S301">
-        <v>-0.5968736942056962</v>
+        <v>-0.5968736942066566</v>
       </c>
     </row>
     <row r="302">
@@ -20902,10 +20902,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N302">
-        <v>57.98657659676809</v>
+        <v>57.98657659676807</v>
       </c>
       <c r="O302">
-        <v>58.0108328128659</v>
+        <v>58.0108328128641</v>
       </c>
       <c r="P302">
         <v>60966</v>
@@ -20970,10 +20970,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N303">
-        <v>57.98657659676809</v>
+        <v>57.98657659676807</v>
       </c>
       <c r="O303">
-        <v>58.0108328128659</v>
+        <v>58.0108328128641</v>
       </c>
       <c r="P303">
         <v>60966</v>
@@ -21038,10 +21038,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N304">
-        <v>57.98657659676809</v>
+        <v>57.98657659676807</v>
       </c>
       <c r="O304">
-        <v>58.0108328128659</v>
+        <v>58.0108328128641</v>
       </c>
       <c r="P304">
         <v>60966</v>
@@ -21052,7 +21052,7 @@
         </is>
       </c>
       <c r="S304">
-        <v>0.9354526786854556</v>
+        <v>0.9354526786854334</v>
       </c>
     </row>
     <row r="305">
@@ -21106,10 +21106,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N305">
-        <v>57.98657659676809</v>
+        <v>57.98657659676807</v>
       </c>
       <c r="O305">
-        <v>58.0108328128659</v>
+        <v>58.0108328128641</v>
       </c>
       <c r="P305">
         <v>60966</v>
@@ -21120,7 +21120,7 @@
         </is>
       </c>
       <c r="S305">
-        <v>0.9597088947832622</v>
+        <v>0.9597088947814636</v>
       </c>
     </row>
     <row r="306">
@@ -21174,10 +21174,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N306">
-        <v>24.28635160555294</v>
+        <v>24.28635160555295</v>
       </c>
       <c r="O306">
-        <v>24.30807920702841</v>
+        <v>24.30807920702731</v>
       </c>
       <c r="P306">
         <v>54906</v>
@@ -21242,10 +21242,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N307">
-        <v>24.28635160555294</v>
+        <v>24.28635160555295</v>
       </c>
       <c r="O307">
-        <v>24.30807920702841</v>
+        <v>24.30807920702731</v>
       </c>
       <c r="P307">
         <v>54906</v>
@@ -21310,10 +21310,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N308">
-        <v>24.28635160555294</v>
+        <v>24.28635160555295</v>
       </c>
       <c r="O308">
-        <v>24.30807920702841</v>
+        <v>24.30807920702731</v>
       </c>
       <c r="P308">
         <v>54906</v>
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="S308">
-        <v>-0.3936985826528322</v>
+        <v>-0.3936985826528183</v>
       </c>
     </row>
     <row r="309">
@@ -21378,10 +21378,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N309">
-        <v>24.28635160555294</v>
+        <v>24.28635160555295</v>
       </c>
       <c r="O309">
-        <v>24.30807920702841</v>
+        <v>24.30807920702731</v>
       </c>
       <c r="P309">
         <v>54906</v>
@@ -21392,7 +21392,7 @@
         </is>
       </c>
       <c r="S309">
-        <v>-0.3719709811773608</v>
+        <v>-0.3719709811784599</v>
       </c>
     </row>
     <row r="310">
@@ -21446,10 +21446,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N310">
-        <v>86.70056156845875</v>
+        <v>86.70056156845874</v>
       </c>
       <c r="O310">
-        <v>96.82340183287785</v>
+        <v>96.82340183287779</v>
       </c>
       <c r="P310">
         <v>55751</v>
@@ -21514,10 +21514,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N311">
-        <v>86.70056156845875</v>
+        <v>86.70056156845874</v>
       </c>
       <c r="O311">
-        <v>96.82340183287785</v>
+        <v>96.82340183287779</v>
       </c>
       <c r="P311">
         <v>55751</v>
@@ -21582,10 +21582,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N312">
-        <v>86.70056156845875</v>
+        <v>86.70056156845874</v>
       </c>
       <c r="O312">
-        <v>96.82340183287785</v>
+        <v>96.82340183287779</v>
       </c>
       <c r="P312">
         <v>55751</v>
@@ -21596,7 +21596,7 @@
         </is>
       </c>
       <c r="S312">
-        <v>-3.50657111129371</v>
+        <v>-3.506571111293733</v>
       </c>
     </row>
     <row r="313">
@@ -21650,10 +21650,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N313">
-        <v>86.70056156845875</v>
+        <v>86.70056156845874</v>
       </c>
       <c r="O313">
-        <v>96.82340183287785</v>
+        <v>96.82340183287779</v>
       </c>
       <c r="P313">
         <v>55751</v>
@@ -21664,7 +21664,7 @@
         </is>
       </c>
       <c r="S313">
-        <v>6.616269153125376</v>
+        <v>6.61626915312532</v>
       </c>
     </row>
     <row r="314">
@@ -21718,10 +21718,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N314">
-        <v>59.81528043082665</v>
+        <v>59.81528043082663</v>
       </c>
       <c r="O314">
-        <v>60.34381502084475</v>
+        <v>60.34381502084364</v>
       </c>
       <c r="P314">
         <v>60920</v>
@@ -21786,10 +21786,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N315">
-        <v>59.81528043082665</v>
+        <v>59.81528043082663</v>
       </c>
       <c r="O315">
-        <v>60.34381502084475</v>
+        <v>60.34381502084364</v>
       </c>
       <c r="P315">
         <v>60920</v>
@@ -21854,10 +21854,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N316">
-        <v>59.81528043082665</v>
+        <v>59.81528043082663</v>
       </c>
       <c r="O316">
-        <v>60.34381502084475</v>
+        <v>60.34381502084364</v>
       </c>
       <c r="P316">
         <v>60920</v>
@@ -21868,7 +21868,7 @@
         </is>
       </c>
       <c r="S316">
-        <v>-1.367740548997121</v>
+        <v>-1.367740548997154</v>
       </c>
     </row>
     <row r="317">
@@ -21922,10 +21922,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N317">
-        <v>59.81528043082665</v>
+        <v>59.81528043082663</v>
       </c>
       <c r="O317">
-        <v>60.34381502084475</v>
+        <v>60.34381502084364</v>
       </c>
       <c r="P317">
         <v>60920</v>
@@ -21936,7 +21936,7 @@
         </is>
       </c>
       <c r="S317">
-        <v>-0.8392059589790279</v>
+        <v>-0.8392059589801382</v>
       </c>
     </row>
     <row r="318">
@@ -21990,10 +21990,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N318">
-        <v>51.87442533665195</v>
+        <v>51.87442533665201</v>
       </c>
       <c r="O318">
-        <v>55.19320995384758</v>
+        <v>55.19320995384727</v>
       </c>
       <c r="P318">
         <v>61000</v>
@@ -22058,10 +22058,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N319">
-        <v>51.87442533665195</v>
+        <v>51.87442533665201</v>
       </c>
       <c r="O319">
-        <v>55.19320995384758</v>
+        <v>55.19320995384727</v>
       </c>
       <c r="P319">
         <v>61000</v>
@@ -22126,10 +22126,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N320">
-        <v>51.87442533665195</v>
+        <v>51.87442533665201</v>
       </c>
       <c r="O320">
-        <v>55.19320995384758</v>
+        <v>55.19320995384727</v>
       </c>
       <c r="P320">
         <v>61000</v>
@@ -22140,7 +22140,7 @@
         </is>
       </c>
       <c r="S320">
-        <v>-0.2309273630907271</v>
+        <v>-0.2309273630906716</v>
       </c>
     </row>
     <row r="321">
@@ -22194,10 +22194,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N321">
-        <v>51.87442533665195</v>
+        <v>51.87442533665201</v>
       </c>
       <c r="O321">
-        <v>55.19320995384758</v>
+        <v>55.19320995384727</v>
       </c>
       <c r="P321">
         <v>61000</v>
@@ -22208,7 +22208,7 @@
         </is>
       </c>
       <c r="S321">
-        <v>3.087857254104898</v>
+        <v>3.087857254104587</v>
       </c>
     </row>
     <row r="322">
@@ -22262,10 +22262,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N322">
-        <v>88.60775405607038</v>
+        <v>88.60775405607029</v>
       </c>
       <c r="O322">
-        <v>92.81092514217534</v>
+        <v>92.81092514217536</v>
       </c>
       <c r="P322">
         <v>60928</v>
@@ -22330,10 +22330,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N323">
-        <v>88.60775405607038</v>
+        <v>88.60775405607029</v>
       </c>
       <c r="O323">
-        <v>92.81092514217534</v>
+        <v>92.81092514217536</v>
       </c>
       <c r="P323">
         <v>60928</v>
@@ -22398,10 +22398,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N324">
-        <v>88.60775405607038</v>
+        <v>88.60775405607029</v>
       </c>
       <c r="O324">
-        <v>92.81092514217534</v>
+        <v>92.81092514217536</v>
       </c>
       <c r="P324">
         <v>60928</v>
@@ -22412,7 +22412,7 @@
         </is>
       </c>
       <c r="S324">
-        <v>-0.3433119337773349</v>
+        <v>-0.3433119337774126</v>
       </c>
     </row>
     <row r="325">
@@ -22466,10 +22466,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N325">
-        <v>88.60775405607038</v>
+        <v>88.60775405607029</v>
       </c>
       <c r="O325">
-        <v>92.81092514217534</v>
+        <v>92.81092514217536</v>
       </c>
       <c r="P325">
         <v>60928</v>
@@ -22480,7 +22480,7 @@
         </is>
       </c>
       <c r="S325">
-        <v>3.859859152327627</v>
+        <v>3.859859152327649</v>
       </c>
     </row>
     <row r="326">
@@ -22534,10 +22534,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N326">
-        <v>92.49798818801629</v>
+        <v>92.49798818801627</v>
       </c>
       <c r="O326">
-        <v>89.42387194359381</v>
+        <v>89.42387194359372</v>
       </c>
       <c r="P326">
         <v>61000</v>
@@ -22602,10 +22602,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N327">
-        <v>92.49798818801629</v>
+        <v>92.49798818801627</v>
       </c>
       <c r="O327">
-        <v>89.42387194359381</v>
+        <v>89.42387194359372</v>
       </c>
       <c r="P327">
         <v>61000</v>
@@ -22670,10 +22670,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N328">
-        <v>92.49798818801629</v>
+        <v>92.49798818801627</v>
       </c>
       <c r="O328">
-        <v>89.42387194359381</v>
+        <v>89.42387194359372</v>
       </c>
       <c r="P328">
         <v>61000</v>
@@ -22684,7 +22684,7 @@
         </is>
       </c>
       <c r="S328">
-        <v>0.9126431762666587</v>
+        <v>0.9126431762666365</v>
       </c>
     </row>
     <row r="329">
@@ -22738,10 +22738,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N329">
-        <v>92.49798818801629</v>
+        <v>92.49798818801627</v>
       </c>
       <c r="O329">
-        <v>89.42387194359381</v>
+        <v>89.42387194359372</v>
       </c>
       <c r="P329">
         <v>61000</v>
@@ -22752,7 +22752,7 @@
         </is>
       </c>
       <c r="S329">
-        <v>-2.161473068155828</v>
+        <v>-2.161473068155906</v>
       </c>
     </row>
     <row r="330">
@@ -22806,10 +22806,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N330">
-        <v>56.80719956100195</v>
+        <v>56.80719956100185</v>
       </c>
       <c r="O330">
-        <v>53.77092581252965</v>
+        <v>53.77092581252928</v>
       </c>
       <c r="P330">
         <v>45790</v>
@@ -22874,10 +22874,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N331">
-        <v>56.80719956100195</v>
+        <v>56.80719956100185</v>
       </c>
       <c r="O331">
-        <v>53.77092581252965</v>
+        <v>53.77092581252928</v>
       </c>
       <c r="P331">
         <v>45790</v>
@@ -22942,10 +22942,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N332">
-        <v>56.80719956100195</v>
+        <v>56.80719956100185</v>
       </c>
       <c r="O332">
-        <v>53.77092581252965</v>
+        <v>53.77092581252928</v>
       </c>
       <c r="P332">
         <v>45790</v>
@@ -22956,7 +22956,7 @@
         </is>
       </c>
       <c r="S332">
-        <v>0.3061338125185942</v>
+        <v>0.3061338125184943</v>
       </c>
     </row>
     <row r="333">
@@ -23010,10 +23010,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N333">
-        <v>56.80719956100195</v>
+        <v>56.80719956100185</v>
       </c>
       <c r="O333">
-        <v>53.77092581252965</v>
+        <v>53.77092581252928</v>
       </c>
       <c r="P333">
         <v>45790</v>
@@ -23024,7 +23024,7 @@
         </is>
       </c>
       <c r="S333">
-        <v>-2.730139935953713</v>
+        <v>-2.730139935954079</v>
       </c>
     </row>
     <row r="334">
@@ -23078,10 +23078,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N334">
-        <v>62.07721827600816</v>
+        <v>62.0772182760082</v>
       </c>
       <c r="O334">
-        <v>94.75407612852125</v>
+        <v>94.75407612852116</v>
       </c>
       <c r="P334">
         <v>48462</v>
@@ -23146,10 +23146,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N335">
-        <v>62.07721827600816</v>
+        <v>62.0772182760082</v>
       </c>
       <c r="O335">
-        <v>94.75407612852125</v>
+        <v>94.75407612852116</v>
       </c>
       <c r="P335">
         <v>48462</v>
@@ -23214,10 +23214,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N336">
-        <v>62.07721827600816</v>
+        <v>62.0772182760082</v>
       </c>
       <c r="O336">
-        <v>94.75407612852125</v>
+        <v>94.75407612852116</v>
       </c>
       <c r="P336">
         <v>48462</v>
@@ -23228,7 +23228,7 @@
         </is>
       </c>
       <c r="S336">
-        <v>0.244385146496795</v>
+        <v>0.2443851464968394</v>
       </c>
     </row>
     <row r="337">
@@ -23282,10 +23282,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N337">
-        <v>62.07721827600816</v>
+        <v>62.0772182760082</v>
       </c>
       <c r="O337">
-        <v>94.75407612852125</v>
+        <v>94.75407612852116</v>
       </c>
       <c r="P337">
         <v>48462</v>
@@ -23296,7 +23296,7 @@
         </is>
       </c>
       <c r="S337">
-        <v>32.92124299900988</v>
+        <v>32.92124299900981</v>
       </c>
     </row>
     <row r="338">
@@ -23350,10 +23350,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N338">
-        <v>15.79903111329061</v>
+        <v>15.79903111329064</v>
       </c>
       <c r="O338">
-        <v>15.79902656857579</v>
+        <v>15.7990265685755</v>
       </c>
       <c r="P338">
         <v>60000</v>
@@ -23418,10 +23418,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N339">
-        <v>15.79903111329061</v>
+        <v>15.79903111329064</v>
       </c>
       <c r="O339">
-        <v>15.79902656857579</v>
+        <v>15.7990265685755</v>
       </c>
       <c r="P339">
         <v>60000</v>
@@ -23486,10 +23486,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N340">
-        <v>15.79903111329061</v>
+        <v>15.79903111329064</v>
       </c>
       <c r="O340">
-        <v>15.79902656857579</v>
+        <v>15.7990265685755</v>
       </c>
       <c r="P340">
         <v>60000</v>
@@ -23500,7 +23500,7 @@
         </is>
       </c>
       <c r="S340">
-        <v>-2.973342908037155</v>
+        <v>-2.97334290803713</v>
       </c>
     </row>
     <row r="341">
@@ -23554,10 +23554,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N341">
-        <v>15.79903111329061</v>
+        <v>15.79903111329064</v>
       </c>
       <c r="O341">
-        <v>15.79902656857579</v>
+        <v>15.7990265685755</v>
       </c>
       <c r="P341">
         <v>60000</v>
@@ -23568,7 +23568,7 @@
         </is>
       </c>
       <c r="S341">
-        <v>-2.973347452751979</v>
+        <v>-2.97334745275227</v>
       </c>
     </row>
     <row r="342">
@@ -23622,10 +23622,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N342">
-        <v>29.1234330717829</v>
+        <v>29.12343307178292</v>
       </c>
       <c r="O342">
-        <v>29.12342358088578</v>
+        <v>29.12342358088552</v>
       </c>
       <c r="P342">
         <v>60000</v>
@@ -23690,10 +23690,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N343">
-        <v>29.1234330717829</v>
+        <v>29.12343307178292</v>
       </c>
       <c r="O343">
-        <v>29.12342358088578</v>
+        <v>29.12342358088552</v>
       </c>
       <c r="P343">
         <v>60000</v>
@@ -23758,10 +23758,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N344">
-        <v>29.1234330717829</v>
+        <v>29.12343307178292</v>
       </c>
       <c r="O344">
-        <v>29.12342358088578</v>
+        <v>29.12342358088552</v>
       </c>
       <c r="P344">
         <v>60000</v>
@@ -23772,7 +23772,7 @@
         </is>
       </c>
       <c r="S344">
-        <v>-0.3447521545214938</v>
+        <v>-0.3447521545214771</v>
       </c>
     </row>
     <row r="345">
@@ -23826,10 +23826,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N345">
-        <v>29.1234330717829</v>
+        <v>29.12343307178292</v>
       </c>
       <c r="O345">
-        <v>29.12342358088578</v>
+        <v>29.12342358088552</v>
       </c>
       <c r="P345">
         <v>60000</v>
@@ -23840,7 +23840,7 @@
         </is>
       </c>
       <c r="S345">
-        <v>-0.3447616454186175</v>
+        <v>-0.3447616454188729</v>
       </c>
     </row>
     <row r="346">
@@ -23894,10 +23894,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N346">
-        <v>60.91535036081953</v>
+        <v>60.91535036081957</v>
       </c>
       <c r="O346">
-        <v>60.91538488022671</v>
+        <v>60.91538488022654</v>
       </c>
       <c r="P346">
         <v>59952</v>
@@ -23962,10 +23962,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N347">
-        <v>60.91535036081953</v>
+        <v>60.91535036081957</v>
       </c>
       <c r="O347">
-        <v>60.91538488022671</v>
+        <v>60.91538488022654</v>
       </c>
       <c r="P347">
         <v>59952</v>
@@ -24030,10 +24030,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N348">
-        <v>60.91535036081953</v>
+        <v>60.91535036081957</v>
       </c>
       <c r="O348">
-        <v>60.91538488022671</v>
+        <v>60.91538488022654</v>
       </c>
       <c r="P348">
         <v>59952</v>
@@ -24044,7 +24044,7 @@
         </is>
       </c>
       <c r="S348">
-        <v>2.019584098563187</v>
+        <v>2.019584098563221</v>
       </c>
     </row>
     <row r="349">
@@ -24098,10 +24098,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N349">
-        <v>60.91535036081953</v>
+        <v>60.91535036081957</v>
       </c>
       <c r="O349">
-        <v>60.91538488022671</v>
+        <v>60.91538488022654</v>
       </c>
       <c r="P349">
         <v>59952</v>
@@ -24112,7 +24112,7 @@
         </is>
       </c>
       <c r="S349">
-        <v>2.019618617970365</v>
+        <v>2.019618617970198</v>
       </c>
     </row>
     <row r="350">
@@ -24166,10 +24166,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N350">
-        <v>23.77362779864108</v>
+        <v>23.77362779864106</v>
       </c>
       <c r="O350">
-        <v>23.77362873790611</v>
+        <v>23.77362873790585</v>
       </c>
       <c r="P350">
         <v>55143</v>
@@ -24234,10 +24234,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N351">
-        <v>23.77362779864108</v>
+        <v>23.77362779864106</v>
       </c>
       <c r="O351">
-        <v>23.77362873790611</v>
+        <v>23.77362873790585</v>
       </c>
       <c r="P351">
         <v>55143</v>
@@ -24302,10 +24302,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N352">
-        <v>23.77362779864108</v>
+        <v>23.77362779864106</v>
       </c>
       <c r="O352">
-        <v>23.77362873790611</v>
+        <v>23.77362873790585</v>
       </c>
       <c r="P352">
         <v>55143</v>
@@ -24316,7 +24316,7 @@
         </is>
       </c>
       <c r="S352">
-        <v>-0.3448162932823545</v>
+        <v>-0.3448162932823767</v>
       </c>
     </row>
     <row r="353">
@@ -24370,10 +24370,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N353">
-        <v>23.77362779864108</v>
+        <v>23.77362779864106</v>
       </c>
       <c r="O353">
-        <v>23.77362873790611</v>
+        <v>23.77362873790585</v>
       </c>
       <c r="P353">
         <v>55143</v>
@@ -24384,7 +24384,7 @@
         </is>
       </c>
       <c r="S353">
-        <v>-0.3448153540173249</v>
+        <v>-0.3448153540175858</v>
       </c>
     </row>
     <row r="354">
@@ -24438,10 +24438,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N354">
-        <v>86.61759427225223</v>
+        <v>86.61759427225226</v>
       </c>
       <c r="O354">
-        <v>90.83563195911087</v>
+        <v>90.83563195911086</v>
       </c>
       <c r="P354">
         <v>57277</v>
@@ -24506,10 +24506,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N355">
-        <v>86.61759427225223</v>
+        <v>86.61759427225226</v>
       </c>
       <c r="O355">
-        <v>90.83563195911087</v>
+        <v>90.83563195911086</v>
       </c>
       <c r="P355">
         <v>57277</v>
@@ -24574,10 +24574,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N356">
-        <v>86.61759427225223</v>
+        <v>86.61759427225226</v>
       </c>
       <c r="O356">
-        <v>90.83563195911087</v>
+        <v>90.83563195911086</v>
       </c>
       <c r="P356">
         <v>57277</v>
@@ -24588,7 +24588,7 @@
         </is>
       </c>
       <c r="S356">
-        <v>-2.943012765955744</v>
+        <v>-2.943012765955721</v>
       </c>
     </row>
     <row r="357">
@@ -24642,10 +24642,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N357">
-        <v>86.61759427225223</v>
+        <v>86.61759427225226</v>
       </c>
       <c r="O357">
-        <v>90.83563195911087</v>
+        <v>90.83563195911086</v>
       </c>
       <c r="P357">
         <v>57277</v>
@@ -24656,7 +24656,7 @@
         </is>
       </c>
       <c r="S357">
-        <v>1.27502492090289</v>
+        <v>1.275024920902879</v>
       </c>
     </row>
     <row r="358">
@@ -24710,10 +24710,10 @@
         <v>60.99375995409059</v>
       </c>
       <c r="N358">
-        <v>61.01690685229683</v>
+        <v>61.01690685229691</v>
       </c>
       <c r="O358">
-        <v>60.71393243350647</v>
+        <v>60.71393243350624</v>
       </c>
       <c r="P358">
         <v>59908</v>
@@ -24778,10 +24778,10 @@
         <v>60.99375995409059</v>
       </c>
       <c r="N359">
-        <v>61.01690685229683</v>
+        <v>61.01690685229691</v>
       </c>
       <c r="O359">
-        <v>60.71393243350647</v>
+        <v>60.71393243350624</v>
       </c>
       <c r="P359">
         <v>59908</v>
@@ -24846,10 +24846,10 @@
         <v>60.99375995409059</v>
       </c>
       <c r="N360">
-        <v>61.01690685229683</v>
+        <v>61.01690685229691</v>
       </c>
       <c r="O360">
-        <v>60.71393243350647</v>
+        <v>60.71393243350624</v>
       </c>
       <c r="P360">
         <v>59908</v>
@@ -24860,7 +24860,7 @@
         </is>
       </c>
       <c r="S360">
-        <v>-1.764850130809714</v>
+        <v>-1.764850130809625</v>
       </c>
     </row>
     <row r="361">
@@ -24914,10 +24914,10 @@
         <v>60.99375995409059</v>
       </c>
       <c r="N361">
-        <v>61.01690685229683</v>
+        <v>61.01690685229691</v>
       </c>
       <c r="O361">
-        <v>60.71393243350647</v>
+        <v>60.71393243350624</v>
       </c>
       <c r="P361">
         <v>59908</v>
@@ -24928,7 +24928,7 @@
         </is>
       </c>
       <c r="S361">
-        <v>-2.067824549600072</v>
+        <v>-2.067824549600306</v>
       </c>
     </row>
     <row r="362">
@@ -24982,10 +24982,10 @@
         <v>52.20547113980047</v>
       </c>
       <c r="N362">
-        <v>51.58328699371187</v>
+        <v>51.58328699371179</v>
       </c>
       <c r="O362">
-        <v>51.69280674241718</v>
+        <v>51.69280674241715</v>
       </c>
       <c r="P362">
         <v>59563</v>
@@ -25050,10 +25050,10 @@
         <v>52.20547113980047</v>
       </c>
       <c r="N363">
-        <v>51.58328699371187</v>
+        <v>51.58328699371179</v>
       </c>
       <c r="O363">
-        <v>51.69280674241718</v>
+        <v>51.69280674241715</v>
       </c>
       <c r="P363">
         <v>59563</v>
@@ -25118,10 +25118,10 @@
         <v>52.20547113980047</v>
       </c>
       <c r="N364">
-        <v>51.58328699371187</v>
+        <v>51.58328699371179</v>
       </c>
       <c r="O364">
-        <v>51.69280674241718</v>
+        <v>51.69280674241715</v>
       </c>
       <c r="P364">
         <v>59563</v>
@@ -25132,7 +25132,7 @@
         </is>
       </c>
       <c r="S364">
-        <v>-0.5048808339750743</v>
+        <v>-0.504880833975152</v>
       </c>
     </row>
     <row r="365">
@@ -25186,10 +25186,10 @@
         <v>52.20547113980047</v>
       </c>
       <c r="N365">
-        <v>51.58328699371187</v>
+        <v>51.58328699371179</v>
       </c>
       <c r="O365">
-        <v>51.69280674241718</v>
+        <v>51.69280674241715</v>
       </c>
       <c r="P365">
         <v>59563</v>
@@ -25200,7 +25200,7 @@
         </is>
       </c>
       <c r="S365">
-        <v>-0.395361085269752</v>
+        <v>-0.3953610852697853</v>
       </c>
     </row>
     <row r="366">
@@ -25254,10 +25254,10 @@
         <v>94.03545595788032</v>
       </c>
       <c r="N366">
-        <v>89.30448482920681</v>
+        <v>89.30448482920688</v>
       </c>
       <c r="O366">
-        <v>92.04660792596593</v>
+        <v>92.04660792596596</v>
       </c>
       <c r="P366">
         <v>59952</v>
@@ -25322,10 +25322,10 @@
         <v>94.03545595788032</v>
       </c>
       <c r="N367">
-        <v>89.30448482920681</v>
+        <v>89.30448482920688</v>
       </c>
       <c r="O367">
-        <v>92.04660792596593</v>
+        <v>92.04660792596596</v>
       </c>
       <c r="P367">
         <v>59952</v>
@@ -25390,10 +25390,10 @@
         <v>94.03545595788032</v>
       </c>
       <c r="N368">
-        <v>89.30448482920681</v>
+        <v>89.30448482920688</v>
       </c>
       <c r="O368">
-        <v>92.04660792596593</v>
+        <v>92.04660792596596</v>
       </c>
       <c r="P368">
         <v>59952</v>
@@ -25404,7 +25404,7 @@
         </is>
       </c>
       <c r="S368">
-        <v>-0.4456318395810954</v>
+        <v>-0.4456318395810288</v>
       </c>
     </row>
     <row r="369">
@@ -25458,10 +25458,10 @@
         <v>94.03545595788032</v>
       </c>
       <c r="N369">
-        <v>89.30448482920681</v>
+        <v>89.30448482920688</v>
       </c>
       <c r="O369">
-        <v>92.04660792596593</v>
+        <v>92.04660792596596</v>
       </c>
       <c r="P369">
         <v>59952</v>
@@ -25472,7 +25472,7 @@
         </is>
       </c>
       <c r="S369">
-        <v>2.296491257178013</v>
+        <v>2.296491257178046</v>
       </c>
     </row>
     <row r="370">
@@ -25526,10 +25526,10 @@
         <v>90.81416282496983</v>
       </c>
       <c r="N370">
-        <v>92.88968438627357</v>
+        <v>92.88968438627364</v>
       </c>
       <c r="O370">
-        <v>89.61508203055229</v>
+        <v>89.6150820305524</v>
       </c>
       <c r="P370">
         <v>60000</v>
@@ -25594,10 +25594,10 @@
         <v>90.81416282496983</v>
       </c>
       <c r="N371">
-        <v>92.88968438627357</v>
+        <v>92.88968438627364</v>
       </c>
       <c r="O371">
-        <v>89.61508203055229</v>
+        <v>89.6150820305524</v>
       </c>
       <c r="P371">
         <v>60000</v>
@@ -25662,10 +25662,10 @@
         <v>90.81416282496983</v>
       </c>
       <c r="N372">
-        <v>92.88968438627357</v>
+        <v>92.88968438627364</v>
       </c>
       <c r="O372">
-        <v>89.61508203055229</v>
+        <v>89.6150820305524</v>
       </c>
       <c r="P372">
         <v>60000</v>
@@ -25676,7 +25676,7 @@
         </is>
       </c>
       <c r="S372">
-        <v>0.878090403613152</v>
+        <v>0.8780904036132187</v>
       </c>
     </row>
     <row r="373">
@@ -25730,10 +25730,10 @@
         <v>90.81416282496983</v>
       </c>
       <c r="N373">
-        <v>92.88968438627357</v>
+        <v>92.88968438627364</v>
       </c>
       <c r="O373">
-        <v>89.61508203055229</v>
+        <v>89.6150820305524</v>
       </c>
       <c r="P373">
         <v>60000</v>
@@ -25744,7 +25744,7 @@
         </is>
       </c>
       <c r="S373">
-        <v>-2.396511952108138</v>
+        <v>-2.396511952108016</v>
       </c>
     </row>
     <row r="374">
@@ -25798,10 +25798,10 @@
         <v>66.36932631856995</v>
       </c>
       <c r="N374">
-        <v>68.08470983266751</v>
+        <v>68.0847098326675</v>
       </c>
       <c r="O374">
-        <v>65.01271796233431</v>
+        <v>65.01271796233409</v>
       </c>
       <c r="P374">
         <v>40876</v>
@@ -25866,10 +25866,10 @@
         <v>66.36932631856995</v>
       </c>
       <c r="N375">
-        <v>68.08470983266751</v>
+        <v>68.0847098326675</v>
       </c>
       <c r="O375">
-        <v>65.01271796233431</v>
+        <v>65.01271796233409</v>
       </c>
       <c r="P375">
         <v>40876</v>
@@ -25934,10 +25934,10 @@
         <v>66.36932631856995</v>
       </c>
       <c r="N376">
-        <v>68.08470983266751</v>
+        <v>68.0847098326675</v>
       </c>
       <c r="O376">
-        <v>65.01271796233431</v>
+        <v>65.01271796233409</v>
       </c>
       <c r="P376">
         <v>40876</v>
@@ -25948,7 +25948,7 @@
         </is>
       </c>
       <c r="S376">
-        <v>0.6967417540917009</v>
+        <v>0.6967417540916898</v>
       </c>
     </row>
     <row r="377">
@@ -26002,10 +26002,10 @@
         <v>66.36932631856995</v>
       </c>
       <c r="N377">
-        <v>68.08470983266751</v>
+        <v>68.0847098326675</v>
       </c>
       <c r="O377">
-        <v>65.01271796233431</v>
+        <v>65.01271796233409</v>
       </c>
       <c r="P377">
         <v>40876</v>
@@ -26016,7 +26016,7 @@
         </is>
       </c>
       <c r="S377">
-        <v>-2.375250116241501</v>
+        <v>-2.375250116241723</v>
       </c>
     </row>
     <row r="378">
@@ -26070,10 +26070,10 @@
         <v>7.294531710394677</v>
       </c>
       <c r="N378">
-        <v>57.18663105574594</v>
+        <v>57.18663105574592</v>
       </c>
       <c r="O378">
-        <v>14.7348353518708</v>
+        <v>14.73483535187088</v>
       </c>
       <c r="P378">
         <v>47791</v>
@@ -26138,10 +26138,10 @@
         <v>7.294531710394677</v>
       </c>
       <c r="N379">
-        <v>57.18663105574594</v>
+        <v>57.18663105574592</v>
       </c>
       <c r="O379">
-        <v>14.7348353518708</v>
+        <v>14.73483535187088</v>
       </c>
       <c r="P379">
         <v>47791</v>
@@ -26206,10 +26206,10 @@
         <v>7.294531710394677</v>
       </c>
       <c r="N380">
-        <v>57.18663105574594</v>
+        <v>57.18663105574592</v>
       </c>
       <c r="O380">
-        <v>14.7348353518708</v>
+        <v>14.73483535187088</v>
       </c>
       <c r="P380">
         <v>47791</v>
@@ -26220,7 +26220,7 @@
         </is>
       </c>
       <c r="S380">
-        <v>-9.099751255847721E-05</v>
+        <v>-9.099751258068167E-05</v>
       </c>
     </row>
     <row r="381">
@@ -26274,10 +26274,10 @@
         <v>7.294531710394677</v>
       </c>
       <c r="N381">
-        <v>57.18663105574594</v>
+        <v>57.18663105574592</v>
       </c>
       <c r="O381">
-        <v>14.7348353518708</v>
+        <v>14.73483535187088</v>
       </c>
       <c r="P381">
         <v>47791</v>
@@ -26288,7 +26288,7 @@
         </is>
       </c>
       <c r="S381">
-        <v>-42.4518867013877</v>
+        <v>-42.45188670138761</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix weighted CPS benchmarks; update codebook and figures
</commit_message>
<xml_diff>
--- a/tables_and_figures/input_tables/national_errors.xlsx
+++ b/tables_and_figures/input_tables/national_errors.xlsx
@@ -5670,10 +5670,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N78">
-        <v>21.68983558756392</v>
+        <v>21.68983558756369</v>
       </c>
       <c r="O78">
-        <v>21.68983558756405</v>
+        <v>21.68983558756393</v>
       </c>
       <c r="P78">
         <v>55400</v>
@@ -5738,10 +5738,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N79">
-        <v>21.68983558756392</v>
+        <v>21.68983558756369</v>
       </c>
       <c r="O79">
-        <v>21.68983558756405</v>
+        <v>21.68983558756393</v>
       </c>
       <c r="P79">
         <v>55400</v>
@@ -5806,10 +5806,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N80">
-        <v>21.68983558756392</v>
+        <v>21.68983558756369</v>
       </c>
       <c r="O80">
-        <v>21.68983558756405</v>
+        <v>21.68983558756393</v>
       </c>
       <c r="P80">
         <v>55400</v>
@@ -5820,7 +5820,7 @@
         </is>
       </c>
       <c r="S80">
-        <v>1.936748087924742</v>
+        <v>1.936748087924511</v>
       </c>
     </row>
     <row r="81">
@@ -5874,10 +5874,10 @@
         <v>19.71418188895098</v>
       </c>
       <c r="N81">
-        <v>21.68983558756392</v>
+        <v>21.68983558756369</v>
       </c>
       <c r="O81">
-        <v>21.68983558756405</v>
+        <v>21.68983558756393</v>
       </c>
       <c r="P81">
         <v>55400</v>
@@ -5888,7 +5888,7 @@
         </is>
       </c>
       <c r="S81">
-        <v>1.936748087924864</v>
+        <v>1.936748087924747</v>
       </c>
     </row>
     <row r="82">
@@ -5942,10 +5942,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N82">
-        <v>32.13108402346401</v>
+        <v>32.131084023464</v>
       </c>
       <c r="O82">
-        <v>32.13108402346418</v>
+        <v>32.13108402346392</v>
       </c>
       <c r="P82">
         <v>55400</v>
@@ -6010,10 +6010,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N83">
-        <v>32.13108402346401</v>
+        <v>32.131084023464</v>
       </c>
       <c r="O83">
-        <v>32.13108402346418</v>
+        <v>32.13108402346392</v>
       </c>
       <c r="P83">
         <v>55400</v>
@@ -6078,10 +6078,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N84">
-        <v>32.13108402346401</v>
+        <v>32.131084023464</v>
       </c>
       <c r="O84">
-        <v>32.13108402346418</v>
+        <v>32.13108402346392</v>
       </c>
       <c r="P84">
         <v>55400</v>
@@ -6092,7 +6092,7 @@
         </is>
       </c>
       <c r="S84">
-        <v>0.4445337920600756</v>
+        <v>0.44453379206007</v>
       </c>
     </row>
     <row r="85">
@@ -6146,10 +6146,10 @@
         <v>34.574542787282</v>
       </c>
       <c r="N85">
-        <v>32.13108402346401</v>
+        <v>32.131084023464</v>
       </c>
       <c r="O85">
-        <v>32.13108402346418</v>
+        <v>32.13108402346392</v>
       </c>
       <c r="P85">
         <v>55400</v>
@@ -6160,7 +6160,7 @@
         </is>
       </c>
       <c r="S85">
-        <v>0.4445337920602477</v>
+        <v>0.4445337920599868</v>
       </c>
     </row>
     <row r="86">
@@ -6214,10 +6214,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N86">
-        <v>60.64538348494989</v>
+        <v>60.64538348495072</v>
       </c>
       <c r="O86">
-        <v>60.64538348495076</v>
+        <v>60.64538348495044</v>
       </c>
       <c r="P86">
         <v>55400</v>
@@ -6282,10 +6282,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N87">
-        <v>60.64538348494989</v>
+        <v>60.64538348495072</v>
       </c>
       <c r="O87">
-        <v>60.64538348495076</v>
+        <v>60.64538348495044</v>
       </c>
       <c r="P87">
         <v>55400</v>
@@ -6350,10 +6350,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N88">
-        <v>60.64538348494989</v>
+        <v>60.64538348495072</v>
       </c>
       <c r="O88">
-        <v>60.64538348495076</v>
+        <v>60.64538348495044</v>
       </c>
       <c r="P88">
         <v>55400</v>
@@ -6364,7 +6364,7 @@
         </is>
       </c>
       <c r="S88">
-        <v>-0.2387361085909201</v>
+        <v>-0.2387361085900874</v>
       </c>
     </row>
     <row r="89">
@@ -6418,10 +6418,10 @@
         <v>49.75314441747606</v>
       </c>
       <c r="N89">
-        <v>60.64538348494989</v>
+        <v>60.64538348495072</v>
       </c>
       <c r="O89">
-        <v>60.64538348495076</v>
+        <v>60.64538348495044</v>
       </c>
       <c r="P89">
         <v>55400</v>
@@ -6432,7 +6432,7 @@
         </is>
       </c>
       <c r="S89">
-        <v>-0.238736108590043</v>
+        <v>-0.238736108590365</v>
       </c>
     </row>
     <row r="90">
@@ -6486,10 +6486,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N90">
-        <v>23.19167199619754</v>
+        <v>23.19167199619718</v>
       </c>
       <c r="O90">
-        <v>23.19287782028184</v>
+        <v>23.19287782028157</v>
       </c>
       <c r="P90">
         <v>48612</v>
@@ -6554,10 +6554,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N91">
-        <v>23.19167199619754</v>
+        <v>23.19167199619718</v>
       </c>
       <c r="O91">
-        <v>23.19287782028184</v>
+        <v>23.19287782028157</v>
       </c>
       <c r="P91">
         <v>48612</v>
@@ -6622,10 +6622,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N92">
-        <v>23.19167199619754</v>
+        <v>23.19167199619718</v>
       </c>
       <c r="O92">
-        <v>23.19287782028184</v>
+        <v>23.19287782028157</v>
       </c>
       <c r="P92">
         <v>48612</v>
@@ -6636,7 +6636,7 @@
         </is>
       </c>
       <c r="S92">
-        <v>-0.2830345174885757</v>
+        <v>-0.2830345174889337</v>
       </c>
     </row>
     <row r="93">
@@ -6690,10 +6690,10 @@
         <v>22.91056164538115</v>
       </c>
       <c r="N93">
-        <v>23.19167199619754</v>
+        <v>23.19167199619718</v>
       </c>
       <c r="O93">
-        <v>23.19287782028184</v>
+        <v>23.19287782028157</v>
       </c>
       <c r="P93">
         <v>48612</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="S93">
-        <v>-0.2818286934042763</v>
+        <v>-0.2818286934045483</v>
       </c>
     </row>
     <row r="94">
@@ -6758,10 +6758,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N94">
-        <v>90.07772910426883</v>
+        <v>90.07772910426878</v>
       </c>
       <c r="O94">
-        <v>95.56945283348823</v>
+        <v>95.5694528334882</v>
       </c>
       <c r="P94">
         <v>49058</v>
@@ -6826,10 +6826,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N95">
-        <v>90.07772910426883</v>
+        <v>90.07772910426878</v>
       </c>
       <c r="O95">
-        <v>95.56945283348823</v>
+        <v>95.5694528334882</v>
       </c>
       <c r="P95">
         <v>49058</v>
@@ -6894,10 +6894,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N96">
-        <v>90.07772910426883</v>
+        <v>90.07772910426878</v>
       </c>
       <c r="O96">
-        <v>95.56945283348823</v>
+        <v>95.5694528334882</v>
       </c>
       <c r="P96">
         <v>49058</v>
@@ -6908,7 +6908,7 @@
         </is>
       </c>
       <c r="S96">
-        <v>-2.036080868973866</v>
+        <v>-2.0360808689739</v>
       </c>
     </row>
     <row r="97">
@@ -6962,10 +6962,10 @@
         <v>97.35418313024078</v>
       </c>
       <c r="N97">
-        <v>90.07772910426883</v>
+        <v>90.07772910426878</v>
       </c>
       <c r="O97">
-        <v>95.56945283348823</v>
+        <v>95.5694528334882</v>
       </c>
       <c r="P97">
         <v>49058</v>
@@ -6976,7 +6976,7 @@
         </is>
       </c>
       <c r="S97">
-        <v>3.455642860245545</v>
+        <v>3.455642860245511</v>
       </c>
     </row>
     <row r="98">
@@ -7030,10 +7030,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N98">
-        <v>60.39792154911977</v>
+        <v>60.39792154911988</v>
       </c>
       <c r="O98">
-        <v>61.3884842702589</v>
+        <v>61.38848427025866</v>
       </c>
       <c r="P98">
         <v>55325</v>
@@ -7098,10 +7098,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N99">
-        <v>60.39792154911977</v>
+        <v>60.39792154911988</v>
       </c>
       <c r="O99">
-        <v>61.3884842702589</v>
+        <v>61.38848427025866</v>
       </c>
       <c r="P99">
         <v>55325</v>
@@ -7166,10 +7166,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N100">
-        <v>60.39792154911977</v>
+        <v>60.39792154911988</v>
       </c>
       <c r="O100">
-        <v>61.3884842702589</v>
+        <v>61.38848427025866</v>
       </c>
       <c r="P100">
         <v>55325</v>
@@ -7180,7 +7180,7 @@
         </is>
       </c>
       <c r="S100">
-        <v>-1.447053910698781</v>
+        <v>-1.44705391069867</v>
       </c>
     </row>
     <row r="101">
@@ -7234,10 +7234,10 @@
         <v>61.33920356117392</v>
       </c>
       <c r="N101">
-        <v>60.39792154911977</v>
+        <v>60.39792154911988</v>
       </c>
       <c r="O101">
-        <v>61.3884842702589</v>
+        <v>61.38848427025866</v>
       </c>
       <c r="P101">
         <v>55325</v>
@@ -7248,7 +7248,7 @@
         </is>
       </c>
       <c r="S101">
-        <v>-0.4564911895596491</v>
+        <v>-0.4564911895598933</v>
       </c>
     </row>
     <row r="102">
@@ -7302,10 +7302,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N102">
-        <v>51.9685103540086</v>
+        <v>51.96851035400858</v>
       </c>
       <c r="O102">
-        <v>55.16820532599615</v>
+        <v>55.16820532599596</v>
       </c>
       <c r="P102">
         <v>55400</v>
@@ -7370,10 +7370,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N103">
-        <v>51.9685103540086</v>
+        <v>51.96851035400858</v>
       </c>
       <c r="O103">
-        <v>55.16820532599615</v>
+        <v>55.16820532599596</v>
       </c>
       <c r="P103">
         <v>55400</v>
@@ -7438,10 +7438,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N104">
-        <v>51.9685103540086</v>
+        <v>51.96851035400858</v>
       </c>
       <c r="O104">
-        <v>55.16820532599615</v>
+        <v>55.16820532599596</v>
       </c>
       <c r="P104">
         <v>55400</v>
@@ -7452,7 +7452,7 @@
         </is>
       </c>
       <c r="S104">
-        <v>-0.4053152415142924</v>
+        <v>-0.4053152415143146</v>
       </c>
     </row>
     <row r="105">
@@ -7506,10 +7506,10 @@
         <v>51.97518434916385</v>
       </c>
       <c r="N105">
-        <v>51.9685103540086</v>
+        <v>51.96851035400858</v>
       </c>
       <c r="O105">
-        <v>55.16820532599615</v>
+        <v>55.16820532599596</v>
       </c>
       <c r="P105">
         <v>55400</v>
@@ -7520,7 +7520,7 @@
         </is>
       </c>
       <c r="S105">
-        <v>2.794379730473251</v>
+        <v>2.794379730473062</v>
       </c>
     </row>
     <row r="106">
@@ -7574,10 +7574,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N106">
-        <v>87.32994267910608</v>
+        <v>87.32994267910654</v>
       </c>
       <c r="O106">
-        <v>92.33804839648158</v>
+        <v>92.33804839648147</v>
       </c>
       <c r="P106">
         <v>55242</v>
@@ -7642,10 +7642,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N107">
-        <v>87.32994267910608</v>
+        <v>87.32994267910654</v>
       </c>
       <c r="O107">
-        <v>92.33804839648158</v>
+        <v>92.33804839648147</v>
       </c>
       <c r="P107">
         <v>55242</v>
@@ -7710,10 +7710,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N108">
-        <v>87.32994267910608</v>
+        <v>87.32994267910654</v>
       </c>
       <c r="O108">
-        <v>92.33804839648158</v>
+        <v>92.33804839648147</v>
       </c>
       <c r="P108">
         <v>55242</v>
@@ -7724,7 +7724,7 @@
         </is>
       </c>
       <c r="S108">
-        <v>-0.1009559809642679</v>
+        <v>-0.1009559809638128</v>
       </c>
     </row>
     <row r="109">
@@ -7778,10 +7778,10 @@
         <v>92.92783958842196</v>
       </c>
       <c r="N109">
-        <v>87.32994267910608</v>
+        <v>87.32994267910654</v>
       </c>
       <c r="O109">
-        <v>92.33804839648158</v>
+        <v>92.33804839648147</v>
       </c>
       <c r="P109">
         <v>55242</v>
@@ -7792,7 +7792,7 @@
         </is>
       </c>
       <c r="S109">
-        <v>4.907149736411231</v>
+        <v>4.907149736411109</v>
       </c>
     </row>
     <row r="110">
@@ -7846,10 +7846,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N110">
-        <v>90.29738719024508</v>
+        <v>90.29738719024533</v>
       </c>
       <c r="O110">
-        <v>85.14002215874885</v>
+        <v>85.14002215874858</v>
       </c>
       <c r="P110">
         <v>55400</v>
@@ -7914,10 +7914,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N111">
-        <v>90.29738719024508</v>
+        <v>90.29738719024533</v>
       </c>
       <c r="O111">
-        <v>85.14002215874885</v>
+        <v>85.14002215874858</v>
       </c>
       <c r="P111">
         <v>55400</v>
@@ -7982,10 +7982,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N112">
-        <v>90.29738719024508</v>
+        <v>90.29738719024533</v>
       </c>
       <c r="O112">
-        <v>85.14002215874885</v>
+        <v>85.14002215874858</v>
       </c>
       <c r="P112">
         <v>55400</v>
@@ -7996,7 +7996,7 @@
         </is>
       </c>
       <c r="S112">
-        <v>0.729413685619984</v>
+        <v>0.7294136856202504</v>
       </c>
     </row>
     <row r="113">
@@ -8050,10 +8050,10 @@
         <v>86.30129201699636</v>
       </c>
       <c r="N113">
-        <v>90.29738719024508</v>
+        <v>90.29738719024533</v>
       </c>
       <c r="O113">
-        <v>85.14002215874885</v>
+        <v>85.14002215874858</v>
       </c>
       <c r="P113">
         <v>55400</v>
@@ -8064,7 +8064,7 @@
         </is>
       </c>
       <c r="S113">
-        <v>-4.427951345876235</v>
+        <v>-4.427951345876502</v>
       </c>
     </row>
     <row r="114">
@@ -8118,10 +8118,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N114">
-        <v>81.97678428265853</v>
+        <v>81.97678428265843</v>
       </c>
       <c r="O114">
-        <v>78.85814310205289</v>
+        <v>78.85814310205271</v>
       </c>
       <c r="P114">
         <v>37859</v>
@@ -8186,10 +8186,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N115">
-        <v>81.97678428265853</v>
+        <v>81.97678428265843</v>
       </c>
       <c r="O115">
-        <v>78.85814310205289</v>
+        <v>78.85814310205271</v>
       </c>
       <c r="P115">
         <v>37859</v>
@@ -8254,10 +8254,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N116">
-        <v>81.97678428265853</v>
+        <v>81.97678428265843</v>
       </c>
       <c r="O116">
-        <v>78.85814310205289</v>
+        <v>78.85814310205271</v>
       </c>
       <c r="P116">
         <v>37859</v>
@@ -8268,7 +8268,7 @@
         </is>
       </c>
       <c r="S116">
-        <v>-0.8086498910109485</v>
+        <v>-0.8086498910110373</v>
       </c>
     </row>
     <row r="117">
@@ -8322,10 +8322,10 @@
         <v>78.40310703823478</v>
       </c>
       <c r="N117">
-        <v>81.97678428265853</v>
+        <v>81.97678428265843</v>
       </c>
       <c r="O117">
-        <v>78.85814310205289</v>
+        <v>78.85814310205271</v>
       </c>
       <c r="P117">
         <v>37859</v>
@@ -8336,7 +8336,7 @@
         </is>
       </c>
       <c r="S117">
-        <v>-3.927291071616579</v>
+        <v>-3.927291071616756</v>
       </c>
     </row>
     <row r="118">
@@ -8390,10 +8390,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N118">
-        <v>61.84561105159655</v>
+        <v>61.84561105159537</v>
       </c>
       <c r="O118">
-        <v>26.29907721541566</v>
+        <v>26.29907721541595</v>
       </c>
       <c r="P118">
         <v>44776</v>
@@ -8458,10 +8458,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N119">
-        <v>61.84561105159655</v>
+        <v>61.84561105159537</v>
       </c>
       <c r="O119">
-        <v>26.29907721541566</v>
+        <v>26.29907721541595</v>
       </c>
       <c r="P119">
         <v>44776</v>
@@ -8526,10 +8526,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N120">
-        <v>61.84561105159655</v>
+        <v>61.84561105159537</v>
       </c>
       <c r="O120">
-        <v>26.29907721541566</v>
+        <v>26.29907721541595</v>
       </c>
       <c r="P120">
         <v>44776</v>
@@ -8540,7 +8540,7 @@
         </is>
       </c>
       <c r="S120">
-        <v>0.3570698780801185</v>
+        <v>0.3570698780789416</v>
       </c>
     </row>
     <row r="121">
@@ -8594,10 +8594,10 @@
         <v>27.81811575108459</v>
       </c>
       <c r="N121">
-        <v>61.84561105159655</v>
+        <v>61.84561105159537</v>
       </c>
       <c r="O121">
-        <v>26.29907721541566</v>
+        <v>26.29907721541595</v>
       </c>
       <c r="P121">
         <v>44776</v>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="S121">
-        <v>-35.18946395810077</v>
+        <v>-35.18946395810048</v>
       </c>
     </row>
     <row r="122">
@@ -8662,10 +8662,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N122">
-        <v>18.78381922591106</v>
+        <v>18.78381922591102</v>
       </c>
       <c r="O122">
-        <v>18.78376405592467</v>
+        <v>18.78376405592434</v>
       </c>
       <c r="P122">
         <v>54535</v>
@@ -8730,10 +8730,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N123">
-        <v>18.78381922591106</v>
+        <v>18.78381922591102</v>
       </c>
       <c r="O123">
-        <v>18.78376405592467</v>
+        <v>18.78376405592434</v>
       </c>
       <c r="P123">
         <v>54535</v>
@@ -8798,10 +8798,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N124">
-        <v>18.78381922591106</v>
+        <v>18.78381922591102</v>
       </c>
       <c r="O124">
-        <v>18.78376405592467</v>
+        <v>18.78376405592434</v>
       </c>
       <c r="P124">
         <v>54535</v>
@@ -8812,7 +8812,7 @@
         </is>
       </c>
       <c r="S124">
-        <v>-0.5877807213773428</v>
+        <v>-0.5877807213773845</v>
       </c>
     </row>
     <row r="125">
@@ -8866,10 +8866,10 @@
         <v>19.55956107979261</v>
       </c>
       <c r="N125">
-        <v>18.78381922591106</v>
+        <v>18.78381922591102</v>
       </c>
       <c r="O125">
-        <v>18.78376405592467</v>
+        <v>18.78376405592434</v>
       </c>
       <c r="P125">
         <v>54535</v>
@@ -8880,7 +8880,7 @@
         </is>
       </c>
       <c r="S125">
-        <v>-0.587835891363736</v>
+        <v>-0.5878358913640636</v>
       </c>
     </row>
     <row r="126">
@@ -8934,10 +8934,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N126">
-        <v>30.53786279215646</v>
+        <v>30.53786279215657</v>
       </c>
       <c r="O126">
-        <v>30.53774451303555</v>
+        <v>30.53774451303544</v>
       </c>
       <c r="P126">
         <v>54535</v>
@@ -9002,10 +9002,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N127">
-        <v>30.53786279215646</v>
+        <v>30.53786279215657</v>
       </c>
       <c r="O127">
-        <v>30.53774451303555</v>
+        <v>30.53774451303544</v>
       </c>
       <c r="P127">
         <v>54535</v>
@@ -9070,10 +9070,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N128">
-        <v>30.53786279215646</v>
+        <v>30.53786279215657</v>
       </c>
       <c r="O128">
-        <v>30.53774451303555</v>
+        <v>30.53774451303544</v>
       </c>
       <c r="P128">
         <v>54535</v>
@@ -9084,7 +9084,7 @@
         </is>
       </c>
       <c r="S128">
-        <v>-0.1367483492706933</v>
+        <v>-0.1367483492705823</v>
       </c>
     </row>
     <row r="129">
@@ -9138,10 +9138,10 @@
         <v>30.49659378673363</v>
       </c>
       <c r="N129">
-        <v>30.53786279215646</v>
+        <v>30.53786279215657</v>
       </c>
       <c r="O129">
-        <v>30.53774451303555</v>
+        <v>30.53774451303544</v>
       </c>
       <c r="P129">
         <v>54535</v>
@@ -9152,7 +9152,7 @@
         </is>
       </c>
       <c r="S129">
-        <v>-0.136866628391602</v>
+        <v>-0.136866628391713</v>
       </c>
     </row>
     <row r="130">
@@ -9206,10 +9206,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N130">
-        <v>60.0704815986113</v>
+        <v>60.07048159861138</v>
       </c>
       <c r="O130">
-        <v>60.07051969567441</v>
+        <v>60.07051969567385</v>
       </c>
       <c r="P130">
         <v>54535</v>
@@ -9274,10 +9274,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N131">
-        <v>60.0704815986113</v>
+        <v>60.07048159861138</v>
       </c>
       <c r="O131">
-        <v>60.07051969567441</v>
+        <v>60.07051969567385</v>
       </c>
       <c r="P131">
         <v>54535</v>
@@ -9342,10 +9342,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N132">
-        <v>60.0704815986113</v>
+        <v>60.07048159861138</v>
       </c>
       <c r="O132">
-        <v>60.07051969567441</v>
+        <v>60.07051969567385</v>
       </c>
       <c r="P132">
         <v>54535</v>
@@ -9356,7 +9356,7 @@
         </is>
       </c>
       <c r="S132">
-        <v>-0.7931925941981666</v>
+        <v>-0.7931925941980889</v>
       </c>
     </row>
     <row r="133">
@@ -9410,10 +9410,10 @@
         <v>46.0408366864019</v>
       </c>
       <c r="N133">
-        <v>60.0704815986113</v>
+        <v>60.07048159861138</v>
       </c>
       <c r="O133">
-        <v>60.07051969567441</v>
+        <v>60.07051969567385</v>
       </c>
       <c r="P133">
         <v>54535</v>
@@ -9424,7 +9424,7 @@
         </is>
       </c>
       <c r="S133">
-        <v>-0.7931544971350624</v>
+        <v>-0.7931544971356175</v>
       </c>
     </row>
     <row r="134">
@@ -9478,10 +9478,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N134">
-        <v>22.8075281326633</v>
+        <v>22.80752813266336</v>
       </c>
       <c r="O134">
-        <v>22.80764277056721</v>
+        <v>22.80764277056756</v>
       </c>
       <c r="P134">
         <v>47918</v>
@@ -9546,10 +9546,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N135">
-        <v>22.8075281326633</v>
+        <v>22.80752813266336</v>
       </c>
       <c r="O135">
-        <v>22.80764277056721</v>
+        <v>22.80764277056756</v>
       </c>
       <c r="P135">
         <v>47918</v>
@@ -9614,10 +9614,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N136">
-        <v>22.8075281326633</v>
+        <v>22.80752813266336</v>
       </c>
       <c r="O136">
-        <v>22.80764277056721</v>
+        <v>22.80764277056756</v>
       </c>
       <c r="P136">
         <v>47918</v>
@@ -9628,7 +9628,7 @@
         </is>
       </c>
       <c r="S136">
-        <v>-0.6564727659102182</v>
+        <v>-0.6564727659101488</v>
       </c>
     </row>
     <row r="137">
@@ -9682,10 +9682,10 @@
         <v>22.21829840823713</v>
       </c>
       <c r="N137">
-        <v>22.8075281326633</v>
+        <v>22.80752813266336</v>
       </c>
       <c r="O137">
-        <v>22.80764277056721</v>
+        <v>22.80764277056756</v>
       </c>
       <c r="P137">
         <v>47918</v>
@@ -9696,7 +9696,7 @@
         </is>
       </c>
       <c r="S137">
-        <v>-0.6563581280063013</v>
+        <v>-0.6563581280059488</v>
       </c>
     </row>
     <row r="138">
@@ -9750,7 +9750,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N138">
-        <v>89.057646837029</v>
+        <v>89.05764683702921</v>
       </c>
       <c r="O138">
         <v>96.53969112716689</v>
@@ -9818,7 +9818,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N139">
-        <v>89.057646837029</v>
+        <v>89.05764683702921</v>
       </c>
       <c r="O139">
         <v>96.53969112716689</v>
@@ -9886,7 +9886,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N140">
-        <v>89.057646837029</v>
+        <v>89.05764683702921</v>
       </c>
       <c r="O140">
         <v>96.53969112716689</v>
@@ -9900,7 +9900,7 @@
         </is>
       </c>
       <c r="S140">
-        <v>-2.609675776510978</v>
+        <v>-2.609675776510767</v>
       </c>
     </row>
     <row r="141">
@@ -9954,7 +9954,7 @@
         <v>97.70353186034932</v>
       </c>
       <c r="N141">
-        <v>89.057646837029</v>
+        <v>89.05764683702921</v>
       </c>
       <c r="O141">
         <v>96.53969112716689</v>
@@ -10022,10 +10022,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N142">
-        <v>61.88484918229447</v>
+        <v>61.88484918229459</v>
       </c>
       <c r="O142">
-        <v>61.4772745944154</v>
+        <v>61.47727459441587</v>
       </c>
       <c r="P142">
         <v>54426</v>
@@ -10090,10 +10090,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N143">
-        <v>61.88484918229447</v>
+        <v>61.88484918229459</v>
       </c>
       <c r="O143">
-        <v>61.4772745944154</v>
+        <v>61.47727459441587</v>
       </c>
       <c r="P143">
         <v>54426</v>
@@ -10158,10 +10158,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N144">
-        <v>61.88484918229447</v>
+        <v>61.88484918229459</v>
       </c>
       <c r="O144">
-        <v>61.4772745944154</v>
+        <v>61.47727459441587</v>
       </c>
       <c r="P144">
         <v>54426</v>
@@ -10172,7 +10172,7 @@
         </is>
       </c>
       <c r="S144">
-        <v>-1.127829715025674</v>
+        <v>-1.127829715025552</v>
       </c>
     </row>
     <row r="145">
@@ -10226,10 +10226,10 @@
         <v>60.16767859230833</v>
       </c>
       <c r="N145">
-        <v>61.88484918229447</v>
+        <v>61.88484918229459</v>
       </c>
       <c r="O145">
-        <v>61.4772745944154</v>
+        <v>61.47727459441587</v>
       </c>
       <c r="P145">
         <v>54426</v>
@@ -10240,7 +10240,7 @@
         </is>
       </c>
       <c r="S145">
-        <v>-1.535404302904742</v>
+        <v>-1.535404302904275</v>
       </c>
     </row>
     <row r="146">
@@ -10294,10 +10294,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N146">
-        <v>52.10416026488397</v>
+        <v>52.10416026488398</v>
       </c>
       <c r="O146">
-        <v>53.71180101699645</v>
+        <v>53.71180101699651</v>
       </c>
       <c r="P146">
         <v>54535</v>
@@ -10362,10 +10362,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N147">
-        <v>52.10416026488397</v>
+        <v>52.10416026488398</v>
       </c>
       <c r="O147">
-        <v>53.71180101699645</v>
+        <v>53.71180101699651</v>
       </c>
       <c r="P147">
         <v>54535</v>
@@ -10430,10 +10430,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N148">
-        <v>52.10416026488397</v>
+        <v>52.10416026488398</v>
       </c>
       <c r="O148">
-        <v>53.71180101699645</v>
+        <v>53.71180101699651</v>
       </c>
       <c r="P148">
         <v>54535</v>
@@ -10444,7 +10444,7 @@
         </is>
       </c>
       <c r="S148">
-        <v>-0.1882192833705831</v>
+        <v>-0.188219283370572</v>
       </c>
     </row>
     <row r="149">
@@ -10498,10 +10498,10 @@
         <v>51.81970969080953</v>
       </c>
       <c r="N149">
-        <v>52.10416026488397</v>
+        <v>52.10416026488398</v>
       </c>
       <c r="O149">
-        <v>53.71180101699645</v>
+        <v>53.71180101699651</v>
       </c>
       <c r="P149">
         <v>54535</v>
@@ -10512,7 +10512,7 @@
         </is>
       </c>
       <c r="S149">
-        <v>1.419421468741899</v>
+        <v>1.419421468741955</v>
       </c>
     </row>
     <row r="150">
@@ -10566,10 +10566,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N150">
-        <v>88.10981089169665</v>
+        <v>88.10981089169675</v>
       </c>
       <c r="O150">
-        <v>92.81601489807952</v>
+        <v>92.81601489807957</v>
       </c>
       <c r="P150">
         <v>54281</v>
@@ -10634,10 +10634,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N151">
-        <v>88.10981089169665</v>
+        <v>88.10981089169675</v>
       </c>
       <c r="O151">
-        <v>92.81601489807952</v>
+        <v>92.81601489807957</v>
       </c>
       <c r="P151">
         <v>54281</v>
@@ -10702,10 +10702,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N152">
-        <v>88.10981089169665</v>
+        <v>88.10981089169675</v>
       </c>
       <c r="O152">
-        <v>92.81601489807952</v>
+        <v>92.81601489807957</v>
       </c>
       <c r="P152">
         <v>54281</v>
@@ -10716,7 +10716,7 @@
         </is>
       </c>
       <c r="S152">
-        <v>0.03641639628380045</v>
+        <v>0.03641639628391147</v>
       </c>
     </row>
     <row r="153">
@@ -10770,10 +10770,10 @@
         <v>93.85406722827751</v>
       </c>
       <c r="N153">
-        <v>88.10981089169665</v>
+        <v>88.10981089169675</v>
       </c>
       <c r="O153">
-        <v>92.81601489807952</v>
+        <v>92.81601489807957</v>
       </c>
       <c r="P153">
         <v>54281</v>
@@ -10784,7 +10784,7 @@
         </is>
       </c>
       <c r="S153">
-        <v>4.742620402666664</v>
+        <v>4.742620402666731</v>
       </c>
     </row>
     <row r="154">
@@ -10838,10 +10838,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N154">
-        <v>90.59641787470704</v>
+        <v>90.59641787470699</v>
       </c>
       <c r="O154">
-        <v>86.4560265318876</v>
+        <v>86.45602653188774</v>
       </c>
       <c r="P154">
         <v>54534</v>
@@ -10906,10 +10906,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N155">
-        <v>90.59641787470704</v>
+        <v>90.59641787470699</v>
       </c>
       <c r="O155">
-        <v>86.4560265318876</v>
+        <v>86.45602653188774</v>
       </c>
       <c r="P155">
         <v>54534</v>
@@ -10974,10 +10974,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N156">
-        <v>90.59641787470704</v>
+        <v>90.59641787470699</v>
       </c>
       <c r="O156">
-        <v>86.4560265318876</v>
+        <v>86.45602653188774</v>
       </c>
       <c r="P156">
         <v>54534</v>
@@ -10988,7 +10988,7 @@
         </is>
       </c>
       <c r="S156">
-        <v>0.6425753431986925</v>
+        <v>0.642575343198637</v>
       </c>
     </row>
     <row r="157">
@@ -11042,10 +11042,10 @@
         <v>87.6320105705225</v>
       </c>
       <c r="N157">
-        <v>90.59641787470704</v>
+        <v>90.59641787470699</v>
       </c>
       <c r="O157">
-        <v>86.4560265318876</v>
+        <v>86.45602653188774</v>
       </c>
       <c r="P157">
         <v>54534</v>
@@ -11056,7 +11056,7 @@
         </is>
       </c>
       <c r="S157">
-        <v>-3.497815999620746</v>
+        <v>-3.497815999620613</v>
       </c>
     </row>
     <row r="158">
@@ -11110,10 +11110,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N158">
-        <v>81.45050683818823</v>
+        <v>81.45050683818815</v>
       </c>
       <c r="O158">
-        <v>77.4884120909541</v>
+        <v>77.48841209095431</v>
       </c>
       <c r="P158">
         <v>39772</v>
@@ -11178,10 +11178,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N159">
-        <v>81.45050683818823</v>
+        <v>81.45050683818815</v>
       </c>
       <c r="O159">
-        <v>77.4884120909541</v>
+        <v>77.48841209095431</v>
       </c>
       <c r="P159">
         <v>39772</v>
@@ -11246,10 +11246,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N160">
-        <v>81.45050683818823</v>
+        <v>81.45050683818815</v>
       </c>
       <c r="O160">
-        <v>77.4884120909541</v>
+        <v>77.48841209095431</v>
       </c>
       <c r="P160">
         <v>39772</v>
@@ -11260,7 +11260,7 @@
         </is>
       </c>
       <c r="S160">
-        <v>-0.5301548422915192</v>
+        <v>-0.5301548422915969</v>
       </c>
     </row>
     <row r="161">
@@ -11314,10 +11314,10 @@
         <v>77.14401961658972</v>
       </c>
       <c r="N161">
-        <v>81.45050683818823</v>
+        <v>81.45050683818815</v>
       </c>
       <c r="O161">
-        <v>77.4884120909541</v>
+        <v>77.48841209095431</v>
       </c>
       <c r="P161">
         <v>39772</v>
@@ -11328,7 +11328,7 @@
         </is>
       </c>
       <c r="S161">
-        <v>-4.492249589525644</v>
+        <v>-4.492249589525443</v>
       </c>
     </row>
     <row r="162">
@@ -11382,10 +11382,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N162">
-        <v>53.97907512970576</v>
+        <v>53.97907512970481</v>
       </c>
       <c r="O162">
-        <v>90.77842736117594</v>
+        <v>90.77842736117616</v>
       </c>
       <c r="P162">
         <v>42552</v>
@@ -11450,10 +11450,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N163">
-        <v>53.97907512970576</v>
+        <v>53.97907512970481</v>
       </c>
       <c r="O163">
-        <v>90.77842736117594</v>
+        <v>90.77842736117616</v>
       </c>
       <c r="P163">
         <v>42552</v>
@@ -11518,10 +11518,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N164">
-        <v>53.97907512970576</v>
+        <v>53.97907512970481</v>
       </c>
       <c r="O164">
-        <v>90.77842736117594</v>
+        <v>90.77842736117616</v>
       </c>
       <c r="P164">
         <v>42552</v>
@@ -11532,7 +11532,7 @@
         </is>
       </c>
       <c r="S164">
-        <v>0.0008416705650216016</v>
+        <v>0.0008416705640779121</v>
       </c>
     </row>
     <row r="165">
@@ -11586,10 +11586,10 @@
         <v>94.73858354545469</v>
       </c>
       <c r="N165">
-        <v>53.97907512970576</v>
+        <v>53.97907512970481</v>
       </c>
       <c r="O165">
-        <v>90.77842736117594</v>
+        <v>90.77842736117616</v>
       </c>
       <c r="P165">
         <v>42552</v>
@@ -11600,7 +11600,7 @@
         </is>
       </c>
       <c r="S165">
-        <v>36.8001939020352</v>
+        <v>36.80019390203542</v>
       </c>
     </row>
     <row r="166">
@@ -20358,10 +20358,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N294">
-        <v>15.41815523864194</v>
+        <v>15.41815523864195</v>
       </c>
       <c r="O294">
-        <v>15.39358401703903</v>
+        <v>15.39358401703959</v>
       </c>
       <c r="P294">
         <v>61000</v>
@@ -20426,10 +20426,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N295">
-        <v>15.41815523864194</v>
+        <v>15.41815523864195</v>
       </c>
       <c r="O295">
-        <v>15.39358401703903</v>
+        <v>15.39358401703959</v>
       </c>
       <c r="P295">
         <v>61000</v>
@@ -20494,10 +20494,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N296">
-        <v>15.41815523864194</v>
+        <v>15.41815523864195</v>
       </c>
       <c r="O296">
-        <v>15.39358401703903</v>
+        <v>15.39358401703959</v>
       </c>
       <c r="P296">
         <v>61000</v>
@@ -20508,7 +20508,7 @@
         </is>
       </c>
       <c r="S296">
-        <v>-2.434066014787231</v>
+        <v>-2.43406601478722</v>
       </c>
     </row>
     <row r="297">
@@ -20562,10 +20562,10 @@
         <v>13.71421764662618</v>
       </c>
       <c r="N297">
-        <v>15.41815523864194</v>
+        <v>15.41815523864195</v>
       </c>
       <c r="O297">
-        <v>15.39358401703903</v>
+        <v>15.39358401703959</v>
       </c>
       <c r="P297">
         <v>61000</v>
@@ -20576,7 +20576,7 @@
         </is>
       </c>
       <c r="S297">
-        <v>-2.458637236390146</v>
+        <v>-2.458637236389585</v>
       </c>
     </row>
     <row r="298">
@@ -20630,10 +20630,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N298">
-        <v>28.57244554318082</v>
+        <v>28.57244554318077</v>
       </c>
       <c r="O298">
-        <v>28.56364349950706</v>
+        <v>28.56364349950802</v>
       </c>
       <c r="P298">
         <v>61000</v>
@@ -20698,10 +20698,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N299">
-        <v>28.57244554318082</v>
+        <v>28.57244554318077</v>
       </c>
       <c r="O299">
-        <v>28.56364349950706</v>
+        <v>28.56364349950802</v>
       </c>
       <c r="P299">
         <v>61000</v>
@@ -20766,10 +20766,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N300">
-        <v>28.57244554318082</v>
+        <v>28.57244554318077</v>
       </c>
       <c r="O300">
-        <v>28.56364349950706</v>
+        <v>28.56364349950802</v>
       </c>
       <c r="P300">
         <v>61000</v>
@@ -20780,7 +20780,7 @@
         </is>
       </c>
       <c r="S300">
-        <v>-0.5880716505328953</v>
+        <v>-0.5880716505329397</v>
       </c>
     </row>
     <row r="301">
@@ -20834,10 +20834,10 @@
         <v>29.42277298055462</v>
       </c>
       <c r="N301">
-        <v>28.57244554318082</v>
+        <v>28.57244554318077</v>
       </c>
       <c r="O301">
-        <v>28.56364349950706</v>
+        <v>28.56364349950802</v>
       </c>
       <c r="P301">
         <v>61000</v>
@@ -20848,7 +20848,7 @@
         </is>
       </c>
       <c r="S301">
-        <v>-0.5968736942066566</v>
+        <v>-0.5968736942056962</v>
       </c>
     </row>
     <row r="302">
@@ -20902,10 +20902,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N302">
-        <v>57.98657659676807</v>
+        <v>57.98657659676809</v>
       </c>
       <c r="O302">
-        <v>58.0108328128641</v>
+        <v>58.0108328128659</v>
       </c>
       <c r="P302">
         <v>60966</v>
@@ -20970,10 +20970,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N303">
-        <v>57.98657659676807</v>
+        <v>57.98657659676809</v>
       </c>
       <c r="O303">
-        <v>58.0108328128641</v>
+        <v>58.0108328128659</v>
       </c>
       <c r="P303">
         <v>60966</v>
@@ -21038,10 +21038,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N304">
-        <v>57.98657659676807</v>
+        <v>57.98657659676809</v>
       </c>
       <c r="O304">
-        <v>58.0108328128641</v>
+        <v>58.0108328128659</v>
       </c>
       <c r="P304">
         <v>60966</v>
@@ -21052,7 +21052,7 @@
         </is>
       </c>
       <c r="S304">
-        <v>0.9354526786854334</v>
+        <v>0.9354526786854556</v>
       </c>
     </row>
     <row r="305">
@@ -21106,10 +21106,10 @@
         <v>45.4639903673616</v>
       </c>
       <c r="N305">
-        <v>57.98657659676807</v>
+        <v>57.98657659676809</v>
       </c>
       <c r="O305">
-        <v>58.0108328128641</v>
+        <v>58.0108328128659</v>
       </c>
       <c r="P305">
         <v>60966</v>
@@ -21120,7 +21120,7 @@
         </is>
       </c>
       <c r="S305">
-        <v>0.9597088947814636</v>
+        <v>0.9597088947832622</v>
       </c>
     </row>
     <row r="306">
@@ -21174,10 +21174,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N306">
-        <v>24.28635160555295</v>
+        <v>24.28635160555294</v>
       </c>
       <c r="O306">
-        <v>24.30807920702731</v>
+        <v>24.30807920702841</v>
       </c>
       <c r="P306">
         <v>54906</v>
@@ -21242,10 +21242,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N307">
-        <v>24.28635160555295</v>
+        <v>24.28635160555294</v>
       </c>
       <c r="O307">
-        <v>24.30807920702731</v>
+        <v>24.30807920702841</v>
       </c>
       <c r="P307">
         <v>54906</v>
@@ -21310,10 +21310,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N308">
-        <v>24.28635160555295</v>
+        <v>24.28635160555294</v>
       </c>
       <c r="O308">
-        <v>24.30807920702731</v>
+        <v>24.30807920702841</v>
       </c>
       <c r="P308">
         <v>54906</v>
@@ -21324,7 +21324,7 @@
         </is>
       </c>
       <c r="S308">
-        <v>-0.3936985826528183</v>
+        <v>-0.3936985826528322</v>
       </c>
     </row>
     <row r="309">
@@ -21378,10 +21378,10 @@
         <v>22.87686769960688</v>
       </c>
       <c r="N309">
-        <v>24.28635160555295</v>
+        <v>24.28635160555294</v>
       </c>
       <c r="O309">
-        <v>24.30807920702731</v>
+        <v>24.30807920702841</v>
       </c>
       <c r="P309">
         <v>54906</v>
@@ -21392,7 +21392,7 @@
         </is>
       </c>
       <c r="S309">
-        <v>-0.3719709811784599</v>
+        <v>-0.3719709811773608</v>
       </c>
     </row>
     <row r="310">
@@ -21446,10 +21446,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N310">
-        <v>86.70056156845874</v>
+        <v>86.70056156845875</v>
       </c>
       <c r="O310">
-        <v>96.82340183287779</v>
+        <v>96.82340183287785</v>
       </c>
       <c r="P310">
         <v>55751</v>
@@ -21514,10 +21514,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N311">
-        <v>86.70056156845874</v>
+        <v>86.70056156845875</v>
       </c>
       <c r="O311">
-        <v>96.82340183287779</v>
+        <v>96.82340183287785</v>
       </c>
       <c r="P311">
         <v>55751</v>
@@ -21582,10 +21582,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N312">
-        <v>86.70056156845874</v>
+        <v>86.70056156845875</v>
       </c>
       <c r="O312">
-        <v>96.82340183287779</v>
+        <v>96.82340183287785</v>
       </c>
       <c r="P312">
         <v>55751</v>
@@ -21596,7 +21596,7 @@
         </is>
       </c>
       <c r="S312">
-        <v>-3.506571111293733</v>
+        <v>-3.50657111129371</v>
       </c>
     </row>
     <row r="313">
@@ -21650,10 +21650,10 @@
         <v>96.75096455756443</v>
       </c>
       <c r="N313">
-        <v>86.70056156845874</v>
+        <v>86.70056156845875</v>
       </c>
       <c r="O313">
-        <v>96.82340183287779</v>
+        <v>96.82340183287785</v>
       </c>
       <c r="P313">
         <v>55751</v>
@@ -21664,7 +21664,7 @@
         </is>
       </c>
       <c r="S313">
-        <v>6.61626915312532</v>
+        <v>6.616269153125376</v>
       </c>
     </row>
     <row r="314">
@@ -21718,10 +21718,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N314">
-        <v>59.81528043082663</v>
+        <v>59.81528043082665</v>
       </c>
       <c r="O314">
-        <v>60.34381502084364</v>
+        <v>60.34381502084475</v>
       </c>
       <c r="P314">
         <v>60920</v>
@@ -21786,10 +21786,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N315">
-        <v>59.81528043082663</v>
+        <v>59.81528043082665</v>
       </c>
       <c r="O315">
-        <v>60.34381502084364</v>
+        <v>60.34381502084475</v>
       </c>
       <c r="P315">
         <v>60920</v>
@@ -21854,10 +21854,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N316">
-        <v>59.81528043082663</v>
+        <v>59.81528043082665</v>
       </c>
       <c r="O316">
-        <v>60.34381502084364</v>
+        <v>60.34381502084475</v>
       </c>
       <c r="P316">
         <v>60920</v>
@@ -21868,7 +21868,7 @@
         </is>
       </c>
       <c r="S316">
-        <v>-1.367740548997154</v>
+        <v>-1.367740548997121</v>
       </c>
     </row>
     <row r="317">
@@ -21922,10 +21922,10 @@
         <v>60.51866627019677</v>
       </c>
       <c r="N317">
-        <v>59.81528043082663</v>
+        <v>59.81528043082665</v>
       </c>
       <c r="O317">
-        <v>60.34381502084364</v>
+        <v>60.34381502084475</v>
       </c>
       <c r="P317">
         <v>60920</v>
@@ -21936,7 +21936,7 @@
         </is>
       </c>
       <c r="S317">
-        <v>-0.8392059589801382</v>
+        <v>-0.8392059589790279</v>
       </c>
     </row>
     <row r="318">
@@ -21990,10 +21990,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N318">
-        <v>51.87442533665201</v>
+        <v>51.87442533665195</v>
       </c>
       <c r="O318">
-        <v>55.19320995384727</v>
+        <v>55.19320995384758</v>
       </c>
       <c r="P318">
         <v>61000</v>
@@ -22058,10 +22058,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N319">
-        <v>51.87442533665201</v>
+        <v>51.87442533665195</v>
       </c>
       <c r="O319">
-        <v>55.19320995384727</v>
+        <v>55.19320995384758</v>
       </c>
       <c r="P319">
         <v>61000</v>
@@ -22126,10 +22126,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N320">
-        <v>51.87442533665201</v>
+        <v>51.87442533665195</v>
       </c>
       <c r="O320">
-        <v>55.19320995384727</v>
+        <v>55.19320995384758</v>
       </c>
       <c r="P320">
         <v>61000</v>
@@ -22140,7 +22140,7 @@
         </is>
       </c>
       <c r="S320">
-        <v>-0.2309273630906716</v>
+        <v>-0.2309273630907271</v>
       </c>
     </row>
     <row r="321">
@@ -22194,10 +22194,10 @@
         <v>51.49802933758593</v>
       </c>
       <c r="N321">
-        <v>51.87442533665201</v>
+        <v>51.87442533665195</v>
       </c>
       <c r="O321">
-        <v>55.19320995384727</v>
+        <v>55.19320995384758</v>
       </c>
       <c r="P321">
         <v>61000</v>
@@ -22208,7 +22208,7 @@
         </is>
       </c>
       <c r="S321">
-        <v>3.087857254104587</v>
+        <v>3.087857254104898</v>
       </c>
     </row>
     <row r="322">
@@ -22262,10 +22262,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N322">
-        <v>88.60775405607029</v>
+        <v>88.60775405607038</v>
       </c>
       <c r="O322">
-        <v>92.81092514217536</v>
+        <v>92.81092514217534</v>
       </c>
       <c r="P322">
         <v>60928</v>
@@ -22330,10 +22330,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N323">
-        <v>88.60775405607029</v>
+        <v>88.60775405607038</v>
       </c>
       <c r="O323">
-        <v>92.81092514217536</v>
+        <v>92.81092514217534</v>
       </c>
       <c r="P323">
         <v>60928</v>
@@ -22398,10 +22398,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N324">
-        <v>88.60775405607029</v>
+        <v>88.60775405607038</v>
       </c>
       <c r="O324">
-        <v>92.81092514217536</v>
+        <v>92.81092514217534</v>
       </c>
       <c r="P324">
         <v>60928</v>
@@ -22412,7 +22412,7 @@
         </is>
       </c>
       <c r="S324">
-        <v>-0.3433119337774126</v>
+        <v>-0.3433119337773349</v>
       </c>
     </row>
     <row r="325">
@@ -22466,10 +22466,10 @@
         <v>94.03767983644056</v>
       </c>
       <c r="N325">
-        <v>88.60775405607029</v>
+        <v>88.60775405607038</v>
       </c>
       <c r="O325">
-        <v>92.81092514217536</v>
+        <v>92.81092514217534</v>
       </c>
       <c r="P325">
         <v>60928</v>
@@ -22480,7 +22480,7 @@
         </is>
       </c>
       <c r="S325">
-        <v>3.859859152327649</v>
+        <v>3.859859152327627</v>
       </c>
     </row>
     <row r="326">
@@ -22534,10 +22534,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N326">
-        <v>92.49798818801627</v>
+        <v>92.49798818801629</v>
       </c>
       <c r="O326">
-        <v>89.42387194359372</v>
+        <v>89.42387194359381</v>
       </c>
       <c r="P326">
         <v>61000</v>
@@ -22602,10 +22602,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N327">
-        <v>92.49798818801627</v>
+        <v>92.49798818801629</v>
       </c>
       <c r="O327">
-        <v>89.42387194359372</v>
+        <v>89.42387194359381</v>
       </c>
       <c r="P327">
         <v>61000</v>
@@ -22670,10 +22670,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N328">
-        <v>92.49798818801627</v>
+        <v>92.49798818801629</v>
       </c>
       <c r="O328">
-        <v>89.42387194359372</v>
+        <v>89.42387194359381</v>
       </c>
       <c r="P328">
         <v>61000</v>
@@ -22684,7 +22684,7 @@
         </is>
       </c>
       <c r="S328">
-        <v>0.9126431762666365</v>
+        <v>0.9126431762666587</v>
       </c>
     </row>
     <row r="329">
@@ -22738,10 +22738,10 @@
         <v>90.12539655528288</v>
       </c>
       <c r="N329">
-        <v>92.49798818801627</v>
+        <v>92.49798818801629</v>
       </c>
       <c r="O329">
-        <v>89.42387194359372</v>
+        <v>89.42387194359381</v>
       </c>
       <c r="P329">
         <v>61000</v>
@@ -22752,7 +22752,7 @@
         </is>
       </c>
       <c r="S329">
-        <v>-2.161473068155906</v>
+        <v>-2.161473068155828</v>
       </c>
     </row>
     <row r="330">
@@ -22806,10 +22806,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N330">
-        <v>56.80719956100185</v>
+        <v>56.80719956100195</v>
       </c>
       <c r="O330">
-        <v>53.77092581252928</v>
+        <v>53.77092581252965</v>
       </c>
       <c r="P330">
         <v>45790</v>
@@ -22874,10 +22874,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N331">
-        <v>56.80719956100185</v>
+        <v>56.80719956100195</v>
       </c>
       <c r="O331">
-        <v>53.77092581252928</v>
+        <v>53.77092581252965</v>
       </c>
       <c r="P331">
         <v>45790</v>
@@ -22942,10 +22942,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N332">
-        <v>56.80719956100185</v>
+        <v>56.80719956100195</v>
       </c>
       <c r="O332">
-        <v>53.77092581252928</v>
+        <v>53.77092581252965</v>
       </c>
       <c r="P332">
         <v>45790</v>
@@ -22956,7 +22956,7 @@
         </is>
       </c>
       <c r="S332">
-        <v>0.3061338125184943</v>
+        <v>0.3061338125185942</v>
       </c>
     </row>
     <row r="333">
@@ -23010,10 +23010,10 @@
         <v>56.56833363518013</v>
       </c>
       <c r="N333">
-        <v>56.80719956100185</v>
+        <v>56.80719956100195</v>
       </c>
       <c r="O333">
-        <v>53.77092581252928</v>
+        <v>53.77092581252965</v>
       </c>
       <c r="P333">
         <v>45790</v>
@@ -23024,7 +23024,7 @@
         </is>
       </c>
       <c r="S333">
-        <v>-2.730139935954079</v>
+        <v>-2.730139935953713</v>
       </c>
     </row>
     <row r="334">
@@ -23078,10 +23078,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N334">
-        <v>62.0772182760082</v>
+        <v>62.07721827600816</v>
       </c>
       <c r="O334">
-        <v>94.75407612852116</v>
+        <v>94.75407612852125</v>
       </c>
       <c r="P334">
         <v>48462</v>
@@ -23146,10 +23146,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N335">
-        <v>62.0772182760082</v>
+        <v>62.07721827600816</v>
       </c>
       <c r="O335">
-        <v>94.75407612852116</v>
+        <v>94.75407612852125</v>
       </c>
       <c r="P335">
         <v>48462</v>
@@ -23214,10 +23214,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N336">
-        <v>62.0772182760082</v>
+        <v>62.07721827600816</v>
       </c>
       <c r="O336">
-        <v>94.75407612852116</v>
+        <v>94.75407612852125</v>
       </c>
       <c r="P336">
         <v>48462</v>
@@ -23228,7 +23228,7 @@
         </is>
       </c>
       <c r="S336">
-        <v>0.2443851464968394</v>
+        <v>0.244385146496795</v>
       </c>
     </row>
     <row r="337">
@@ -23282,10 +23282,10 @@
         <v>90.08926438227013</v>
       </c>
       <c r="N337">
-        <v>62.0772182760082</v>
+        <v>62.07721827600816</v>
       </c>
       <c r="O337">
-        <v>94.75407612852116</v>
+        <v>94.75407612852125</v>
       </c>
       <c r="P337">
         <v>48462</v>
@@ -23296,7 +23296,7 @@
         </is>
       </c>
       <c r="S337">
-        <v>32.92124299900981</v>
+        <v>32.92124299900988</v>
       </c>
     </row>
     <row r="338">
@@ -23350,10 +23350,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N338">
-        <v>15.79903111329064</v>
+        <v>15.79903111329061</v>
       </c>
       <c r="O338">
-        <v>15.7990265685755</v>
+        <v>15.79902656857579</v>
       </c>
       <c r="P338">
         <v>60000</v>
@@ -23418,10 +23418,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N339">
-        <v>15.79903111329064</v>
+        <v>15.79903111329061</v>
       </c>
       <c r="O339">
-        <v>15.7990265685755</v>
+        <v>15.79902656857579</v>
       </c>
       <c r="P339">
         <v>60000</v>
@@ -23486,10 +23486,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N340">
-        <v>15.79903111329064</v>
+        <v>15.79903111329061</v>
       </c>
       <c r="O340">
-        <v>15.7990265685755</v>
+        <v>15.79902656857579</v>
       </c>
       <c r="P340">
         <v>60000</v>
@@ -23500,7 +23500,7 @@
         </is>
       </c>
       <c r="S340">
-        <v>-2.97334290803713</v>
+        <v>-2.973342908037155</v>
       </c>
     </row>
     <row r="341">
@@ -23554,10 +23554,10 @@
         <v>13.63679623448249</v>
       </c>
       <c r="N341">
-        <v>15.79903111329064</v>
+        <v>15.79903111329061</v>
       </c>
       <c r="O341">
-        <v>15.7990265685755</v>
+        <v>15.79902656857579</v>
       </c>
       <c r="P341">
         <v>60000</v>
@@ -23568,7 +23568,7 @@
         </is>
       </c>
       <c r="S341">
-        <v>-2.97334745275227</v>
+        <v>-2.973347452751979</v>
       </c>
     </row>
     <row r="342">
@@ -23622,10 +23622,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N342">
-        <v>29.12343307178292</v>
+        <v>29.1234330717829</v>
       </c>
       <c r="O342">
-        <v>29.12342358088552</v>
+        <v>29.12342358088578</v>
       </c>
       <c r="P342">
         <v>60000</v>
@@ -23690,10 +23690,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N343">
-        <v>29.12343307178292</v>
+        <v>29.1234330717829</v>
       </c>
       <c r="O343">
-        <v>29.12342358088552</v>
+        <v>29.12342358088578</v>
       </c>
       <c r="P343">
         <v>60000</v>
@@ -23758,10 +23758,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N344">
-        <v>29.12343307178292</v>
+        <v>29.1234330717829</v>
       </c>
       <c r="O344">
-        <v>29.12342358088552</v>
+        <v>29.12342358088578</v>
       </c>
       <c r="P344">
         <v>60000</v>
@@ -23772,7 +23772,7 @@
         </is>
       </c>
       <c r="S344">
-        <v>-0.3447521545214771</v>
+        <v>-0.3447521545214938</v>
       </c>
     </row>
     <row r="345">
@@ -23826,10 +23826,10 @@
         <v>28.71709917682972</v>
       </c>
       <c r="N345">
-        <v>29.12343307178292</v>
+        <v>29.1234330717829</v>
       </c>
       <c r="O345">
-        <v>29.12342358088552</v>
+        <v>29.12342358088578</v>
       </c>
       <c r="P345">
         <v>60000</v>
@@ -23840,7 +23840,7 @@
         </is>
       </c>
       <c r="S345">
-        <v>-0.3447616454188729</v>
+        <v>-0.3447616454186175</v>
       </c>
     </row>
     <row r="346">
@@ -23894,10 +23894,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N346">
-        <v>60.91535036081957</v>
+        <v>60.91535036081953</v>
       </c>
       <c r="O346">
-        <v>60.91538488022654</v>
+        <v>60.91538488022671</v>
       </c>
       <c r="P346">
         <v>59952</v>
@@ -23962,10 +23962,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N347">
-        <v>60.91535036081957</v>
+        <v>60.91535036081953</v>
       </c>
       <c r="O347">
-        <v>60.91538488022654</v>
+        <v>60.91538488022671</v>
       </c>
       <c r="P347">
         <v>59952</v>
@@ -24030,10 +24030,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N348">
-        <v>60.91535036081957</v>
+        <v>60.91535036081953</v>
       </c>
       <c r="O348">
-        <v>60.91538488022654</v>
+        <v>60.91538488022671</v>
       </c>
       <c r="P348">
         <v>59952</v>
@@ -24044,7 +24044,7 @@
         </is>
       </c>
       <c r="S348">
-        <v>2.019584098563221</v>
+        <v>2.019584098563187</v>
       </c>
     </row>
     <row r="349">
@@ -24098,10 +24098,10 @@
         <v>49.38494464192657</v>
       </c>
       <c r="N349">
-        <v>60.91535036081957</v>
+        <v>60.91535036081953</v>
       </c>
       <c r="O349">
-        <v>60.91538488022654</v>
+        <v>60.91538488022671</v>
       </c>
       <c r="P349">
         <v>59952</v>
@@ -24112,7 +24112,7 @@
         </is>
       </c>
       <c r="S349">
-        <v>2.019618617970198</v>
+        <v>2.019618617970365</v>
       </c>
     </row>
     <row r="350">
@@ -24166,10 +24166,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N350">
-        <v>23.77362779864106</v>
+        <v>23.77362779864108</v>
       </c>
       <c r="O350">
-        <v>23.77362873790585</v>
+        <v>23.77362873790611</v>
       </c>
       <c r="P350">
         <v>55143</v>
@@ -24234,10 +24234,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N351">
-        <v>23.77362779864106</v>
+        <v>23.77362779864108</v>
       </c>
       <c r="O351">
-        <v>23.77362873790585</v>
+        <v>23.77362873790611</v>
       </c>
       <c r="P351">
         <v>55143</v>
@@ -24302,10 +24302,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N352">
-        <v>23.77362779864106</v>
+        <v>23.77362779864108</v>
       </c>
       <c r="O352">
-        <v>23.77362873790585</v>
+        <v>23.77362873790611</v>
       </c>
       <c r="P352">
         <v>55143</v>
@@ -24316,7 +24316,7 @@
         </is>
       </c>
       <c r="S352">
-        <v>-0.3448162932823767</v>
+        <v>-0.3448162932823545</v>
       </c>
     </row>
     <row r="353">
@@ -24370,10 +24370,10 @@
         <v>22.5997561136882</v>
       </c>
       <c r="N353">
-        <v>23.77362779864106</v>
+        <v>23.77362779864108</v>
       </c>
       <c r="O353">
-        <v>23.77362873790585</v>
+        <v>23.77362873790611</v>
       </c>
       <c r="P353">
         <v>55143</v>
@@ -24384,7 +24384,7 @@
         </is>
       </c>
       <c r="S353">
-        <v>-0.3448153540175858</v>
+        <v>-0.3448153540173249</v>
       </c>
     </row>
     <row r="354">
@@ -24438,10 +24438,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N354">
-        <v>86.61759427225226</v>
+        <v>86.61759427225223</v>
       </c>
       <c r="O354">
-        <v>90.83563195911086</v>
+        <v>90.83563195911087</v>
       </c>
       <c r="P354">
         <v>57277</v>
@@ -24506,10 +24506,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N355">
-        <v>86.61759427225226</v>
+        <v>86.61759427225223</v>
       </c>
       <c r="O355">
-        <v>90.83563195911086</v>
+        <v>90.83563195911087</v>
       </c>
       <c r="P355">
         <v>57277</v>
@@ -24574,10 +24574,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N356">
-        <v>86.61759427225226</v>
+        <v>86.61759427225223</v>
       </c>
       <c r="O356">
-        <v>90.83563195911086</v>
+        <v>90.83563195911087</v>
       </c>
       <c r="P356">
         <v>57277</v>
@@ -24588,7 +24588,7 @@
         </is>
       </c>
       <c r="S356">
-        <v>-2.943012765955721</v>
+        <v>-2.943012765955744</v>
       </c>
     </row>
     <row r="357">
@@ -24642,10 +24642,10 @@
         <v>91.09254484367177</v>
       </c>
       <c r="N357">
-        <v>86.61759427225226</v>
+        <v>86.61759427225223</v>
       </c>
       <c r="O357">
-        <v>90.83563195911086</v>
+        <v>90.83563195911087</v>
       </c>
       <c r="P357">
         <v>57277</v>
@@ -24656,7 +24656,7 @@
         </is>
       </c>
       <c r="S357">
-        <v>1.275024920902879</v>
+        <v>1.27502492090289</v>
       </c>
     </row>
     <row r="358">
@@ -24710,10 +24710,10 @@
         <v>60.99375995409059</v>
       </c>
       <c r="N358">
-        <v>61.01690685229691</v>
+        <v>61.01690685229683</v>
       </c>
       <c r="O358">
-        <v>60.71393243350624</v>
+        <v>60.71393243350647</v>
       </c>
       <c r="P358">
         <v>59908</v>
@@ -24778,10 +24778,10 @@
         <v>60.99375995409059</v>
       </c>
       <c r="N359">
-        <v>61.01690685229691</v>
+        <v>61.01690685229683</v>
       </c>
       <c r="O359">
-        <v>60.71393243350624</v>
+        <v>60.71393243350647</v>
       </c>
       <c r="P359">
         <v>59908</v>
@@ -24846,10 +24846,10 @@
         <v>60.99375995409059</v>
       </c>
       <c r="N360">
-        <v>61.01690685229691</v>
+        <v>61.01690685229683</v>
       </c>
       <c r="O360">
-        <v>60.71393243350624</v>
+        <v>60.71393243350647</v>
       </c>
       <c r="P360">
         <v>59908</v>
@@ -24860,7 +24860,7 @@
         </is>
       </c>
       <c r="S360">
-        <v>-1.764850130809625</v>
+        <v>-1.764850130809714</v>
       </c>
     </row>
     <row r="361">
@@ -24914,10 +24914,10 @@
         <v>60.99375995409059</v>
       </c>
       <c r="N361">
-        <v>61.01690685229691</v>
+        <v>61.01690685229683</v>
       </c>
       <c r="O361">
-        <v>60.71393243350624</v>
+        <v>60.71393243350647</v>
       </c>
       <c r="P361">
         <v>59908</v>
@@ -24928,7 +24928,7 @@
         </is>
       </c>
       <c r="S361">
-        <v>-2.067824549600306</v>
+        <v>-2.067824549600072</v>
       </c>
     </row>
     <row r="362">
@@ -24982,10 +24982,10 @@
         <v>52.20547113980047</v>
       </c>
       <c r="N362">
-        <v>51.58328699371179</v>
+        <v>51.58328699371187</v>
       </c>
       <c r="O362">
-        <v>51.69280674241715</v>
+        <v>51.69280674241718</v>
       </c>
       <c r="P362">
         <v>59563</v>
@@ -25050,10 +25050,10 @@
         <v>52.20547113980047</v>
       </c>
       <c r="N363">
-        <v>51.58328699371179</v>
+        <v>51.58328699371187</v>
       </c>
       <c r="O363">
-        <v>51.69280674241715</v>
+        <v>51.69280674241718</v>
       </c>
       <c r="P363">
         <v>59563</v>
@@ -25118,10 +25118,10 @@
         <v>52.20547113980047</v>
       </c>
       <c r="N364">
-        <v>51.58328699371179</v>
+        <v>51.58328699371187</v>
       </c>
       <c r="O364">
-        <v>51.69280674241715</v>
+        <v>51.69280674241718</v>
       </c>
       <c r="P364">
         <v>59563</v>
@@ -25132,7 +25132,7 @@
         </is>
       </c>
       <c r="S364">
-        <v>-0.504880833975152</v>
+        <v>-0.5048808339750743</v>
       </c>
     </row>
     <row r="365">
@@ -25186,10 +25186,10 @@
         <v>52.20547113980047</v>
       </c>
       <c r="N365">
-        <v>51.58328699371179</v>
+        <v>51.58328699371187</v>
       </c>
       <c r="O365">
-        <v>51.69280674241715</v>
+        <v>51.69280674241718</v>
       </c>
       <c r="P365">
         <v>59563</v>
@@ -25200,7 +25200,7 @@
         </is>
       </c>
       <c r="S365">
-        <v>-0.3953610852697853</v>
+        <v>-0.395361085269752</v>
       </c>
     </row>
     <row r="366">
@@ -25254,10 +25254,10 @@
         <v>94.03545595788032</v>
       </c>
       <c r="N366">
-        <v>89.30448482920688</v>
+        <v>89.30448482920681</v>
       </c>
       <c r="O366">
-        <v>92.04660792596596</v>
+        <v>92.04660792596593</v>
       </c>
       <c r="P366">
         <v>59952</v>
@@ -25322,10 +25322,10 @@
         <v>94.03545595788032</v>
       </c>
       <c r="N367">
-        <v>89.30448482920688</v>
+        <v>89.30448482920681</v>
       </c>
       <c r="O367">
-        <v>92.04660792596596</v>
+        <v>92.04660792596593</v>
       </c>
       <c r="P367">
         <v>59952</v>
@@ -25390,10 +25390,10 @@
         <v>94.03545595788032</v>
       </c>
       <c r="N368">
-        <v>89.30448482920688</v>
+        <v>89.30448482920681</v>
       </c>
       <c r="O368">
-        <v>92.04660792596596</v>
+        <v>92.04660792596593</v>
       </c>
       <c r="P368">
         <v>59952</v>
@@ -25404,7 +25404,7 @@
         </is>
       </c>
       <c r="S368">
-        <v>-0.4456318395810288</v>
+        <v>-0.4456318395810954</v>
       </c>
     </row>
     <row r="369">
@@ -25458,10 +25458,10 @@
         <v>94.03545595788032</v>
       </c>
       <c r="N369">
-        <v>89.30448482920688</v>
+        <v>89.30448482920681</v>
       </c>
       <c r="O369">
-        <v>92.04660792596596</v>
+        <v>92.04660792596593</v>
       </c>
       <c r="P369">
         <v>59952</v>
@@ -25472,7 +25472,7 @@
         </is>
       </c>
       <c r="S369">
-        <v>2.296491257178046</v>
+        <v>2.296491257178013</v>
       </c>
     </row>
     <row r="370">
@@ -25526,10 +25526,10 @@
         <v>90.81416282496983</v>
       </c>
       <c r="N370">
-        <v>92.88968438627364</v>
+        <v>92.88968438627357</v>
       </c>
       <c r="O370">
-        <v>89.6150820305524</v>
+        <v>89.61508203055229</v>
       </c>
       <c r="P370">
         <v>60000</v>
@@ -25594,10 +25594,10 @@
         <v>90.81416282496983</v>
       </c>
       <c r="N371">
-        <v>92.88968438627364</v>
+        <v>92.88968438627357</v>
       </c>
       <c r="O371">
-        <v>89.6150820305524</v>
+        <v>89.61508203055229</v>
       </c>
       <c r="P371">
         <v>60000</v>
@@ -25662,10 +25662,10 @@
         <v>90.81416282496983</v>
       </c>
       <c r="N372">
-        <v>92.88968438627364</v>
+        <v>92.88968438627357</v>
       </c>
       <c r="O372">
-        <v>89.6150820305524</v>
+        <v>89.61508203055229</v>
       </c>
       <c r="P372">
         <v>60000</v>
@@ -25676,7 +25676,7 @@
         </is>
       </c>
       <c r="S372">
-        <v>0.8780904036132187</v>
+        <v>0.878090403613152</v>
       </c>
     </row>
     <row r="373">
@@ -25730,10 +25730,10 @@
         <v>90.81416282496983</v>
       </c>
       <c r="N373">
-        <v>92.88968438627364</v>
+        <v>92.88968438627357</v>
       </c>
       <c r="O373">
-        <v>89.6150820305524</v>
+        <v>89.61508203055229</v>
       </c>
       <c r="P373">
         <v>60000</v>
@@ -25744,7 +25744,7 @@
         </is>
       </c>
       <c r="S373">
-        <v>-2.396511952108016</v>
+        <v>-2.396511952108138</v>
       </c>
     </row>
     <row r="374">
@@ -25798,10 +25798,10 @@
         <v>66.36932631856995</v>
       </c>
       <c r="N374">
-        <v>68.0847098326675</v>
+        <v>68.08470983266751</v>
       </c>
       <c r="O374">
-        <v>65.01271796233409</v>
+        <v>65.01271796233431</v>
       </c>
       <c r="P374">
         <v>40876</v>
@@ -25866,10 +25866,10 @@
         <v>66.36932631856995</v>
       </c>
       <c r="N375">
-        <v>68.0847098326675</v>
+        <v>68.08470983266751</v>
       </c>
       <c r="O375">
-        <v>65.01271796233409</v>
+        <v>65.01271796233431</v>
       </c>
       <c r="P375">
         <v>40876</v>
@@ -25934,10 +25934,10 @@
         <v>66.36932631856995</v>
       </c>
       <c r="N376">
-        <v>68.0847098326675</v>
+        <v>68.08470983266751</v>
       </c>
       <c r="O376">
-        <v>65.01271796233409</v>
+        <v>65.01271796233431</v>
       </c>
       <c r="P376">
         <v>40876</v>
@@ -25948,7 +25948,7 @@
         </is>
       </c>
       <c r="S376">
-        <v>0.6967417540916898</v>
+        <v>0.6967417540917009</v>
       </c>
     </row>
     <row r="377">
@@ -26002,10 +26002,10 @@
         <v>66.36932631856995</v>
       </c>
       <c r="N377">
-        <v>68.0847098326675</v>
+        <v>68.08470983266751</v>
       </c>
       <c r="O377">
-        <v>65.01271796233409</v>
+        <v>65.01271796233431</v>
       </c>
       <c r="P377">
         <v>40876</v>
@@ -26016,7 +26016,7 @@
         </is>
       </c>
       <c r="S377">
-        <v>-2.375250116241723</v>
+        <v>-2.375250116241501</v>
       </c>
     </row>
     <row r="378">
@@ -26070,10 +26070,10 @@
         <v>7.294531710394677</v>
       </c>
       <c r="N378">
-        <v>57.18663105574592</v>
+        <v>57.18663105574594</v>
       </c>
       <c r="O378">
-        <v>14.73483535187088</v>
+        <v>14.7348353518708</v>
       </c>
       <c r="P378">
         <v>47791</v>
@@ -26138,10 +26138,10 @@
         <v>7.294531710394677</v>
       </c>
       <c r="N379">
-        <v>57.18663105574592</v>
+        <v>57.18663105574594</v>
       </c>
       <c r="O379">
-        <v>14.73483535187088</v>
+        <v>14.7348353518708</v>
       </c>
       <c r="P379">
         <v>47791</v>
@@ -26206,10 +26206,10 @@
         <v>7.294531710394677</v>
       </c>
       <c r="N380">
-        <v>57.18663105574592</v>
+        <v>57.18663105574594</v>
       </c>
       <c r="O380">
-        <v>14.73483535187088</v>
+        <v>14.7348353518708</v>
       </c>
       <c r="P380">
         <v>47791</v>
@@ -26220,7 +26220,7 @@
         </is>
       </c>
       <c r="S380">
-        <v>-9.099751258068167E-05</v>
+        <v>-9.099751255847721E-05</v>
       </c>
     </row>
     <row r="381">
@@ -26274,10 +26274,10 @@
         <v>7.294531710394677</v>
       </c>
       <c r="N381">
-        <v>57.18663105574592</v>
+        <v>57.18663105574594</v>
       </c>
       <c r="O381">
-        <v>14.73483535187088</v>
+        <v>14.7348353518708</v>
       </c>
       <c r="P381">
         <v>47791</v>
@@ -26288,7 +26288,7 @@
         </is>
       </c>
       <c r="S381">
-        <v>-42.45188670138761</v>
+        <v>-42.4518867013877</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update benchmark inputs and analysis outputs
</commit_message>
<xml_diff>
--- a/tables_and_figures/input_tables/national_errors.xlsx
+++ b/tables_and_figures/input_tables/national_errors.xlsx
@@ -18701,7 +18701,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G270" t="b">
@@ -18714,7 +18714,7 @@
         <v>0</v>
       </c>
       <c r="J270" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K270">
         <v>87.37047875398824</v>
@@ -18769,7 +18769,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G271" t="b">
@@ -18782,7 +18782,7 @@
         <v>0</v>
       </c>
       <c r="J271" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K271">
         <v>87.37047875398824</v>
@@ -18837,7 +18837,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G272" t="b">
@@ -18850,7 +18850,7 @@
         <v>0</v>
       </c>
       <c r="J272" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K272">
         <v>87.37047875398824</v>
@@ -18905,7 +18905,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G273" t="b">
@@ -18918,7 +18918,7 @@
         <v>0</v>
       </c>
       <c r="J273" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K273">
         <v>87.37047875398824</v>
@@ -21421,7 +21421,7 @@
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G310" t="b">
@@ -21434,7 +21434,7 @@
         <v>0</v>
       </c>
       <c r="J310" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K310">
         <v>86.62346554656978</v>
@@ -21489,7 +21489,7 @@
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G311" t="b">
@@ -21502,7 +21502,7 @@
         <v>0</v>
       </c>
       <c r="J311" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K311">
         <v>86.62346554656978</v>
@@ -21557,7 +21557,7 @@
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G312" t="b">
@@ -21570,7 +21570,7 @@
         <v>0</v>
       </c>
       <c r="J312" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K312">
         <v>86.62346554656978</v>
@@ -21625,7 +21625,7 @@
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G313" t="b">
@@ -21638,7 +21638,7 @@
         <v>0</v>
       </c>
       <c r="J313" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K313">
         <v>86.62346554656978</v>
@@ -24413,7 +24413,7 @@
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G354" t="b">
@@ -24426,7 +24426,7 @@
         <v>0</v>
       </c>
       <c r="J354" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K354">
         <v>86.61759112435755</v>
@@ -24481,7 +24481,7 @@
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G355" t="b">
@@ -24494,7 +24494,7 @@
         <v>0</v>
       </c>
       <c r="J355" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K355">
         <v>86.61759112435755</v>
@@ -24549,7 +24549,7 @@
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G356" t="b">
@@ -24562,7 +24562,7 @@
         <v>0</v>
       </c>
       <c r="J356" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K356">
         <v>86.61759112435755</v>
@@ -24617,7 +24617,7 @@
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="G357" t="b">
@@ -24630,7 +24630,7 @@
         <v>0</v>
       </c>
       <c r="J357" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K357">
         <v>86.61759112435755</v>

</xml_diff>